<commit_message>
Auto commit - 09021722
</commit_message>
<xml_diff>
--- a/IM/202609_HL_Maintain_Report.xlsx
+++ b/IM/202609_HL_Maintain_Report.xlsx
@@ -11,14 +11,14 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Report'!$1:$2</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Report'!$A$1:$AK$12</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Report'!$A$1:$AK$17</definedName>
   </definedNames>
   <calcPr calcId="999999" calcMode="auto" calcCompleted="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="129">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="166">
   <si>
     <t>萊爾富 工作統計表  篩選月份：202609   (  製表日期:2026-09-02  )</t>
   </si>
@@ -401,6 +401,56 @@
     <t>2026-09-01 16:25:00</t>
   </si>
   <si>
+    <t>E5075115090201</t>
+  </si>
+  <si>
+    <t>龜山復興店</t>
+  </si>
+  <si>
+    <t>2026-09-02 07:05:49</t>
+  </si>
+  <si>
+    <t>星期三</t>
+  </si>
+  <si>
+    <t>凌晨</t>
+  </si>
+  <si>
+    <t>HLD3</t>
+  </si>
+  <si>
+    <t>HL-熱感發票機</t>
+  </si>
+  <si>
+    <t>D301</t>
+  </si>
+  <si>
+    <t>發票切刀卡紙，切紙不正常</t>
+  </si>
+  <si>
+    <t>門市反應TM2發票機(BSC10)無法正常裁切紙張會切不斷，門市已有重裝紙捲重開機仍異常....須請台芝到店協助(發票列印完無法裁切,或裁切一半,做動不正常)</t>
+  </si>
+  <si>
+    <t>THILF05075</t>
+  </si>
+  <si>
+    <t>2026-09-02 09:06:41</t>
+  </si>
+  <si>
+    <t>2026-09-02 13:30:00</t>
+  </si>
+  <si>
+    <t>2026-09-02 14:00:00</t>
+  </si>
+  <si>
+    <t>2026-09-03 13:06:00</t>
+  </si>
+  <si>
+    <t>更換發票機
+換下8155003142
+換上8155005808</t>
+  </si>
+  <si>
     <t>中和自治店</t>
   </si>
   <si>
@@ -417,6 +467,69 @@
   </si>
   <si>
     <t>2026-09-02 10:52:00</t>
+  </si>
+  <si>
+    <t>三重溪美店</t>
+  </si>
+  <si>
+    <t>THILF04191</t>
+  </si>
+  <si>
+    <t>2026-09-02 13:55:15</t>
+  </si>
+  <si>
+    <t>2026-09-02 13:20:00</t>
+  </si>
+  <si>
+    <t>2026-09-02 13:42:00</t>
+  </si>
+  <si>
+    <t>D620</t>
+  </si>
+  <si>
+    <t>三重福隆店</t>
+  </si>
+  <si>
+    <t>THILF0D620</t>
+  </si>
+  <si>
+    <t>2026-09-02 14:43:57</t>
+  </si>
+  <si>
+    <t>2026-09-02 14:05:00</t>
+  </si>
+  <si>
+    <t>2026-09-02 14:27:00</t>
+  </si>
+  <si>
+    <t>三重公園店</t>
+  </si>
+  <si>
+    <t>THILF04352</t>
+  </si>
+  <si>
+    <t>2026-09-02 15:04:59</t>
+  </si>
+  <si>
+    <t>2026-09-02 14:40:00</t>
+  </si>
+  <si>
+    <t>2026-09-02 15:00:00</t>
+  </si>
+  <si>
+    <t>北縣天龍店</t>
+  </si>
+  <si>
+    <t>THILF03840</t>
+  </si>
+  <si>
+    <t>2026-09-02 15:39:35</t>
+  </si>
+  <si>
+    <t>2026-09-02 15:10:00</t>
+  </si>
+  <si>
+    <t>2026-09-02 15:32:00</t>
   </si>
 </sst>
 </file>
@@ -830,7 +943,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AK12"/>
+  <dimension ref="A1:AK17"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="true" style="0"/>
@@ -1792,38 +1905,58 @@
         <v>10</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>61</v>
+        <v>38</v>
       </c>
       <c r="C12" s="3">
-        <v>2026090431</v>
-      </c>
-      <c r="D12" s="3"/>
-      <c r="E12" s="3"/>
+        <v>2026090392</v>
+      </c>
+      <c r="D12" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="E12" s="3" t="s">
+        <v>40</v>
+      </c>
       <c r="F12" s="3">
-        <v>3318</v>
+        <v>5075</v>
       </c>
       <c r="G12" s="3" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="H12" s="3" t="s">
-        <v>124</v>
-      </c>
-      <c r="I12" s="3"/>
-      <c r="J12" s="3"/>
-      <c r="K12" s="3"/>
-      <c r="L12" s="3"/>
-      <c r="M12" s="4"/>
-      <c r="N12" s="3"/>
-      <c r="O12" s="4"/>
-      <c r="P12" s="4"/>
+        <v>90</v>
+      </c>
+      <c r="I12" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="J12" s="3" t="s">
+        <v>126</v>
+      </c>
+      <c r="K12" s="3" t="s">
+        <v>127</v>
+      </c>
+      <c r="L12" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="M12" s="4" t="s">
+        <v>129</v>
+      </c>
+      <c r="N12" s="3" t="s">
+        <v>130</v>
+      </c>
+      <c r="O12" s="4" t="s">
+        <v>131</v>
+      </c>
+      <c r="P12" s="10" t="s">
+        <v>132</v>
+      </c>
       <c r="Q12" s="3" t="s">
-        <v>125</v>
+        <v>133</v>
       </c>
       <c r="R12" s="3" t="s">
         <v>51</v>
       </c>
       <c r="S12" s="3" t="s">
-        <v>52</v>
+        <v>92</v>
       </c>
       <c r="T12" s="3">
         <v>1</v>
@@ -1832,37 +1965,430 @@
         <v>53</v>
       </c>
       <c r="V12" s="3" t="s">
-        <v>126</v>
+        <v>134</v>
       </c>
       <c r="W12" s="3" t="s">
-        <v>127</v>
+        <v>135</v>
       </c>
       <c r="X12" s="3" t="s">
-        <v>128</v>
-      </c>
-      <c r="Y12" s="3"/>
+        <v>136</v>
+      </c>
+      <c r="Y12" s="3" t="s">
+        <v>137</v>
+      </c>
       <c r="Z12" s="3">
-        <v>0.4</v>
+        <v>0.5</v>
       </c>
       <c r="AA12" s="3"/>
       <c r="AB12" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="AC12" s="4" t="s">
-        <v>67</v>
-      </c>
-      <c r="AD12" s="3" t="s">
-        <v>60</v>
-      </c>
+      <c r="AC12" s="10" t="s">
+        <v>138</v>
+      </c>
+      <c r="AD12" s="3"/>
       <c r="AE12" s="3"/>
       <c r="AF12" s="3"/>
       <c r="AG12" s="3"/>
       <c r="AH12" s="3"/>
       <c r="AI12" s="3"/>
-      <c r="AJ12" s="3" t="s">
-        <v>60</v>
-      </c>
+      <c r="AJ12" s="3"/>
       <c r="AK12" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="13" spans="1:37">
+      <c r="A13" s="7">
+        <v>11</v>
+      </c>
+      <c r="B13" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="C13" s="7">
+        <v>2026090431</v>
+      </c>
+      <c r="D13" s="7"/>
+      <c r="E13" s="7"/>
+      <c r="F13" s="7">
+        <v>3318</v>
+      </c>
+      <c r="G13" s="7" t="s">
+        <v>139</v>
+      </c>
+      <c r="H13" s="7" t="s">
+        <v>140</v>
+      </c>
+      <c r="I13" s="7"/>
+      <c r="J13" s="7"/>
+      <c r="K13" s="7"/>
+      <c r="L13" s="7"/>
+      <c r="M13" s="8"/>
+      <c r="N13" s="7"/>
+      <c r="O13" s="8"/>
+      <c r="P13" s="9"/>
+      <c r="Q13" s="7" t="s">
+        <v>141</v>
+      </c>
+      <c r="R13" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S13" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="T13" s="7">
+        <v>1</v>
+      </c>
+      <c r="U13" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V13" s="7" t="s">
+        <v>142</v>
+      </c>
+      <c r="W13" s="7" t="s">
+        <v>143</v>
+      </c>
+      <c r="X13" s="7" t="s">
+        <v>144</v>
+      </c>
+      <c r="Y13" s="7"/>
+      <c r="Z13" s="7">
+        <v>0.4</v>
+      </c>
+      <c r="AA13" s="7"/>
+      <c r="AB13" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC13" s="9" t="s">
+        <v>67</v>
+      </c>
+      <c r="AD13" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE13" s="7"/>
+      <c r="AF13" s="7"/>
+      <c r="AG13" s="7"/>
+      <c r="AH13" s="7"/>
+      <c r="AI13" s="7"/>
+      <c r="AJ13" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AK13" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="14" spans="1:37">
+      <c r="A14" s="3">
+        <v>12</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="C14" s="3">
+        <v>2026090468</v>
+      </c>
+      <c r="D14" s="3"/>
+      <c r="E14" s="3"/>
+      <c r="F14" s="3">
+        <v>4191</v>
+      </c>
+      <c r="G14" s="3" t="s">
+        <v>145</v>
+      </c>
+      <c r="H14" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="I14" s="3"/>
+      <c r="J14" s="3"/>
+      <c r="K14" s="3"/>
+      <c r="L14" s="3"/>
+      <c r="M14" s="4"/>
+      <c r="N14" s="3"/>
+      <c r="O14" s="4"/>
+      <c r="P14" s="10"/>
+      <c r="Q14" s="3" t="s">
+        <v>146</v>
+      </c>
+      <c r="R14" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S14" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="T14" s="3">
+        <v>1</v>
+      </c>
+      <c r="U14" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V14" s="3" t="s">
+        <v>147</v>
+      </c>
+      <c r="W14" s="3" t="s">
+        <v>148</v>
+      </c>
+      <c r="X14" s="3" t="s">
+        <v>149</v>
+      </c>
+      <c r="Y14" s="3"/>
+      <c r="Z14" s="3">
+        <v>0.4</v>
+      </c>
+      <c r="AA14" s="3"/>
+      <c r="AB14" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC14" s="10" t="s">
+        <v>67</v>
+      </c>
+      <c r="AD14" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE14" s="3"/>
+      <c r="AF14" s="3"/>
+      <c r="AG14" s="3"/>
+      <c r="AH14" s="3"/>
+      <c r="AI14" s="3"/>
+      <c r="AJ14" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AK14" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="15" spans="1:37">
+      <c r="A15" s="7">
+        <v>13</v>
+      </c>
+      <c r="B15" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="C15" s="7">
+        <v>2026090475</v>
+      </c>
+      <c r="D15" s="7"/>
+      <c r="E15" s="7"/>
+      <c r="F15" s="7" t="s">
+        <v>150</v>
+      </c>
+      <c r="G15" s="7" t="s">
+        <v>151</v>
+      </c>
+      <c r="H15" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="I15" s="7"/>
+      <c r="J15" s="7"/>
+      <c r="K15" s="7"/>
+      <c r="L15" s="7"/>
+      <c r="M15" s="8"/>
+      <c r="N15" s="7"/>
+      <c r="O15" s="8"/>
+      <c r="P15" s="9"/>
+      <c r="Q15" s="7" t="s">
+        <v>152</v>
+      </c>
+      <c r="R15" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S15" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="T15" s="7">
+        <v>1</v>
+      </c>
+      <c r="U15" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V15" s="7" t="s">
+        <v>153</v>
+      </c>
+      <c r="W15" s="7" t="s">
+        <v>154</v>
+      </c>
+      <c r="X15" s="7" t="s">
+        <v>155</v>
+      </c>
+      <c r="Y15" s="7"/>
+      <c r="Z15" s="7">
+        <v>0.4</v>
+      </c>
+      <c r="AA15" s="7"/>
+      <c r="AB15" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC15" s="9" t="s">
+        <v>67</v>
+      </c>
+      <c r="AD15" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE15" s="7"/>
+      <c r="AF15" s="7"/>
+      <c r="AG15" s="7"/>
+      <c r="AH15" s="7"/>
+      <c r="AI15" s="7"/>
+      <c r="AJ15" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AK15" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="16" spans="1:37">
+      <c r="A16" s="3">
+        <v>14</v>
+      </c>
+      <c r="B16" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="C16" s="3">
+        <v>2026090482</v>
+      </c>
+      <c r="D16" s="3"/>
+      <c r="E16" s="3"/>
+      <c r="F16" s="3">
+        <v>4352</v>
+      </c>
+      <c r="G16" s="3" t="s">
+        <v>156</v>
+      </c>
+      <c r="H16" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="I16" s="3"/>
+      <c r="J16" s="3"/>
+      <c r="K16" s="3"/>
+      <c r="L16" s="3"/>
+      <c r="M16" s="4"/>
+      <c r="N16" s="3"/>
+      <c r="O16" s="4"/>
+      <c r="P16" s="10"/>
+      <c r="Q16" s="3" t="s">
+        <v>157</v>
+      </c>
+      <c r="R16" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S16" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="T16" s="3">
+        <v>1</v>
+      </c>
+      <c r="U16" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V16" s="3" t="s">
+        <v>158</v>
+      </c>
+      <c r="W16" s="3" t="s">
+        <v>159</v>
+      </c>
+      <c r="X16" s="3" t="s">
+        <v>160</v>
+      </c>
+      <c r="Y16" s="3"/>
+      <c r="Z16" s="3">
+        <v>0.3</v>
+      </c>
+      <c r="AA16" s="3"/>
+      <c r="AB16" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC16" s="10" t="s">
+        <v>67</v>
+      </c>
+      <c r="AD16" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE16" s="3"/>
+      <c r="AF16" s="3"/>
+      <c r="AG16" s="3"/>
+      <c r="AH16" s="3"/>
+      <c r="AI16" s="3"/>
+      <c r="AJ16" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AK16" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="17" spans="1:37">
+      <c r="A17" s="7">
+        <v>15</v>
+      </c>
+      <c r="B17" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="C17" s="7">
+        <v>2026090493</v>
+      </c>
+      <c r="D17" s="7"/>
+      <c r="E17" s="7"/>
+      <c r="F17" s="7">
+        <v>3840</v>
+      </c>
+      <c r="G17" s="7" t="s">
+        <v>161</v>
+      </c>
+      <c r="H17" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="I17" s="7"/>
+      <c r="J17" s="7"/>
+      <c r="K17" s="7"/>
+      <c r="L17" s="7"/>
+      <c r="M17" s="8"/>
+      <c r="N17" s="7"/>
+      <c r="O17" s="8"/>
+      <c r="P17" s="8"/>
+      <c r="Q17" s="7" t="s">
+        <v>162</v>
+      </c>
+      <c r="R17" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S17" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="T17" s="7">
+        <v>1</v>
+      </c>
+      <c r="U17" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V17" s="7" t="s">
+        <v>163</v>
+      </c>
+      <c r="W17" s="7" t="s">
+        <v>164</v>
+      </c>
+      <c r="X17" s="7" t="s">
+        <v>165</v>
+      </c>
+      <c r="Y17" s="7"/>
+      <c r="Z17" s="7">
+        <v>0.4</v>
+      </c>
+      <c r="AA17" s="7"/>
+      <c r="AB17" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC17" s="8" t="s">
+        <v>67</v>
+      </c>
+      <c r="AD17" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE17" s="7"/>
+      <c r="AF17" s="7"/>
+      <c r="AG17" s="7"/>
+      <c r="AH17" s="7"/>
+      <c r="AI17" s="7"/>
+      <c r="AJ17" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AK17" s="7" t="s">
         <v>60</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto commit - 09031504
</commit_message>
<xml_diff>
--- a/IM/202609_HL_Maintain_Report.xlsx
+++ b/IM/202609_HL_Maintain_Report.xlsx
@@ -11,16 +11,16 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Report'!$1:$2</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Report'!$A$1:$AK$17</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Report'!$A$1:$AK$24</definedName>
   </definedNames>
   <calcPr calcId="999999" calcMode="auto" calcCompleted="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="166">
-  <si>
-    <t>萊爾富 工作統計表  篩選月份：202609   (  製表日期:2026-09-02  )</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="215">
+  <si>
+    <t>萊爾富 工作統計表  篩選月份：202609   (  製表日期:2026-09-03  )</t>
   </si>
   <si>
     <t>項次</t>
@@ -484,6 +484,54 @@
     <t>2026-09-02 13:42:00</t>
   </si>
   <si>
+    <t>1D111115090202</t>
+  </si>
+  <si>
+    <t>D111</t>
+  </si>
+  <si>
+    <t>板橋府中店</t>
+  </si>
+  <si>
+    <t>新北市板橋區</t>
+  </si>
+  <si>
+    <t>2026-09-02 14:00:27</t>
+  </si>
+  <si>
+    <t>HL23</t>
+  </si>
+  <si>
+    <t>HL-TM主機</t>
+  </si>
+  <si>
+    <t>觸控不良(游標偏移)</t>
+  </si>
+  <si>
+    <t>門市反應TM1(TCX800)觸控亂跳，未點選螢幕但會一直發出點選螢幕的逼逼聲，與門市確認螢幕未貼保護貼、文宣，已有協助門市執行觸控校正仍異常....請台芝到店協助</t>
+  </si>
+  <si>
+    <t>THILF0D111</t>
+  </si>
+  <si>
+    <t>狄澤洋</t>
+  </si>
+  <si>
+    <t>2026-09-02 14:02:29</t>
+  </si>
+  <si>
+    <t>2026-09-03 12:35:00</t>
+  </si>
+  <si>
+    <t>2026-09-03 13:00:00</t>
+  </si>
+  <si>
+    <t>2026-09-03 18:02:00</t>
+  </si>
+  <si>
+    <t>螢幕清潔線路重新插拔，觀察一段時間測試正常</t>
+  </si>
+  <si>
     <t>D620</t>
   </si>
   <si>
@@ -530,6 +578,105 @@
   </si>
   <si>
     <t>2026-09-02 15:32:00</t>
+  </si>
+  <si>
+    <t>EC660115090201</t>
+  </si>
+  <si>
+    <t>C660</t>
+  </si>
+  <si>
+    <t>中和永安市場</t>
+  </si>
+  <si>
+    <t>2026-09-02 22:51:26</t>
+  </si>
+  <si>
+    <t>夜間</t>
+  </si>
+  <si>
+    <t>門市反應TM1(TCX800)觸控不良卡頓很難按都要多點幾次，已協助操作觸控校正重啟仍異常，確認無張貼文宣貼紙，....須請台芝到店協助	(機一觸控不好按.按都要深按.還會有所延遲.麻煩查修.謝謝)09/03  09:03  TM1協助觸控校正，09:30 再去電確認...廖</t>
+  </si>
+  <si>
+    <t>THILF0C660</t>
+  </si>
+  <si>
+    <t>2026-09-03 09:39:41</t>
+  </si>
+  <si>
+    <t>2026-09-03 14:00:00</t>
+  </si>
+  <si>
+    <t>2026-09-04 13:39:00</t>
+  </si>
+  <si>
+    <t>換上8185002267。 換下8185000572</t>
+  </si>
+  <si>
+    <t>蘆竹蘆興店</t>
+  </si>
+  <si>
+    <t>桃園市蘆竹區</t>
+  </si>
+  <si>
+    <t>THILF02988</t>
+  </si>
+  <si>
+    <t>2026-09-03 12:20:37</t>
+  </si>
+  <si>
+    <t>2026-09-03 11:50:00</t>
+  </si>
+  <si>
+    <t>2026-09-03 12:10:00</t>
+  </si>
+  <si>
+    <t>L501</t>
+  </si>
+  <si>
+    <t>車麗屋板橋店</t>
+  </si>
+  <si>
+    <t>THILF0L501</t>
+  </si>
+  <si>
+    <t>2026-09-03 12:30:22</t>
+  </si>
+  <si>
+    <t>2026-09-03 12:15:00</t>
+  </si>
+  <si>
+    <t>2026-09-03 12:29:00</t>
+  </si>
+  <si>
+    <t>2026-09-03 13:01:53</t>
+  </si>
+  <si>
+    <t>蘆竹領航星</t>
+  </si>
+  <si>
+    <t>THILF04601</t>
+  </si>
+  <si>
+    <t>2026-09-03 13:54:48</t>
+  </si>
+  <si>
+    <t>2026-09-03 13:10:00</t>
+  </si>
+  <si>
+    <t>2026-09-03 13:30:00</t>
+  </si>
+  <si>
+    <t>桃縣桃科店</t>
+  </si>
+  <si>
+    <t>THILF02620</t>
+  </si>
+  <si>
+    <t>2026-09-03 14:13:18</t>
+  </si>
+  <si>
+    <t>2026-09-03 13:40:00</t>
   </si>
 </sst>
 </file>
@@ -943,7 +1090,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AK17"/>
+  <dimension ref="A1:AK24"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="true" style="0"/>
@@ -2160,38 +2307,58 @@
         <v>13</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>61</v>
+        <v>38</v>
       </c>
       <c r="C15" s="7">
-        <v>2026090475</v>
-      </c>
-      <c r="D15" s="7"/>
-      <c r="E15" s="7"/>
+        <v>2026090469</v>
+      </c>
+      <c r="D15" s="7" t="s">
+        <v>150</v>
+      </c>
+      <c r="E15" s="7" t="s">
+        <v>40</v>
+      </c>
       <c r="F15" s="7" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="G15" s="7" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="H15" s="7" t="s">
-        <v>42</v>
-      </c>
-      <c r="I15" s="7"/>
-      <c r="J15" s="7"/>
-      <c r="K15" s="7"/>
-      <c r="L15" s="7"/>
-      <c r="M15" s="8"/>
-      <c r="N15" s="7"/>
-      <c r="O15" s="8"/>
-      <c r="P15" s="9"/>
+        <v>153</v>
+      </c>
+      <c r="I15" s="7" t="s">
+        <v>154</v>
+      </c>
+      <c r="J15" s="7" t="s">
+        <v>126</v>
+      </c>
+      <c r="K15" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="L15" s="7" t="s">
+        <v>155</v>
+      </c>
+      <c r="M15" s="8" t="s">
+        <v>156</v>
+      </c>
+      <c r="N15" s="7">
+        <v>2307</v>
+      </c>
+      <c r="O15" s="8" t="s">
+        <v>157</v>
+      </c>
+      <c r="P15" s="9" t="s">
+        <v>158</v>
+      </c>
       <c r="Q15" s="7" t="s">
-        <v>152</v>
+        <v>159</v>
       </c>
       <c r="R15" s="7" t="s">
         <v>51</v>
       </c>
       <c r="S15" s="7" t="s">
-        <v>52</v>
+        <v>160</v>
       </c>
       <c r="T15" s="7">
         <v>1</v>
@@ -2200,15 +2367,17 @@
         <v>53</v>
       </c>
       <c r="V15" s="7" t="s">
-        <v>153</v>
+        <v>161</v>
       </c>
       <c r="W15" s="7" t="s">
-        <v>154</v>
+        <v>162</v>
       </c>
       <c r="X15" s="7" t="s">
-        <v>155</v>
-      </c>
-      <c r="Y15" s="7"/>
+        <v>163</v>
+      </c>
+      <c r="Y15" s="7" t="s">
+        <v>164</v>
+      </c>
       <c r="Z15" s="7">
         <v>0.4</v>
       </c>
@@ -2217,19 +2386,15 @@
         <v>58</v>
       </c>
       <c r="AC15" s="9" t="s">
-        <v>67</v>
-      </c>
-      <c r="AD15" s="7" t="s">
-        <v>60</v>
-      </c>
+        <v>165</v>
+      </c>
+      <c r="AD15" s="7"/>
       <c r="AE15" s="7"/>
       <c r="AF15" s="7"/>
       <c r="AG15" s="7"/>
       <c r="AH15" s="7"/>
       <c r="AI15" s="7"/>
-      <c r="AJ15" s="7" t="s">
-        <v>60</v>
-      </c>
+      <c r="AJ15" s="7"/>
       <c r="AK15" s="7" t="s">
         <v>60</v>
       </c>
@@ -2242,15 +2407,15 @@
         <v>61</v>
       </c>
       <c r="C16" s="3">
-        <v>2026090482</v>
+        <v>2026090475</v>
       </c>
       <c r="D16" s="3"/>
       <c r="E16" s="3"/>
-      <c r="F16" s="3">
-        <v>4352</v>
+      <c r="F16" s="3" t="s">
+        <v>166</v>
       </c>
       <c r="G16" s="3" t="s">
-        <v>156</v>
+        <v>167</v>
       </c>
       <c r="H16" s="3" t="s">
         <v>42</v>
@@ -2264,7 +2429,7 @@
       <c r="O16" s="4"/>
       <c r="P16" s="10"/>
       <c r="Q16" s="3" t="s">
-        <v>157</v>
+        <v>168</v>
       </c>
       <c r="R16" s="3" t="s">
         <v>51</v>
@@ -2279,17 +2444,17 @@
         <v>53</v>
       </c>
       <c r="V16" s="3" t="s">
-        <v>158</v>
+        <v>169</v>
       </c>
       <c r="W16" s="3" t="s">
-        <v>159</v>
+        <v>170</v>
       </c>
       <c r="X16" s="3" t="s">
-        <v>160</v>
+        <v>171</v>
       </c>
       <c r="Y16" s="3"/>
       <c r="Z16" s="3">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="AA16" s="3"/>
       <c r="AB16" s="3" t="s">
@@ -2321,15 +2486,15 @@
         <v>61</v>
       </c>
       <c r="C17" s="7">
-        <v>2026090493</v>
+        <v>2026090482</v>
       </c>
       <c r="D17" s="7"/>
       <c r="E17" s="7"/>
       <c r="F17" s="7">
-        <v>3840</v>
+        <v>4352</v>
       </c>
       <c r="G17" s="7" t="s">
-        <v>161</v>
+        <v>172</v>
       </c>
       <c r="H17" s="7" t="s">
         <v>42</v>
@@ -2341,9 +2506,9 @@
       <c r="M17" s="8"/>
       <c r="N17" s="7"/>
       <c r="O17" s="8"/>
-      <c r="P17" s="8"/>
+      <c r="P17" s="9"/>
       <c r="Q17" s="7" t="s">
-        <v>162</v>
+        <v>173</v>
       </c>
       <c r="R17" s="7" t="s">
         <v>51</v>
@@ -2358,23 +2523,23 @@
         <v>53</v>
       </c>
       <c r="V17" s="7" t="s">
-        <v>163</v>
+        <v>174</v>
       </c>
       <c r="W17" s="7" t="s">
-        <v>164</v>
+        <v>175</v>
       </c>
       <c r="X17" s="7" t="s">
-        <v>165</v>
+        <v>176</v>
       </c>
       <c r="Y17" s="7"/>
       <c r="Z17" s="7">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="AA17" s="7"/>
       <c r="AB17" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="AC17" s="8" t="s">
+      <c r="AC17" s="9" t="s">
         <v>67</v>
       </c>
       <c r="AD17" s="7" t="s">
@@ -2389,6 +2554,567 @@
         <v>60</v>
       </c>
       <c r="AK17" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="18" spans="1:37">
+      <c r="A18" s="3">
+        <v>16</v>
+      </c>
+      <c r="B18" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="C18" s="3">
+        <v>2026090493</v>
+      </c>
+      <c r="D18" s="3"/>
+      <c r="E18" s="3"/>
+      <c r="F18" s="3">
+        <v>3840</v>
+      </c>
+      <c r="G18" s="3" t="s">
+        <v>177</v>
+      </c>
+      <c r="H18" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="I18" s="3"/>
+      <c r="J18" s="3"/>
+      <c r="K18" s="3"/>
+      <c r="L18" s="3"/>
+      <c r="M18" s="4"/>
+      <c r="N18" s="3"/>
+      <c r="O18" s="4"/>
+      <c r="P18" s="10"/>
+      <c r="Q18" s="3" t="s">
+        <v>178</v>
+      </c>
+      <c r="R18" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S18" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="T18" s="3">
+        <v>1</v>
+      </c>
+      <c r="U18" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V18" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="W18" s="3" t="s">
+        <v>180</v>
+      </c>
+      <c r="X18" s="3" t="s">
+        <v>181</v>
+      </c>
+      <c r="Y18" s="3"/>
+      <c r="Z18" s="3">
+        <v>0.4</v>
+      </c>
+      <c r="AA18" s="3"/>
+      <c r="AB18" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC18" s="10" t="s">
+        <v>67</v>
+      </c>
+      <c r="AD18" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE18" s="3"/>
+      <c r="AF18" s="3"/>
+      <c r="AG18" s="3"/>
+      <c r="AH18" s="3"/>
+      <c r="AI18" s="3"/>
+      <c r="AJ18" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AK18" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="19" spans="1:37">
+      <c r="A19" s="7">
+        <v>17</v>
+      </c>
+      <c r="B19" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="C19" s="7">
+        <v>2026090584</v>
+      </c>
+      <c r="D19" s="7" t="s">
+        <v>182</v>
+      </c>
+      <c r="E19" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="F19" s="7" t="s">
+        <v>183</v>
+      </c>
+      <c r="G19" s="7" t="s">
+        <v>184</v>
+      </c>
+      <c r="H19" s="7" t="s">
+        <v>140</v>
+      </c>
+      <c r="I19" s="7" t="s">
+        <v>185</v>
+      </c>
+      <c r="J19" s="7" t="s">
+        <v>126</v>
+      </c>
+      <c r="K19" s="7" t="s">
+        <v>186</v>
+      </c>
+      <c r="L19" s="7" t="s">
+        <v>155</v>
+      </c>
+      <c r="M19" s="8" t="s">
+        <v>156</v>
+      </c>
+      <c r="N19" s="7">
+        <v>2307</v>
+      </c>
+      <c r="O19" s="8" t="s">
+        <v>157</v>
+      </c>
+      <c r="P19" s="9" t="s">
+        <v>187</v>
+      </c>
+      <c r="Q19" s="7" t="s">
+        <v>188</v>
+      </c>
+      <c r="R19" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S19" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="T19" s="7">
+        <v>1</v>
+      </c>
+      <c r="U19" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V19" s="7" t="s">
+        <v>189</v>
+      </c>
+      <c r="W19" s="7" t="s">
+        <v>163</v>
+      </c>
+      <c r="X19" s="7" t="s">
+        <v>190</v>
+      </c>
+      <c r="Y19" s="7" t="s">
+        <v>191</v>
+      </c>
+      <c r="Z19" s="7">
+        <v>1</v>
+      </c>
+      <c r="AA19" s="7"/>
+      <c r="AB19" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC19" s="9" t="s">
+        <v>192</v>
+      </c>
+      <c r="AD19" s="7"/>
+      <c r="AE19" s="7"/>
+      <c r="AF19" s="7"/>
+      <c r="AG19" s="7"/>
+      <c r="AH19" s="7"/>
+      <c r="AI19" s="7"/>
+      <c r="AJ19" s="7"/>
+      <c r="AK19" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="20" spans="1:37">
+      <c r="A20" s="3">
+        <v>18</v>
+      </c>
+      <c r="B20" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="C20" s="3">
+        <v>2026090632</v>
+      </c>
+      <c r="D20" s="3"/>
+      <c r="E20" s="3"/>
+      <c r="F20" s="3">
+        <v>2988</v>
+      </c>
+      <c r="G20" s="3" t="s">
+        <v>193</v>
+      </c>
+      <c r="H20" s="3" t="s">
+        <v>194</v>
+      </c>
+      <c r="I20" s="3"/>
+      <c r="J20" s="3"/>
+      <c r="K20" s="3"/>
+      <c r="L20" s="3"/>
+      <c r="M20" s="4"/>
+      <c r="N20" s="3"/>
+      <c r="O20" s="4"/>
+      <c r="P20" s="10"/>
+      <c r="Q20" s="3" t="s">
+        <v>195</v>
+      </c>
+      <c r="R20" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S20" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="T20" s="3">
+        <v>1</v>
+      </c>
+      <c r="U20" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V20" s="3" t="s">
+        <v>196</v>
+      </c>
+      <c r="W20" s="3" t="s">
+        <v>197</v>
+      </c>
+      <c r="X20" s="3" t="s">
+        <v>198</v>
+      </c>
+      <c r="Y20" s="3"/>
+      <c r="Z20" s="3">
+        <v>0.3</v>
+      </c>
+      <c r="AA20" s="3"/>
+      <c r="AB20" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC20" s="10" t="s">
+        <v>67</v>
+      </c>
+      <c r="AD20" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE20" s="3"/>
+      <c r="AF20" s="3"/>
+      <c r="AG20" s="3"/>
+      <c r="AH20" s="3"/>
+      <c r="AI20" s="3"/>
+      <c r="AJ20" s="3"/>
+      <c r="AK20" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="21" spans="1:37">
+      <c r="A21" s="7">
+        <v>19</v>
+      </c>
+      <c r="B21" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="C21" s="7">
+        <v>2026090634</v>
+      </c>
+      <c r="D21" s="7"/>
+      <c r="E21" s="7"/>
+      <c r="F21" s="7" t="s">
+        <v>199</v>
+      </c>
+      <c r="G21" s="7" t="s">
+        <v>200</v>
+      </c>
+      <c r="H21" s="7" t="s">
+        <v>153</v>
+      </c>
+      <c r="I21" s="7"/>
+      <c r="J21" s="7"/>
+      <c r="K21" s="7"/>
+      <c r="L21" s="7"/>
+      <c r="M21" s="8"/>
+      <c r="N21" s="7"/>
+      <c r="O21" s="8"/>
+      <c r="P21" s="9"/>
+      <c r="Q21" s="7" t="s">
+        <v>201</v>
+      </c>
+      <c r="R21" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S21" s="7" t="s">
+        <v>160</v>
+      </c>
+      <c r="T21" s="7">
+        <v>1</v>
+      </c>
+      <c r="U21" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V21" s="7" t="s">
+        <v>202</v>
+      </c>
+      <c r="W21" s="7" t="s">
+        <v>203</v>
+      </c>
+      <c r="X21" s="7" t="s">
+        <v>204</v>
+      </c>
+      <c r="Y21" s="7"/>
+      <c r="Z21" s="7">
+        <v>0.2</v>
+      </c>
+      <c r="AA21" s="7"/>
+      <c r="AB21" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC21" s="9" t="s">
+        <v>67</v>
+      </c>
+      <c r="AD21" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE21" s="7"/>
+      <c r="AF21" s="7"/>
+      <c r="AG21" s="7"/>
+      <c r="AH21" s="7"/>
+      <c r="AI21" s="7"/>
+      <c r="AJ21" s="7"/>
+      <c r="AK21" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="22" spans="1:37">
+      <c r="A22" s="3">
+        <v>20</v>
+      </c>
+      <c r="B22" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="C22" s="3">
+        <v>2026090635</v>
+      </c>
+      <c r="D22" s="3"/>
+      <c r="E22" s="3"/>
+      <c r="F22" s="3" t="s">
+        <v>151</v>
+      </c>
+      <c r="G22" s="3" t="s">
+        <v>152</v>
+      </c>
+      <c r="H22" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="I22" s="3"/>
+      <c r="J22" s="3"/>
+      <c r="K22" s="3"/>
+      <c r="L22" s="3"/>
+      <c r="M22" s="4"/>
+      <c r="N22" s="3"/>
+      <c r="O22" s="4"/>
+      <c r="P22" s="10"/>
+      <c r="Q22" s="3" t="s">
+        <v>159</v>
+      </c>
+      <c r="R22" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S22" s="3" t="s">
+        <v>160</v>
+      </c>
+      <c r="T22" s="3">
+        <v>1</v>
+      </c>
+      <c r="U22" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V22" s="3" t="s">
+        <v>205</v>
+      </c>
+      <c r="W22" s="3" t="s">
+        <v>162</v>
+      </c>
+      <c r="X22" s="3" t="s">
+        <v>163</v>
+      </c>
+      <c r="Y22" s="3"/>
+      <c r="Z22" s="3">
+        <v>0.4</v>
+      </c>
+      <c r="AA22" s="3"/>
+      <c r="AB22" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC22" s="10" t="s">
+        <v>67</v>
+      </c>
+      <c r="AD22" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE22" s="3"/>
+      <c r="AF22" s="3"/>
+      <c r="AG22" s="3"/>
+      <c r="AH22" s="3"/>
+      <c r="AI22" s="3"/>
+      <c r="AJ22" s="3"/>
+      <c r="AK22" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="23" spans="1:37">
+      <c r="A23" s="7">
+        <v>21</v>
+      </c>
+      <c r="B23" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="C23" s="7">
+        <v>2026090652</v>
+      </c>
+      <c r="D23" s="7"/>
+      <c r="E23" s="7"/>
+      <c r="F23" s="7">
+        <v>4601</v>
+      </c>
+      <c r="G23" s="7" t="s">
+        <v>206</v>
+      </c>
+      <c r="H23" s="7" t="s">
+        <v>194</v>
+      </c>
+      <c r="I23" s="7"/>
+      <c r="J23" s="7"/>
+      <c r="K23" s="7"/>
+      <c r="L23" s="7"/>
+      <c r="M23" s="8"/>
+      <c r="N23" s="7"/>
+      <c r="O23" s="8"/>
+      <c r="P23" s="9"/>
+      <c r="Q23" s="7" t="s">
+        <v>207</v>
+      </c>
+      <c r="R23" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S23" s="7" t="s">
+        <v>92</v>
+      </c>
+      <c r="T23" s="7">
+        <v>1</v>
+      </c>
+      <c r="U23" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V23" s="7" t="s">
+        <v>208</v>
+      </c>
+      <c r="W23" s="7" t="s">
+        <v>209</v>
+      </c>
+      <c r="X23" s="7" t="s">
+        <v>210</v>
+      </c>
+      <c r="Y23" s="7"/>
+      <c r="Z23" s="7">
+        <v>0.3</v>
+      </c>
+      <c r="AA23" s="7"/>
+      <c r="AB23" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC23" s="9" t="s">
+        <v>67</v>
+      </c>
+      <c r="AD23" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE23" s="7"/>
+      <c r="AF23" s="7"/>
+      <c r="AG23" s="7"/>
+      <c r="AH23" s="7"/>
+      <c r="AI23" s="7"/>
+      <c r="AJ23" s="7"/>
+      <c r="AK23" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="24" spans="1:37">
+      <c r="A24" s="3">
+        <v>22</v>
+      </c>
+      <c r="B24" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="C24" s="3">
+        <v>2026090656</v>
+      </c>
+      <c r="D24" s="3"/>
+      <c r="E24" s="3"/>
+      <c r="F24" s="3">
+        <v>2620</v>
+      </c>
+      <c r="G24" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="H24" s="3" t="s">
+        <v>194</v>
+      </c>
+      <c r="I24" s="3"/>
+      <c r="J24" s="3"/>
+      <c r="K24" s="3"/>
+      <c r="L24" s="3"/>
+      <c r="M24" s="4"/>
+      <c r="N24" s="3"/>
+      <c r="O24" s="4"/>
+      <c r="P24" s="4"/>
+      <c r="Q24" s="3" t="s">
+        <v>212</v>
+      </c>
+      <c r="R24" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S24" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="T24" s="3">
+        <v>1</v>
+      </c>
+      <c r="U24" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V24" s="3" t="s">
+        <v>213</v>
+      </c>
+      <c r="W24" s="3" t="s">
+        <v>214</v>
+      </c>
+      <c r="X24" s="3" t="s">
+        <v>190</v>
+      </c>
+      <c r="Y24" s="3"/>
+      <c r="Z24" s="3">
+        <v>0.3</v>
+      </c>
+      <c r="AA24" s="3"/>
+      <c r="AB24" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC24" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="AD24" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE24" s="3"/>
+      <c r="AF24" s="3"/>
+      <c r="AG24" s="3"/>
+      <c r="AH24" s="3"/>
+      <c r="AI24" s="3"/>
+      <c r="AJ24" s="3"/>
+      <c r="AK24" s="3" t="s">
         <v>60</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto commit - 09041823
</commit_message>
<xml_diff>
--- a/IM/202609_HL_Maintain_Report.xlsx
+++ b/IM/202609_HL_Maintain_Report.xlsx
@@ -11,16 +11,16 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Report'!$1:$2</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Report'!$A$1:$AK$24</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Report'!$A$1:$AK$32</definedName>
   </definedNames>
   <calcPr calcId="999999" calcMode="auto" calcCompleted="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="215">
-  <si>
-    <t>萊爾富 工作統計表  篩選月份：202609   (  製表日期:2026-09-03  )</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="285">
+  <si>
+    <t>萊爾富 工作統計表  篩選月份：202609   (  製表日期:2026-09-04  )</t>
   </si>
   <si>
     <t>項次</t>
@@ -613,6 +613,39 @@
     <t>換上8185002267。 換下8185000572</t>
   </si>
   <si>
+    <t>E4101115090201</t>
+  </si>
+  <si>
+    <t>三重溪華店</t>
+  </si>
+  <si>
+    <t>2026-09-02 22:53:41</t>
+  </si>
+  <si>
+    <t>D303</t>
+  </si>
+  <si>
+    <t>門市反應TM1(BSC-10)時常設備亮紅燈無法列印，關機紙捲重裝會正常，但仍頻繁發生...請台芝到店協助(會突然停,不能列卬,燈會一直閃)09/03 09:05 職員告知不清楚，需待10:00店長來後再去電確認...欣</t>
+  </si>
+  <si>
+    <t>THILF04101</t>
+  </si>
+  <si>
+    <t>2026-09-03 10:01:20</t>
+  </si>
+  <si>
+    <t>2026-09-04 10:35:00</t>
+  </si>
+  <si>
+    <t>2026-09-04 10:57:00</t>
+  </si>
+  <si>
+    <t>2026-09-04 14:01:00</t>
+  </si>
+  <si>
+    <t>換下8155003807。換上8155004451</t>
+  </si>
+  <si>
     <t>蘆竹蘆興店</t>
   </si>
   <si>
@@ -677,6 +710,184 @@
   </si>
   <si>
     <t>2026-09-03 13:40:00</t>
+  </si>
+  <si>
+    <t>F777</t>
+  </si>
+  <si>
+    <t>蘆竹南華店</t>
+  </si>
+  <si>
+    <t>THILF0F777</t>
+  </si>
+  <si>
+    <t>2026-09-03 15:44:55</t>
+  </si>
+  <si>
+    <t>2026-09-03 15:10:00</t>
+  </si>
+  <si>
+    <t>2026-09-03 15:30:00</t>
+  </si>
+  <si>
+    <t>1C052115090301</t>
+  </si>
+  <si>
+    <t>C052</t>
+  </si>
+  <si>
+    <t>中和連城店</t>
+  </si>
+  <si>
+    <t>2026-09-03 15:49:20</t>
+  </si>
+  <si>
+    <t>星期四</t>
+  </si>
+  <si>
+    <t>HL27</t>
+  </si>
+  <si>
+    <t>HL-雷射印表機</t>
+  </si>
+  <si>
+    <t>多張吃紙、卡紙</t>
+  </si>
+  <si>
+    <t>門市反應SC雷射印表機(M6600NW)無法傳真，更換設備前都還可以傳真，已有重新拔插線路、確認後方線路都有插好仍無法傳真....請台芝到店協助※案1C052115081901，台芝08/20到店更換印表機</t>
+  </si>
+  <si>
+    <t>THILF0C052</t>
+  </si>
+  <si>
+    <t>2026-09-03 15:51:55</t>
+  </si>
+  <si>
+    <t>2026-09-03 18:36:00</t>
+  </si>
+  <si>
+    <t>2026-09-03 18:56:00</t>
+  </si>
+  <si>
+    <t>2026-09-04 19:51:00</t>
+  </si>
+  <si>
+    <t>影印機傳真電話線插電話無任何反應。已請店家改報修中華電信。</t>
+  </si>
+  <si>
+    <t>E3623115090401</t>
+  </si>
+  <si>
+    <t>三重自強店</t>
+  </si>
+  <si>
+    <t>2026-09-04 08:50:56</t>
+  </si>
+  <si>
+    <t>星期五</t>
+  </si>
+  <si>
+    <t>當機或無畫面</t>
+  </si>
+  <si>
+    <t>門市反應MMK目前畫面為廣告畫面，門市告知正常廣告畫面點選一下後會進入首頁，但點選都無反應...請台芝到店協助(螢幕無反應)</t>
+  </si>
+  <si>
+    <t>THILF03623</t>
+  </si>
+  <si>
+    <t>2026-09-04 09:23:55</t>
+  </si>
+  <si>
+    <t>2026-09-04 11:40:00</t>
+  </si>
+  <si>
+    <t>2026-09-04 12:02:00</t>
+  </si>
+  <si>
+    <t>2026-09-07 13:23:00</t>
+  </si>
+  <si>
+    <t>螢幕排線重新插拔。可正常點擊。</t>
+  </si>
+  <si>
+    <t>2026-09-04 11:40:17</t>
+  </si>
+  <si>
+    <t>2026-09-04 11:20:00</t>
+  </si>
+  <si>
+    <t>12543115090401</t>
+  </si>
+  <si>
+    <t>三重大仁店</t>
+  </si>
+  <si>
+    <t>2026-09-04 12:41:58</t>
+  </si>
+  <si>
+    <t>HL34</t>
+  </si>
+  <si>
+    <t>HL-HUB</t>
+  </si>
+  <si>
+    <t>HUB週期維護</t>
+  </si>
+  <si>
+    <t>2026年07月份 HUB週期維護:1PORT插在2PORT</t>
+  </si>
+  <si>
+    <t>THILF02543</t>
+  </si>
+  <si>
+    <t>2026-09-04 12:43:16</t>
+  </si>
+  <si>
+    <t>2026-09-04 12:50:00</t>
+  </si>
+  <si>
+    <t>2026-09-04 13:06:00</t>
+  </si>
+  <si>
+    <t>2026-09-07 16:43:00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2PORT改插回1PORT+Hub
+</t>
+  </si>
+  <si>
+    <t>C192</t>
+  </si>
+  <si>
+    <t>中和福美店</t>
+  </si>
+  <si>
+    <t>THILF0C192</t>
+  </si>
+  <si>
+    <t>2026-09-04 15:36:55</t>
+  </si>
+  <si>
+    <t>2026-09-04 15:00:00</t>
+  </si>
+  <si>
+    <t>2026-09-04 15:36:00</t>
+  </si>
+  <si>
+    <t>裝潢撤機已完工</t>
+  </si>
+  <si>
+    <t>2026-09-04 15:39:05</t>
+  </si>
+  <si>
+    <t>2026-09-04 15:30:00</t>
+  </si>
+  <si>
+    <t>2026-09-04 15:35:00</t>
+  </si>
+  <si>
+    <t>改裝撤機</t>
   </si>
 </sst>
 </file>
@@ -1090,7 +1301,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AK24"/>
+  <dimension ref="A1:AK32"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="true" style="0"/>
@@ -2738,38 +2949,58 @@
         <v>18</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>61</v>
+        <v>38</v>
       </c>
       <c r="C20" s="3">
-        <v>2026090632</v>
-      </c>
-      <c r="D20" s="3"/>
-      <c r="E20" s="3"/>
+        <v>2026090592</v>
+      </c>
+      <c r="D20" s="3" t="s">
+        <v>193</v>
+      </c>
+      <c r="E20" s="3" t="s">
+        <v>40</v>
+      </c>
       <c r="F20" s="3">
-        <v>2988</v>
+        <v>4101</v>
       </c>
       <c r="G20" s="3" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="H20" s="3" t="s">
-        <v>194</v>
-      </c>
-      <c r="I20" s="3"/>
-      <c r="J20" s="3"/>
-      <c r="K20" s="3"/>
-      <c r="L20" s="3"/>
-      <c r="M20" s="4"/>
-      <c r="N20" s="3"/>
-      <c r="O20" s="4"/>
-      <c r="P20" s="10"/>
+        <v>42</v>
+      </c>
+      <c r="I20" s="3" t="s">
+        <v>195</v>
+      </c>
+      <c r="J20" s="3" t="s">
+        <v>126</v>
+      </c>
+      <c r="K20" s="3" t="s">
+        <v>186</v>
+      </c>
+      <c r="L20" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="M20" s="4" t="s">
+        <v>129</v>
+      </c>
+      <c r="N20" s="3" t="s">
+        <v>196</v>
+      </c>
+      <c r="O20" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="P20" s="10" t="s">
+        <v>197</v>
+      </c>
       <c r="Q20" s="3" t="s">
-        <v>195</v>
+        <v>198</v>
       </c>
       <c r="R20" s="3" t="s">
         <v>51</v>
       </c>
       <c r="S20" s="3" t="s">
-        <v>92</v>
+        <v>52</v>
       </c>
       <c r="T20" s="3">
         <v>1</v>
@@ -2778,28 +3009,28 @@
         <v>53</v>
       </c>
       <c r="V20" s="3" t="s">
-        <v>196</v>
+        <v>199</v>
       </c>
       <c r="W20" s="3" t="s">
-        <v>197</v>
+        <v>200</v>
       </c>
       <c r="X20" s="3" t="s">
-        <v>198</v>
-      </c>
-      <c r="Y20" s="3"/>
+        <v>201</v>
+      </c>
+      <c r="Y20" s="3" t="s">
+        <v>202</v>
+      </c>
       <c r="Z20" s="3">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="AA20" s="3"/>
       <c r="AB20" s="3" t="s">
         <v>58</v>
       </c>
       <c r="AC20" s="10" t="s">
-        <v>67</v>
-      </c>
-      <c r="AD20" s="3" t="s">
-        <v>60</v>
-      </c>
+        <v>203</v>
+      </c>
+      <c r="AD20" s="3"/>
       <c r="AE20" s="3"/>
       <c r="AF20" s="3"/>
       <c r="AG20" s="3"/>
@@ -2818,18 +3049,18 @@
         <v>61</v>
       </c>
       <c r="C21" s="7">
-        <v>2026090634</v>
+        <v>2026090632</v>
       </c>
       <c r="D21" s="7"/>
       <c r="E21" s="7"/>
-      <c r="F21" s="7" t="s">
-        <v>199</v>
+      <c r="F21" s="7">
+        <v>2988</v>
       </c>
       <c r="G21" s="7" t="s">
-        <v>200</v>
+        <v>204</v>
       </c>
       <c r="H21" s="7" t="s">
-        <v>153</v>
+        <v>205</v>
       </c>
       <c r="I21" s="7"/>
       <c r="J21" s="7"/>
@@ -2840,13 +3071,13 @@
       <c r="O21" s="8"/>
       <c r="P21" s="9"/>
       <c r="Q21" s="7" t="s">
-        <v>201</v>
+        <v>206</v>
       </c>
       <c r="R21" s="7" t="s">
         <v>51</v>
       </c>
       <c r="S21" s="7" t="s">
-        <v>160</v>
+        <v>92</v>
       </c>
       <c r="T21" s="7">
         <v>1</v>
@@ -2855,17 +3086,17 @@
         <v>53</v>
       </c>
       <c r="V21" s="7" t="s">
-        <v>202</v>
+        <v>207</v>
       </c>
       <c r="W21" s="7" t="s">
-        <v>203</v>
+        <v>208</v>
       </c>
       <c r="X21" s="7" t="s">
-        <v>204</v>
+        <v>209</v>
       </c>
       <c r="Y21" s="7"/>
       <c r="Z21" s="7">
-        <v>0.2</v>
+        <v>0.3</v>
       </c>
       <c r="AA21" s="7"/>
       <c r="AB21" s="7" t="s">
@@ -2895,15 +3126,15 @@
         <v>61</v>
       </c>
       <c r="C22" s="3">
-        <v>2026090635</v>
+        <v>2026090634</v>
       </c>
       <c r="D22" s="3"/>
       <c r="E22" s="3"/>
       <c r="F22" s="3" t="s">
-        <v>151</v>
+        <v>210</v>
       </c>
       <c r="G22" s="3" t="s">
-        <v>152</v>
+        <v>211</v>
       </c>
       <c r="H22" s="3" t="s">
         <v>153</v>
@@ -2917,7 +3148,7 @@
       <c r="O22" s="4"/>
       <c r="P22" s="10"/>
       <c r="Q22" s="3" t="s">
-        <v>159</v>
+        <v>212</v>
       </c>
       <c r="R22" s="3" t="s">
         <v>51</v>
@@ -2932,17 +3163,17 @@
         <v>53</v>
       </c>
       <c r="V22" s="3" t="s">
-        <v>205</v>
+        <v>213</v>
       </c>
       <c r="W22" s="3" t="s">
-        <v>162</v>
+        <v>214</v>
       </c>
       <c r="X22" s="3" t="s">
-        <v>163</v>
+        <v>215</v>
       </c>
       <c r="Y22" s="3"/>
       <c r="Z22" s="3">
-        <v>0.4</v>
+        <v>0.2</v>
       </c>
       <c r="AA22" s="3"/>
       <c r="AB22" s="3" t="s">
@@ -2972,18 +3203,18 @@
         <v>61</v>
       </c>
       <c r="C23" s="7">
-        <v>2026090652</v>
+        <v>2026090635</v>
       </c>
       <c r="D23" s="7"/>
       <c r="E23" s="7"/>
-      <c r="F23" s="7">
-        <v>4601</v>
+      <c r="F23" s="7" t="s">
+        <v>151</v>
       </c>
       <c r="G23" s="7" t="s">
-        <v>206</v>
+        <v>152</v>
       </c>
       <c r="H23" s="7" t="s">
-        <v>194</v>
+        <v>153</v>
       </c>
       <c r="I23" s="7"/>
       <c r="J23" s="7"/>
@@ -2994,13 +3225,13 @@
       <c r="O23" s="8"/>
       <c r="P23" s="9"/>
       <c r="Q23" s="7" t="s">
-        <v>207</v>
+        <v>159</v>
       </c>
       <c r="R23" s="7" t="s">
         <v>51</v>
       </c>
       <c r="S23" s="7" t="s">
-        <v>92</v>
+        <v>160</v>
       </c>
       <c r="T23" s="7">
         <v>1</v>
@@ -3009,17 +3240,17 @@
         <v>53</v>
       </c>
       <c r="V23" s="7" t="s">
-        <v>208</v>
+        <v>216</v>
       </c>
       <c r="W23" s="7" t="s">
-        <v>209</v>
+        <v>162</v>
       </c>
       <c r="X23" s="7" t="s">
-        <v>210</v>
+        <v>163</v>
       </c>
       <c r="Y23" s="7"/>
       <c r="Z23" s="7">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="AA23" s="7"/>
       <c r="AB23" s="7" t="s">
@@ -3049,18 +3280,18 @@
         <v>61</v>
       </c>
       <c r="C24" s="3">
-        <v>2026090656</v>
+        <v>2026090652</v>
       </c>
       <c r="D24" s="3"/>
       <c r="E24" s="3"/>
       <c r="F24" s="3">
-        <v>2620</v>
+        <v>4601</v>
       </c>
       <c r="G24" s="3" t="s">
-        <v>211</v>
+        <v>217</v>
       </c>
       <c r="H24" s="3" t="s">
-        <v>194</v>
+        <v>205</v>
       </c>
       <c r="I24" s="3"/>
       <c r="J24" s="3"/>
@@ -3069,9 +3300,9 @@
       <c r="M24" s="4"/>
       <c r="N24" s="3"/>
       <c r="O24" s="4"/>
-      <c r="P24" s="4"/>
+      <c r="P24" s="10"/>
       <c r="Q24" s="3" t="s">
-        <v>212</v>
+        <v>218</v>
       </c>
       <c r="R24" s="3" t="s">
         <v>51</v>
@@ -3086,13 +3317,13 @@
         <v>53</v>
       </c>
       <c r="V24" s="3" t="s">
-        <v>213</v>
+        <v>219</v>
       </c>
       <c r="W24" s="3" t="s">
-        <v>214</v>
+        <v>220</v>
       </c>
       <c r="X24" s="3" t="s">
-        <v>190</v>
+        <v>221</v>
       </c>
       <c r="Y24" s="3"/>
       <c r="Z24" s="3">
@@ -3102,7 +3333,7 @@
       <c r="AB24" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="AC24" s="4" t="s">
+      <c r="AC24" s="10" t="s">
         <v>67</v>
       </c>
       <c r="AD24" s="3" t="s">
@@ -3115,6 +3346,684 @@
       <c r="AI24" s="3"/>
       <c r="AJ24" s="3"/>
       <c r="AK24" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="25" spans="1:37">
+      <c r="A25" s="7">
+        <v>23</v>
+      </c>
+      <c r="B25" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="C25" s="7">
+        <v>2026090656</v>
+      </c>
+      <c r="D25" s="7"/>
+      <c r="E25" s="7"/>
+      <c r="F25" s="7">
+        <v>2620</v>
+      </c>
+      <c r="G25" s="7" t="s">
+        <v>222</v>
+      </c>
+      <c r="H25" s="7" t="s">
+        <v>205</v>
+      </c>
+      <c r="I25" s="7"/>
+      <c r="J25" s="7"/>
+      <c r="K25" s="7"/>
+      <c r="L25" s="7"/>
+      <c r="M25" s="8"/>
+      <c r="N25" s="7"/>
+      <c r="O25" s="8"/>
+      <c r="P25" s="9"/>
+      <c r="Q25" s="7" t="s">
+        <v>223</v>
+      </c>
+      <c r="R25" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S25" s="7" t="s">
+        <v>92</v>
+      </c>
+      <c r="T25" s="7">
+        <v>1</v>
+      </c>
+      <c r="U25" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V25" s="7" t="s">
+        <v>224</v>
+      </c>
+      <c r="W25" s="7" t="s">
+        <v>225</v>
+      </c>
+      <c r="X25" s="7" t="s">
+        <v>190</v>
+      </c>
+      <c r="Y25" s="7"/>
+      <c r="Z25" s="7">
+        <v>0.3</v>
+      </c>
+      <c r="AA25" s="7"/>
+      <c r="AB25" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC25" s="9" t="s">
+        <v>67</v>
+      </c>
+      <c r="AD25" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE25" s="7"/>
+      <c r="AF25" s="7"/>
+      <c r="AG25" s="7"/>
+      <c r="AH25" s="7"/>
+      <c r="AI25" s="7"/>
+      <c r="AJ25" s="7"/>
+      <c r="AK25" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="26" spans="1:37">
+      <c r="A26" s="3">
+        <v>24</v>
+      </c>
+      <c r="B26" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="C26" s="3">
+        <v>2026090708</v>
+      </c>
+      <c r="D26" s="3"/>
+      <c r="E26" s="3"/>
+      <c r="F26" s="3" t="s">
+        <v>226</v>
+      </c>
+      <c r="G26" s="3" t="s">
+        <v>227</v>
+      </c>
+      <c r="H26" s="3" t="s">
+        <v>205</v>
+      </c>
+      <c r="I26" s="3"/>
+      <c r="J26" s="3"/>
+      <c r="K26" s="3"/>
+      <c r="L26" s="3"/>
+      <c r="M26" s="4"/>
+      <c r="N26" s="3"/>
+      <c r="O26" s="4"/>
+      <c r="P26" s="10"/>
+      <c r="Q26" s="3" t="s">
+        <v>228</v>
+      </c>
+      <c r="R26" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S26" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="T26" s="3">
+        <v>1</v>
+      </c>
+      <c r="U26" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V26" s="3" t="s">
+        <v>229</v>
+      </c>
+      <c r="W26" s="3" t="s">
+        <v>230</v>
+      </c>
+      <c r="X26" s="3" t="s">
+        <v>231</v>
+      </c>
+      <c r="Y26" s="3"/>
+      <c r="Z26" s="3">
+        <v>0.3</v>
+      </c>
+      <c r="AA26" s="3"/>
+      <c r="AB26" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC26" s="10" t="s">
+        <v>67</v>
+      </c>
+      <c r="AD26" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE26" s="3"/>
+      <c r="AF26" s="3"/>
+      <c r="AG26" s="3"/>
+      <c r="AH26" s="3"/>
+      <c r="AI26" s="3"/>
+      <c r="AJ26" s="3"/>
+      <c r="AK26" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="27" spans="1:37">
+      <c r="A27" s="7">
+        <v>25</v>
+      </c>
+      <c r="B27" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="C27" s="7">
+        <v>2026090714</v>
+      </c>
+      <c r="D27" s="7" t="s">
+        <v>232</v>
+      </c>
+      <c r="E27" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="F27" s="7" t="s">
+        <v>233</v>
+      </c>
+      <c r="G27" s="7" t="s">
+        <v>234</v>
+      </c>
+      <c r="H27" s="7" t="s">
+        <v>140</v>
+      </c>
+      <c r="I27" s="7" t="s">
+        <v>235</v>
+      </c>
+      <c r="J27" s="7" t="s">
+        <v>236</v>
+      </c>
+      <c r="K27" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="L27" s="7" t="s">
+        <v>237</v>
+      </c>
+      <c r="M27" s="8" t="s">
+        <v>238</v>
+      </c>
+      <c r="N27" s="7">
+        <v>2701</v>
+      </c>
+      <c r="O27" s="8" t="s">
+        <v>239</v>
+      </c>
+      <c r="P27" s="9" t="s">
+        <v>240</v>
+      </c>
+      <c r="Q27" s="7" t="s">
+        <v>241</v>
+      </c>
+      <c r="R27" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S27" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="T27" s="7">
+        <v>1</v>
+      </c>
+      <c r="U27" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V27" s="7" t="s">
+        <v>242</v>
+      </c>
+      <c r="W27" s="7" t="s">
+        <v>243</v>
+      </c>
+      <c r="X27" s="7" t="s">
+        <v>244</v>
+      </c>
+      <c r="Y27" s="7" t="s">
+        <v>245</v>
+      </c>
+      <c r="Z27" s="7">
+        <v>0.3</v>
+      </c>
+      <c r="AA27" s="7"/>
+      <c r="AB27" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC27" s="9" t="s">
+        <v>246</v>
+      </c>
+      <c r="AD27" s="7"/>
+      <c r="AE27" s="7"/>
+      <c r="AF27" s="7"/>
+      <c r="AG27" s="7"/>
+      <c r="AH27" s="7"/>
+      <c r="AI27" s="7"/>
+      <c r="AJ27" s="7"/>
+      <c r="AK27" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="28" spans="1:37">
+      <c r="A28" s="3">
+        <v>26</v>
+      </c>
+      <c r="B28" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="C28" s="3">
+        <v>2026090851</v>
+      </c>
+      <c r="D28" s="3" t="s">
+        <v>247</v>
+      </c>
+      <c r="E28" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="F28" s="3">
+        <v>3623</v>
+      </c>
+      <c r="G28" s="3" t="s">
+        <v>248</v>
+      </c>
+      <c r="H28" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="I28" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="J28" s="3" t="s">
+        <v>250</v>
+      </c>
+      <c r="K28" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="L28" s="3" t="s">
+        <v>106</v>
+      </c>
+      <c r="M28" s="4" t="s">
+        <v>107</v>
+      </c>
+      <c r="N28" s="3">
+        <v>5801</v>
+      </c>
+      <c r="O28" s="4" t="s">
+        <v>251</v>
+      </c>
+      <c r="P28" s="10" t="s">
+        <v>252</v>
+      </c>
+      <c r="Q28" s="3" t="s">
+        <v>253</v>
+      </c>
+      <c r="R28" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S28" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="T28" s="3">
+        <v>1</v>
+      </c>
+      <c r="U28" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V28" s="3" t="s">
+        <v>254</v>
+      </c>
+      <c r="W28" s="3" t="s">
+        <v>255</v>
+      </c>
+      <c r="X28" s="3" t="s">
+        <v>256</v>
+      </c>
+      <c r="Y28" s="3" t="s">
+        <v>257</v>
+      </c>
+      <c r="Z28" s="3">
+        <v>0.4</v>
+      </c>
+      <c r="AA28" s="3"/>
+      <c r="AB28" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC28" s="10" t="s">
+        <v>258</v>
+      </c>
+      <c r="AD28" s="3"/>
+      <c r="AE28" s="3"/>
+      <c r="AF28" s="3"/>
+      <c r="AG28" s="3"/>
+      <c r="AH28" s="3"/>
+      <c r="AI28" s="3"/>
+      <c r="AJ28" s="3"/>
+      <c r="AK28" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="29" spans="1:37">
+      <c r="A29" s="7">
+        <v>27</v>
+      </c>
+      <c r="B29" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="C29" s="7">
+        <v>2026090882</v>
+      </c>
+      <c r="D29" s="7"/>
+      <c r="E29" s="7"/>
+      <c r="F29" s="7">
+        <v>4101</v>
+      </c>
+      <c r="G29" s="7" t="s">
+        <v>194</v>
+      </c>
+      <c r="H29" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="I29" s="7"/>
+      <c r="J29" s="7"/>
+      <c r="K29" s="7"/>
+      <c r="L29" s="7"/>
+      <c r="M29" s="8"/>
+      <c r="N29" s="7"/>
+      <c r="O29" s="8"/>
+      <c r="P29" s="9"/>
+      <c r="Q29" s="7" t="s">
+        <v>198</v>
+      </c>
+      <c r="R29" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S29" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="T29" s="7">
+        <v>1</v>
+      </c>
+      <c r="U29" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V29" s="7" t="s">
+        <v>259</v>
+      </c>
+      <c r="W29" s="7" t="s">
+        <v>201</v>
+      </c>
+      <c r="X29" s="7" t="s">
+        <v>260</v>
+      </c>
+      <c r="Y29" s="7"/>
+      <c r="Z29" s="7">
+        <v>0.4</v>
+      </c>
+      <c r="AA29" s="7"/>
+      <c r="AB29" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC29" s="9" t="s">
+        <v>67</v>
+      </c>
+      <c r="AD29" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE29" s="7"/>
+      <c r="AF29" s="7"/>
+      <c r="AG29" s="7"/>
+      <c r="AH29" s="7"/>
+      <c r="AI29" s="7"/>
+      <c r="AJ29" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AK29" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="30" spans="1:37">
+      <c r="A30" s="3">
+        <v>28</v>
+      </c>
+      <c r="B30" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="C30" s="3">
+        <v>2026090897</v>
+      </c>
+      <c r="D30" s="3" t="s">
+        <v>261</v>
+      </c>
+      <c r="E30" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="F30" s="3">
+        <v>2543</v>
+      </c>
+      <c r="G30" s="3" t="s">
+        <v>262</v>
+      </c>
+      <c r="H30" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="I30" s="3" t="s">
+        <v>263</v>
+      </c>
+      <c r="J30" s="3" t="s">
+        <v>250</v>
+      </c>
+      <c r="K30" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="L30" s="3" t="s">
+        <v>264</v>
+      </c>
+      <c r="M30" s="4" t="s">
+        <v>265</v>
+      </c>
+      <c r="N30" s="3">
+        <v>3404</v>
+      </c>
+      <c r="O30" s="4" t="s">
+        <v>266</v>
+      </c>
+      <c r="P30" s="10" t="s">
+        <v>267</v>
+      </c>
+      <c r="Q30" s="3" t="s">
+        <v>268</v>
+      </c>
+      <c r="R30" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S30" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="T30" s="3">
+        <v>1</v>
+      </c>
+      <c r="U30" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V30" s="3" t="s">
+        <v>269</v>
+      </c>
+      <c r="W30" s="3" t="s">
+        <v>270</v>
+      </c>
+      <c r="X30" s="3" t="s">
+        <v>271</v>
+      </c>
+      <c r="Y30" s="3" t="s">
+        <v>272</v>
+      </c>
+      <c r="Z30" s="3">
+        <v>0.3</v>
+      </c>
+      <c r="AA30" s="3"/>
+      <c r="AB30" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC30" s="10" t="s">
+        <v>273</v>
+      </c>
+      <c r="AD30" s="3"/>
+      <c r="AE30" s="3"/>
+      <c r="AF30" s="3"/>
+      <c r="AG30" s="3"/>
+      <c r="AH30" s="3"/>
+      <c r="AI30" s="3"/>
+      <c r="AJ30" s="3"/>
+      <c r="AK30" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="31" spans="1:37">
+      <c r="A31" s="7">
+        <v>29</v>
+      </c>
+      <c r="B31" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="C31" s="7">
+        <v>2026090919</v>
+      </c>
+      <c r="D31" s="7"/>
+      <c r="E31" s="7"/>
+      <c r="F31" s="7" t="s">
+        <v>274</v>
+      </c>
+      <c r="G31" s="7" t="s">
+        <v>275</v>
+      </c>
+      <c r="H31" s="7" t="s">
+        <v>140</v>
+      </c>
+      <c r="I31" s="7"/>
+      <c r="J31" s="7"/>
+      <c r="K31" s="7"/>
+      <c r="L31" s="7"/>
+      <c r="M31" s="8"/>
+      <c r="N31" s="7"/>
+      <c r="O31" s="8"/>
+      <c r="P31" s="9"/>
+      <c r="Q31" s="7" t="s">
+        <v>276</v>
+      </c>
+      <c r="R31" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S31" s="7" t="s">
+        <v>92</v>
+      </c>
+      <c r="T31" s="7">
+        <v>1</v>
+      </c>
+      <c r="U31" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V31" s="7" t="s">
+        <v>277</v>
+      </c>
+      <c r="W31" s="7" t="s">
+        <v>278</v>
+      </c>
+      <c r="X31" s="7" t="s">
+        <v>279</v>
+      </c>
+      <c r="Y31" s="7"/>
+      <c r="Z31" s="7">
+        <v>0.6</v>
+      </c>
+      <c r="AA31" s="7"/>
+      <c r="AB31" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC31" s="9" t="s">
+        <v>280</v>
+      </c>
+      <c r="AD31" s="7"/>
+      <c r="AE31" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AF31" s="7"/>
+      <c r="AG31" s="7"/>
+      <c r="AH31" s="7"/>
+      <c r="AI31" s="7"/>
+      <c r="AJ31" s="7"/>
+      <c r="AK31" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="32" spans="1:37">
+      <c r="A32" s="3">
+        <v>30</v>
+      </c>
+      <c r="B32" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="C32" s="3">
+        <v>2026090921</v>
+      </c>
+      <c r="D32" s="3"/>
+      <c r="E32" s="3"/>
+      <c r="F32" s="3" t="s">
+        <v>274</v>
+      </c>
+      <c r="G32" s="3" t="s">
+        <v>275</v>
+      </c>
+      <c r="H32" s="3" t="s">
+        <v>140</v>
+      </c>
+      <c r="I32" s="3"/>
+      <c r="J32" s="3"/>
+      <c r="K32" s="3"/>
+      <c r="L32" s="3"/>
+      <c r="M32" s="4"/>
+      <c r="N32" s="3"/>
+      <c r="O32" s="4"/>
+      <c r="P32" s="4"/>
+      <c r="Q32" s="3" t="s">
+        <v>276</v>
+      </c>
+      <c r="R32" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S32" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="T32" s="3">
+        <v>1</v>
+      </c>
+      <c r="U32" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V32" s="3" t="s">
+        <v>281</v>
+      </c>
+      <c r="W32" s="3" t="s">
+        <v>282</v>
+      </c>
+      <c r="X32" s="3" t="s">
+        <v>283</v>
+      </c>
+      <c r="Y32" s="3"/>
+      <c r="Z32" s="3">
+        <v>0.1</v>
+      </c>
+      <c r="AA32" s="3"/>
+      <c r="AB32" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC32" s="4" t="s">
+        <v>284</v>
+      </c>
+      <c r="AD32" s="3"/>
+      <c r="AE32" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AF32" s="3"/>
+      <c r="AG32" s="3"/>
+      <c r="AH32" s="3"/>
+      <c r="AI32" s="3"/>
+      <c r="AJ32" s="3"/>
+      <c r="AK32" s="3" t="s">
         <v>60</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto commit - 09081712
</commit_message>
<xml_diff>
--- a/IM/202609_HL_Maintain_Report.xlsx
+++ b/IM/202609_HL_Maintain_Report.xlsx
@@ -11,16 +11,16 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Report'!$1:$2</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Report'!$A$1:$AK$32</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Report'!$A$1:$AK$64</definedName>
   </definedNames>
   <calcPr calcId="999999" calcMode="auto" calcCompleted="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="285">
-  <si>
-    <t>萊爾富 工作統計表  篩選月份：202609   (  製表日期:2026-09-04  )</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="531">
+  <si>
+    <t>萊爾富 工作統計表  篩選月份：202609   (  製表日期:2026-09-08  )</t>
   </si>
   <si>
     <t>項次</t>
@@ -817,6 +817,48 @@
     <t>2026-09-04 11:20:00</t>
   </si>
   <si>
+    <t>E3941115090401</t>
+  </si>
+  <si>
+    <t>永和興工店</t>
+  </si>
+  <si>
+    <t>新北市永和區</t>
+  </si>
+  <si>
+    <t>2026-09-04 12:29:15</t>
+  </si>
+  <si>
+    <t>HL24</t>
+  </si>
+  <si>
+    <t>HL-SC主機</t>
+  </si>
+  <si>
+    <t>鍵盤按鍵不良或無反應</t>
+  </si>
+  <si>
+    <t>門市反應sc鍵盤數字8鍵按到都會一直連點，重新拔插線路仍異常...需請台芝到店協助(數字8會卡住一直888888888888888888888888888888888888)</t>
+  </si>
+  <si>
+    <t>THILF03941</t>
+  </si>
+  <si>
+    <t>2026-09-04 12:35:24</t>
+  </si>
+  <si>
+    <t>2026-09-07 08:35:00</t>
+  </si>
+  <si>
+    <t>2026-09-07 08:52:00</t>
+  </si>
+  <si>
+    <t>2026-09-07 16:35:00</t>
+  </si>
+  <si>
+    <t>更換鍵盤。</t>
+  </si>
+  <si>
     <t>12543115090401</t>
   </si>
   <si>
@@ -888,6 +930,714 @@
   </si>
   <si>
     <t>改裝撤機</t>
+  </si>
+  <si>
+    <t>E4098115090401</t>
+  </si>
+  <si>
+    <t>三重仁美店</t>
+  </si>
+  <si>
+    <t>2026-09-04 20:08:48</t>
+  </si>
+  <si>
+    <t>HLL7</t>
+  </si>
+  <si>
+    <t>HL-咖啡價目電子看板</t>
+  </si>
+  <si>
+    <t>L702</t>
+  </si>
+  <si>
+    <t>AOC無電源反應(黑屏無畫面)</t>
+  </si>
+  <si>
+    <t>門市反應咖啡價目電子看板黑屏無畫面、右下角燈號顯示綠燈，已有至後場重啟電源+數據機並休息20分鐘後再重啟仍黑畫面，確認遙控器有電，以搖控器開關畫面有閃一下、操作音量鍵畫面有出現音量大小標示但都沒有聲音...需請協助(電視黑頻，試過開關重開，還是黑頻。)21:38 門市表示已依序關閉電源、ADSL並休息20分鐘再開ADSL、電源後仍黑畫面，螢幕右下方確認顯示綠燈、操作遙控器音量鍵畫面有出現音量大小標20:43 門市表示找不到ADSL，已再次提醒門市電路編號為297Y271519，門市後續會再請店長協助..愷20:15 請門市依序先關閉店長桌前的看板電源再關ADSL電源休息20分鐘再開啟ADSL電源再開看板電源..愷</t>
+  </si>
+  <si>
+    <t>THILF04098</t>
+  </si>
+  <si>
+    <t>2026-09-04 21:48:16</t>
+  </si>
+  <si>
+    <t>2026-09-07 13:20:00</t>
+  </si>
+  <si>
+    <t>2026-09-07 14:05:00</t>
+  </si>
+  <si>
+    <t>2026-09-08 01:48:00</t>
+  </si>
+  <si>
+    <t>乙太網路失效</t>
+  </si>
+  <si>
+    <t>13227115090501</t>
+  </si>
+  <si>
+    <t>五股四維店</t>
+  </si>
+  <si>
+    <t>新北市五股區</t>
+  </si>
+  <si>
+    <t>2026-09-05 09:07:21</t>
+  </si>
+  <si>
+    <t>星期六</t>
+  </si>
+  <si>
+    <t>門市反應TM2 CCD掃描器(HC76TR)刷讀所有條碼都感應不良，已有進行條碼校正仍無法排除...還請台芝到店協助</t>
+  </si>
+  <si>
+    <t>THILF03227</t>
+  </si>
+  <si>
+    <t>湯家瑋</t>
+  </si>
+  <si>
+    <t>2026-09-05 09:09:03</t>
+  </si>
+  <si>
+    <t>2026-09-07 16:00:00</t>
+  </si>
+  <si>
+    <t>2026-09-07 16:30:00</t>
+  </si>
+  <si>
+    <t>2026-09-08 13:00:00</t>
+  </si>
+  <si>
+    <t>更換手持
+換下8119011530
+換上8119014011</t>
+  </si>
+  <si>
+    <t>E4856115090501</t>
+  </si>
+  <si>
+    <t>新莊小胖店</t>
+  </si>
+  <si>
+    <t>新北市新莊區</t>
+  </si>
+  <si>
+    <t>2026-09-05 03:12:56</t>
+  </si>
+  <si>
+    <t>門市反應TM2發票機(BSC10)無法正常裁切紙張會切不斷，門市已有重裝紙捲重開機仍異常....須請台芝到店協(發票機有時候無法切斷發票紙 沒印完整)09/05 09:00  門市再忙，請客服10分鐘再聯繫...廖</t>
+  </si>
+  <si>
+    <t>THILF04856</t>
+  </si>
+  <si>
+    <t>2026-09-05 09:23:05</t>
+  </si>
+  <si>
+    <t>2026-09-07 16:40:00</t>
+  </si>
+  <si>
+    <t>2026-09-07 17:10:00</t>
+  </si>
+  <si>
+    <t>更換發票機
+換上8155006477
+換下8155003028</t>
+  </si>
+  <si>
+    <t>13890115090501</t>
+  </si>
+  <si>
+    <t>三重美堤店</t>
+  </si>
+  <si>
+    <t>2026-09-05 12:59:44</t>
+  </si>
+  <si>
+    <t>HLF6</t>
+  </si>
+  <si>
+    <t>HL-多卡機QP3000E</t>
+  </si>
+  <si>
+    <t>F604</t>
+  </si>
+  <si>
+    <t>無電源反應</t>
+  </si>
+  <si>
+    <t>門市反映TM2多卡機QP3000E無電源反應，確認線路無脫落..請台芝到店協助</t>
+  </si>
+  <si>
+    <t>THILF03890</t>
+  </si>
+  <si>
+    <t>2026-09-05 13:07:07</t>
+  </si>
+  <si>
+    <t>2026-09-08 09:35:00</t>
+  </si>
+  <si>
+    <t>2026-09-08 09:55:00</t>
+  </si>
+  <si>
+    <t>換下8183001861。換上8183001631</t>
+  </si>
+  <si>
+    <t>1D111115090501</t>
+  </si>
+  <si>
+    <t>2026-09-05 13:05:17</t>
+  </si>
+  <si>
+    <t xml:space="preserve">門市反應TM1(TCX800)觸控亂跳，未點選螢幕但會一直發出點選螢幕的逼逼聲，與門市確認螢幕未貼保護貼、文宣，無法觸控校正重啟後仍異常..須請台芝到店協助  PS. 09/03台芝到店螢幕清潔線路重新插拔，觀察一段時間測試正常 </t>
+  </si>
+  <si>
+    <t>2026-09-05 13:10:28</t>
+  </si>
+  <si>
+    <t>2026-09-07 15:30:00</t>
+  </si>
+  <si>
+    <t>2026-09-07 17:52:00</t>
+  </si>
+  <si>
+    <t>更換UPOS
+換上：8185003918
+換下：8185002465</t>
+  </si>
+  <si>
+    <t>1L517115090501</t>
+  </si>
+  <si>
+    <t>急修件</t>
+  </si>
+  <si>
+    <t>L517</t>
+  </si>
+  <si>
+    <t>車麗屋蘆洲店</t>
+  </si>
+  <si>
+    <t>新北市蘆洲區</t>
+  </si>
+  <si>
+    <t>2026-09-05 14:31:11</t>
+  </si>
+  <si>
+    <t>當機/自動開關機</t>
+  </si>
+  <si>
+    <t>2026/09/05 14:38總公司宸宇確認啟動緊急叫修:門市WEBPOS(SHUTTLE6S)無法連線，PING80不通無法VNC，門市告知中華電信數據機測試正常，且有更換過網路線測試仍異常，已嘗試將SC關機重啟後仍異常...需請台芝到店協助 P.S.如後續處理有更換硬碟，請跟店長宣達：1.請門市先回報代收會計 2.請確認SC的代收資料是否正確 (須與代收單據逐一核對)與門市確認帳務做到9/3有列印報表並已繳回，門市營業時間為10:00~21:00</t>
+  </si>
+  <si>
+    <t>THILF0L517</t>
+  </si>
+  <si>
+    <t>2026-09-05 14:38:50</t>
+  </si>
+  <si>
+    <t>2026-09-05 16:00:00</t>
+  </si>
+  <si>
+    <t>2026-09-05 17:00:00</t>
+  </si>
+  <si>
+    <t>2026-09-06 07:38:00</t>
+  </si>
+  <si>
+    <t>現場插座電源異常，暫用延長線，回報0800測試正常</t>
+  </si>
+  <si>
+    <t>14397115090601</t>
+  </si>
+  <si>
+    <t>三重仁旺店</t>
+  </si>
+  <si>
+    <t>2026-09-06 14:01:50</t>
+  </si>
+  <si>
+    <t>印票機(L90)門市反應TM刷讀MMK列印單據提示印票機狀態異常，請門市檢查印票機只有亮一顆綠燈，門市已將印票機電源重開，紙捲重裝後再到MMK點選偵測印表機仍異常顯示...需請台芝到店協助</t>
+  </si>
+  <si>
+    <t>THILF04397</t>
+  </si>
+  <si>
+    <t>2026-09-06 14:05:34</t>
+  </si>
+  <si>
+    <t>2026-09-07 11:30:00</t>
+  </si>
+  <si>
+    <t>2026-09-07 11:50:00</t>
+  </si>
+  <si>
+    <t>90印票機用網路線點對點life et測試正常.  疑似6號網路線訊號異常導製連線異常。 建議更換</t>
+  </si>
+  <si>
+    <t>14260115090601</t>
+  </si>
+  <si>
+    <t>三重高中店</t>
+  </si>
+  <si>
+    <t>2026-09-06 15:52:02</t>
+  </si>
+  <si>
+    <t>客顯示器畫面不正常</t>
+  </si>
+  <si>
+    <t xml:space="preserve">門市反應TM1(TCX800)客顯畫面很暗幾乎快看不到，門市已有重啟客顯仍異常，VNC查看畫面正常....需請台芝到店協助	</t>
+  </si>
+  <si>
+    <t>THILF04260</t>
+  </si>
+  <si>
+    <t>2026-09-06 15:52:50</t>
+  </si>
+  <si>
+    <t>2026-09-07 09:55:00</t>
+  </si>
+  <si>
+    <t>2026-09-07 10:23:00</t>
+  </si>
+  <si>
+    <t>螢幕黑屏校正。整理排線。重新插拔變壓器</t>
+  </si>
+  <si>
+    <t>ED174115090601</t>
+  </si>
+  <si>
+    <t>D174</t>
+  </si>
+  <si>
+    <t>新莊裕民店</t>
+  </si>
+  <si>
+    <t>2026-09-06 16:20:02</t>
+  </si>
+  <si>
+    <t>門市反應TM2 CCD掃描器(HC76TR)沒有亮燈刷條碼沒有嗶聲，門職告知已有將TM重啟兩次仍無法排除，確認線路無脫落........還請台芝到店協助(掃描器故障 沒辦法刷 也沒有亮燈)</t>
+  </si>
+  <si>
+    <t>THILF0D174</t>
+  </si>
+  <si>
+    <t>2026-09-06 16:37:38</t>
+  </si>
+  <si>
+    <t>2026-09-08 09:00:00</t>
+  </si>
+  <si>
+    <t>2026-09-08 10:00:00</t>
+  </si>
+  <si>
+    <t>重裝io板排線</t>
+  </si>
+  <si>
+    <t>E3941115090701</t>
+  </si>
+  <si>
+    <t>2026-09-07 08:26:40</t>
+  </si>
+  <si>
+    <t>星期一</t>
+  </si>
+  <si>
+    <t>滑鼠故障無作用</t>
+  </si>
+  <si>
+    <t>門市反應SC滑鼠滾輪操作無反應，已嘗試重新拔插後方線路仍異常..請台芝到店協助(滾輪按了沒反應)</t>
+  </si>
+  <si>
+    <t>2026-09-07 09:04:44</t>
+  </si>
+  <si>
+    <t>2026-09-07 16:22:00</t>
+  </si>
+  <si>
+    <t>2026-09-08 13:04:00</t>
+  </si>
+  <si>
+    <t>更換滑鼠</t>
+  </si>
+  <si>
+    <t>12224115090701</t>
+  </si>
+  <si>
+    <t>板橋莒光店</t>
+  </si>
+  <si>
+    <t>2026-09-07 09:04:52</t>
+  </si>
+  <si>
+    <t>無電源反應、無法開機</t>
+  </si>
+  <si>
+    <t xml:space="preserve">09/07 09:10 與總公司宸宇確認啟動緊急叫修:門市正在盤點，反應TM1(TCX800)無電源反應無法開機，已有重新拔插線路、更換至白色插座仍無法開機，PING80不通無法VNC..請台芝到店協助與門市確認今日尚未清帳，入帳日9/7有交易PS若因更換HD.請跟店長宣達:1.請門市先回報代收會計 2.請確認SC的代收資料是否正確 (須與代收單據逐一核對)																																</t>
+  </si>
+  <si>
+    <t>THILF02224</t>
+  </si>
+  <si>
+    <t>2026-09-07 09:11:03</t>
+  </si>
+  <si>
+    <t>2026-09-07 12:53:00</t>
+  </si>
+  <si>
+    <t>2026-09-07 15:11:00</t>
+  </si>
+  <si>
+    <t>取消叫修</t>
+  </si>
+  <si>
+    <t>取消報修</t>
+  </si>
+  <si>
+    <t>1D111115090701</t>
+  </si>
+  <si>
+    <t>2026-09-07 09:14:15</t>
+  </si>
+  <si>
+    <t>2026/9/7 (週一) 上午 09:11 總公司宸宇MAIL:有關D111板橋府中店TM2(TCX800)觸控不良，請協助一般派工，到店更換UPOS211K，謝謝。</t>
+  </si>
+  <si>
+    <t>2026-09-07 09:16:03</t>
+  </si>
+  <si>
+    <t>2026-09-07 18:03:00</t>
+  </si>
+  <si>
+    <t>2026-09-08 13:16:00</t>
+  </si>
+  <si>
+    <t>更換UPOS
+換上：8185003919
+換下：8185000056</t>
+  </si>
+  <si>
+    <t>15656115090701</t>
+  </si>
+  <si>
+    <t>林口AI園區</t>
+  </si>
+  <si>
+    <t>新北市林口區</t>
+  </si>
+  <si>
+    <t>2026-09-07 09:02:43</t>
+  </si>
+  <si>
+    <t>檔案損毀(更換硬碟)</t>
+  </si>
+  <si>
+    <t>2026/9/7 (週一) 上午 09:02 總公司宸宇mail:有關5656林口AI園門市 SC(SHUTTLE7S)第一顆硬碟異常，請協助通知派工到店更換不備份還原請協助緊急派工，到店更換SC第一顆硬碟，資料不備份，謝謝。....請台芝到店協助PS.若因更換HD.請跟店長宣達:1.請門市先回報代收會計 2.請確認SC的代收資料是否正確 (須與代收單據逐一核對)																																與門市確認帳務做到09/06，與通訊功評確認有收到09/06的銷售</t>
+  </si>
+  <si>
+    <t>THILF05656</t>
+  </si>
+  <si>
+    <t>2026-09-07 09:17:01</t>
+  </si>
+  <si>
+    <t>2026-09-07 11:00:00</t>
+  </si>
+  <si>
+    <t>2026-09-07 14:00:00</t>
+  </si>
+  <si>
+    <t>2026-09-07 15:17:00</t>
+  </si>
+  <si>
+    <t>更換第一顆硬碟不備份還原完成</t>
+  </si>
+  <si>
+    <t>2026-09-07 12:22:54</t>
+  </si>
+  <si>
+    <t>2026-09-07 12:12:00</t>
+  </si>
+  <si>
+    <t>L534</t>
+  </si>
+  <si>
+    <t>田倉文興店</t>
+  </si>
+  <si>
+    <t>THILF0L534</t>
+  </si>
+  <si>
+    <t>2026-09-07 14:33:26</t>
+  </si>
+  <si>
+    <t>2026-09-07 14:10:00</t>
+  </si>
+  <si>
+    <t>2026-09-07 14:20:00</t>
+  </si>
+  <si>
+    <t>新莊莊民店</t>
+  </si>
+  <si>
+    <t>THILF03652</t>
+  </si>
+  <si>
+    <t>2026-09-07 14:38:02</t>
+  </si>
+  <si>
+    <t>2026-09-07 14:45:00</t>
+  </si>
+  <si>
+    <t>回裝</t>
+  </si>
+  <si>
+    <t>L533</t>
+  </si>
+  <si>
+    <t>田倉復興店</t>
+  </si>
+  <si>
+    <t>THILF0L533</t>
+  </si>
+  <si>
+    <t>2026-09-07 14:49:20</t>
+  </si>
+  <si>
+    <t>2026-09-07 14:30:00</t>
+  </si>
+  <si>
+    <t>2026-09-07 14:40:00</t>
+  </si>
+  <si>
+    <t>龜山文化二</t>
+  </si>
+  <si>
+    <t>THILF02428</t>
+  </si>
+  <si>
+    <t>2026-09-07 15:20:09</t>
+  </si>
+  <si>
+    <t>2026-09-07 14:50:00</t>
+  </si>
+  <si>
+    <t>2026-09-07 15:10:00</t>
+  </si>
+  <si>
+    <t>龜山復恆店</t>
+  </si>
+  <si>
+    <t>THILF04503</t>
+  </si>
+  <si>
+    <t>2026-09-07 15:45:54</t>
+  </si>
+  <si>
+    <t>2026-09-07 15:20:00</t>
+  </si>
+  <si>
+    <t>2026-09-07 15:40:00</t>
+  </si>
+  <si>
+    <t>龜山樂學店</t>
+  </si>
+  <si>
+    <t>THILF04981</t>
+  </si>
+  <si>
+    <t>2026-09-07 16:21:48</t>
+  </si>
+  <si>
+    <t>2026-09-07 15:55:00</t>
+  </si>
+  <si>
+    <t>2026-09-07 16:15:00</t>
+  </si>
+  <si>
+    <t>龜山樂善店</t>
+  </si>
+  <si>
+    <t>THILF05016</t>
+  </si>
+  <si>
+    <t>2026-09-07 16:58:29</t>
+  </si>
+  <si>
+    <t>2026-09-07 16:50:00</t>
+  </si>
+  <si>
+    <t>2026-09-07 17:30:01</t>
+  </si>
+  <si>
+    <t>2026-09-07 15:00:00</t>
+  </si>
+  <si>
+    <t>13652115090701</t>
+  </si>
+  <si>
+    <t>2026-09-07 17:27:55</t>
+  </si>
+  <si>
+    <t>不能連線</t>
+  </si>
+  <si>
+    <t>hub(DES1210-28)門市09/07回裝，門市進線告知突然無網路，ping全店僅90、91通，門市告知查看hub僅13port有亮燈，將hub線路重新拔插仍異常，協助開放91hub所有孔位請門市測試將1port插至2port仍ping不通...請台芝到店協助</t>
+  </si>
+  <si>
+    <t>2026-09-07 17:31:01</t>
+  </si>
+  <si>
+    <t>2026-09-07 18:30:00</t>
+  </si>
+  <si>
+    <t>2026-09-07 19:00:00</t>
+  </si>
+  <si>
+    <t>2026-09-08 10:31:00</t>
+  </si>
+  <si>
+    <t>更換HUB
+換下8107005368
+換上8107005406</t>
+  </si>
+  <si>
+    <t>泰山泰富店</t>
+  </si>
+  <si>
+    <t>新北市泰山區</t>
+  </si>
+  <si>
+    <t>THILF03606</t>
+  </si>
+  <si>
+    <t>2026-09-08 11:31:19</t>
+  </si>
+  <si>
+    <t>2026-09-08 10:30:00</t>
+  </si>
+  <si>
+    <t>2026-09-08 10:50:00</t>
+  </si>
+  <si>
+    <t>龜山連莊店</t>
+  </si>
+  <si>
+    <t>THILF04933</t>
+  </si>
+  <si>
+    <t>2026-09-08 12:06:29</t>
+  </si>
+  <si>
+    <t>2026-09-08 11:40:00</t>
+  </si>
+  <si>
+    <t>2026-09-08 12:00:00</t>
+  </si>
+  <si>
+    <t>15604115090801</t>
+  </si>
+  <si>
+    <t>龜山長壽店</t>
+  </si>
+  <si>
+    <t>2026-09-08 12:57:23</t>
+  </si>
+  <si>
+    <t>2026年07月份 HUB週期維護:8PORT插在9PORT</t>
+  </si>
+  <si>
+    <t>THILF05604</t>
+  </si>
+  <si>
+    <t>2026-09-08 12:59:23</t>
+  </si>
+  <si>
+    <t>2026-09-08 12:33:00</t>
+  </si>
+  <si>
+    <t>2026-09-08 13:03:00</t>
+  </si>
+  <si>
+    <t>2026-09-09 16:59:00</t>
+  </si>
+  <si>
+    <t>將HUB其中9PORT改回8PORT
++HUB</t>
+  </si>
+  <si>
+    <t>龜山同福店</t>
+  </si>
+  <si>
+    <t>THILF04690</t>
+  </si>
+  <si>
+    <t>2026-09-08 13:33:07</t>
+  </si>
+  <si>
+    <t>2026-09-08 13:20:00</t>
+  </si>
+  <si>
+    <t>板橋板豐店</t>
+  </si>
+  <si>
+    <t>THILF03551</t>
+  </si>
+  <si>
+    <t>2026-09-08 14:20:08</t>
+  </si>
+  <si>
+    <t>2026-09-08 11:00:00</t>
+  </si>
+  <si>
+    <t>2026-09-08 14:20:00</t>
+  </si>
+  <si>
+    <t>裝潢回裝已完工
+使用ADSL、商顯已安裝</t>
+  </si>
+  <si>
+    <t>2026-09-08 14:20:37</t>
+  </si>
+  <si>
+    <t>2026-09-08 14:00:00</t>
+  </si>
+  <si>
+    <t>裝潢回裝</t>
+  </si>
+  <si>
+    <t>龜山大同店</t>
+  </si>
+  <si>
+    <t>THILF03017</t>
+  </si>
+  <si>
+    <t>2026-09-08 14:38:02</t>
+  </si>
+  <si>
+    <t>2026-09-08 14:10:00</t>
+  </si>
+  <si>
+    <t>2026-09-08 14:30:00</t>
+  </si>
+  <si>
+    <t>中和國際店</t>
+  </si>
+  <si>
+    <t>THILF02180</t>
+  </si>
+  <si>
+    <t>2026-09-08 16:59:04</t>
+  </si>
+  <si>
+    <t>2026-09-08 16:35:00</t>
+  </si>
+  <si>
+    <t>2026-09-08 16:57:00</t>
   </si>
 </sst>
 </file>
@@ -1301,7 +2051,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AK32"/>
+  <dimension ref="A1:AK64"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="true" style="0"/>
@@ -3784,7 +4534,7 @@
         <v>38</v>
       </c>
       <c r="C30" s="3">
-        <v>2026090897</v>
+        <v>2026090896</v>
       </c>
       <c r="D30" s="3" t="s">
         <v>261</v>
@@ -3793,16 +4543,16 @@
         <v>40</v>
       </c>
       <c r="F30" s="3">
-        <v>2543</v>
+        <v>3941</v>
       </c>
       <c r="G30" s="3" t="s">
         <v>262</v>
       </c>
       <c r="H30" s="3" t="s">
-        <v>42</v>
+        <v>263</v>
       </c>
       <c r="I30" s="3" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="J30" s="3" t="s">
         <v>250</v>
@@ -3811,22 +4561,22 @@
         <v>45</v>
       </c>
       <c r="L30" s="3" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="M30" s="4" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="N30" s="3">
-        <v>3404</v>
+        <v>2402</v>
       </c>
       <c r="O30" s="4" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="P30" s="10" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="Q30" s="3" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="R30" s="3" t="s">
         <v>51</v>
@@ -3841,16 +4591,16 @@
         <v>53</v>
       </c>
       <c r="V30" s="3" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="W30" s="3" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="X30" s="3" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="Y30" s="3" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="Z30" s="3">
         <v>0.3</v>
@@ -3860,7 +4610,7 @@
         <v>58</v>
       </c>
       <c r="AC30" s="10" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="AD30" s="3"/>
       <c r="AE30" s="3"/>
@@ -3878,38 +4628,58 @@
         <v>29</v>
       </c>
       <c r="B31" s="7" t="s">
-        <v>61</v>
+        <v>38</v>
       </c>
       <c r="C31" s="7">
-        <v>2026090919</v>
-      </c>
-      <c r="D31" s="7"/>
-      <c r="E31" s="7"/>
-      <c r="F31" s="7" t="s">
-        <v>274</v>
+        <v>2026090897</v>
+      </c>
+      <c r="D31" s="7" t="s">
+        <v>275</v>
+      </c>
+      <c r="E31" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="F31" s="7">
+        <v>2543</v>
       </c>
       <c r="G31" s="7" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="H31" s="7" t="s">
-        <v>140</v>
-      </c>
-      <c r="I31" s="7"/>
-      <c r="J31" s="7"/>
-      <c r="K31" s="7"/>
-      <c r="L31" s="7"/>
-      <c r="M31" s="8"/>
-      <c r="N31" s="7"/>
-      <c r="O31" s="8"/>
-      <c r="P31" s="9"/>
+        <v>42</v>
+      </c>
+      <c r="I31" s="7" t="s">
+        <v>277</v>
+      </c>
+      <c r="J31" s="7" t="s">
+        <v>250</v>
+      </c>
+      <c r="K31" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="L31" s="7" t="s">
+        <v>278</v>
+      </c>
+      <c r="M31" s="8" t="s">
+        <v>279</v>
+      </c>
+      <c r="N31" s="7">
+        <v>3404</v>
+      </c>
+      <c r="O31" s="8" t="s">
+        <v>280</v>
+      </c>
+      <c r="P31" s="9" t="s">
+        <v>281</v>
+      </c>
       <c r="Q31" s="7" t="s">
-        <v>276</v>
+        <v>282</v>
       </c>
       <c r="R31" s="7" t="s">
         <v>51</v>
       </c>
       <c r="S31" s="7" t="s">
-        <v>92</v>
+        <v>52</v>
       </c>
       <c r="T31" s="7">
         <v>1</v>
@@ -3918,29 +4688,29 @@
         <v>53</v>
       </c>
       <c r="V31" s="7" t="s">
-        <v>277</v>
+        <v>283</v>
       </c>
       <c r="W31" s="7" t="s">
-        <v>278</v>
+        <v>284</v>
       </c>
       <c r="X31" s="7" t="s">
-        <v>279</v>
-      </c>
-      <c r="Y31" s="7"/>
+        <v>285</v>
+      </c>
+      <c r="Y31" s="7" t="s">
+        <v>286</v>
+      </c>
       <c r="Z31" s="7">
-        <v>0.6</v>
+        <v>0.3</v>
       </c>
       <c r="AA31" s="7"/>
       <c r="AB31" s="7" t="s">
         <v>58</v>
       </c>
       <c r="AC31" s="9" t="s">
-        <v>280</v>
+        <v>287</v>
       </c>
       <c r="AD31" s="7"/>
-      <c r="AE31" s="7" t="s">
-        <v>60</v>
-      </c>
+      <c r="AE31" s="7"/>
       <c r="AF31" s="7"/>
       <c r="AG31" s="7"/>
       <c r="AH31" s="7"/>
@@ -3958,15 +4728,15 @@
         <v>61</v>
       </c>
       <c r="C32" s="3">
-        <v>2026090921</v>
+        <v>2026090919</v>
       </c>
       <c r="D32" s="3"/>
       <c r="E32" s="3"/>
       <c r="F32" s="3" t="s">
-        <v>274</v>
+        <v>288</v>
       </c>
       <c r="G32" s="3" t="s">
-        <v>275</v>
+        <v>289</v>
       </c>
       <c r="H32" s="3" t="s">
         <v>140</v>
@@ -3978,15 +4748,15 @@
       <c r="M32" s="4"/>
       <c r="N32" s="3"/>
       <c r="O32" s="4"/>
-      <c r="P32" s="4"/>
+      <c r="P32" s="10"/>
       <c r="Q32" s="3" t="s">
-        <v>276</v>
+        <v>290</v>
       </c>
       <c r="R32" s="3" t="s">
         <v>51</v>
       </c>
       <c r="S32" s="3" t="s">
-        <v>52</v>
+        <v>92</v>
       </c>
       <c r="T32" s="3">
         <v>1</v>
@@ -3995,24 +4765,24 @@
         <v>53</v>
       </c>
       <c r="V32" s="3" t="s">
-        <v>281</v>
+        <v>291</v>
       </c>
       <c r="W32" s="3" t="s">
-        <v>282</v>
+        <v>292</v>
       </c>
       <c r="X32" s="3" t="s">
-        <v>283</v>
+        <v>293</v>
       </c>
       <c r="Y32" s="3"/>
       <c r="Z32" s="3">
-        <v>0.1</v>
+        <v>0.6</v>
       </c>
       <c r="AA32" s="3"/>
       <c r="AB32" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="AC32" s="4" t="s">
-        <v>284</v>
+      <c r="AC32" s="10" t="s">
+        <v>294</v>
       </c>
       <c r="AD32" s="3"/>
       <c r="AE32" s="3" t="s">
@@ -4024,6 +4794,2776 @@
       <c r="AI32" s="3"/>
       <c r="AJ32" s="3"/>
       <c r="AK32" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="33" spans="1:37">
+      <c r="A33" s="7">
+        <v>31</v>
+      </c>
+      <c r="B33" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="C33" s="7">
+        <v>2026090921</v>
+      </c>
+      <c r="D33" s="7"/>
+      <c r="E33" s="7"/>
+      <c r="F33" s="7" t="s">
+        <v>288</v>
+      </c>
+      <c r="G33" s="7" t="s">
+        <v>289</v>
+      </c>
+      <c r="H33" s="7" t="s">
+        <v>140</v>
+      </c>
+      <c r="I33" s="7"/>
+      <c r="J33" s="7"/>
+      <c r="K33" s="7"/>
+      <c r="L33" s="7"/>
+      <c r="M33" s="8"/>
+      <c r="N33" s="7"/>
+      <c r="O33" s="8"/>
+      <c r="P33" s="9"/>
+      <c r="Q33" s="7" t="s">
+        <v>290</v>
+      </c>
+      <c r="R33" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S33" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="T33" s="7">
+        <v>1</v>
+      </c>
+      <c r="U33" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V33" s="7" t="s">
+        <v>295</v>
+      </c>
+      <c r="W33" s="7" t="s">
+        <v>296</v>
+      </c>
+      <c r="X33" s="7" t="s">
+        <v>297</v>
+      </c>
+      <c r="Y33" s="7"/>
+      <c r="Z33" s="7">
+        <v>0.1</v>
+      </c>
+      <c r="AA33" s="7"/>
+      <c r="AB33" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC33" s="9" t="s">
+        <v>298</v>
+      </c>
+      <c r="AD33" s="7"/>
+      <c r="AE33" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AF33" s="7"/>
+      <c r="AG33" s="7"/>
+      <c r="AH33" s="7"/>
+      <c r="AI33" s="7"/>
+      <c r="AJ33" s="7"/>
+      <c r="AK33" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="34" spans="1:37">
+      <c r="A34" s="3">
+        <v>32</v>
+      </c>
+      <c r="B34" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="C34" s="3">
+        <v>2026091001</v>
+      </c>
+      <c r="D34" s="3" t="s">
+        <v>299</v>
+      </c>
+      <c r="E34" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="F34" s="3">
+        <v>4098</v>
+      </c>
+      <c r="G34" s="3" t="s">
+        <v>300</v>
+      </c>
+      <c r="H34" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="I34" s="3" t="s">
+        <v>301</v>
+      </c>
+      <c r="J34" s="3" t="s">
+        <v>250</v>
+      </c>
+      <c r="K34" s="3" t="s">
+        <v>186</v>
+      </c>
+      <c r="L34" s="3" t="s">
+        <v>302</v>
+      </c>
+      <c r="M34" s="4" t="s">
+        <v>303</v>
+      </c>
+      <c r="N34" s="3" t="s">
+        <v>304</v>
+      </c>
+      <c r="O34" s="4" t="s">
+        <v>305</v>
+      </c>
+      <c r="P34" s="10" t="s">
+        <v>306</v>
+      </c>
+      <c r="Q34" s="3" t="s">
+        <v>307</v>
+      </c>
+      <c r="R34" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S34" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="T34" s="3">
+        <v>1</v>
+      </c>
+      <c r="U34" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V34" s="3" t="s">
+        <v>308</v>
+      </c>
+      <c r="W34" s="3" t="s">
+        <v>309</v>
+      </c>
+      <c r="X34" s="3" t="s">
+        <v>310</v>
+      </c>
+      <c r="Y34" s="3" t="s">
+        <v>311</v>
+      </c>
+      <c r="Z34" s="3">
+        <v>0.8</v>
+      </c>
+      <c r="AA34" s="3"/>
+      <c r="AB34" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC34" s="10" t="s">
+        <v>312</v>
+      </c>
+      <c r="AD34" s="3"/>
+      <c r="AE34" s="3"/>
+      <c r="AF34" s="3"/>
+      <c r="AG34" s="3"/>
+      <c r="AH34" s="3"/>
+      <c r="AI34" s="3"/>
+      <c r="AJ34" s="3"/>
+      <c r="AK34" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="35" spans="1:37">
+      <c r="A35" s="7">
+        <v>33</v>
+      </c>
+      <c r="B35" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="C35" s="7">
+        <v>2026091002</v>
+      </c>
+      <c r="D35" s="7" t="s">
+        <v>313</v>
+      </c>
+      <c r="E35" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="F35" s="7">
+        <v>3227</v>
+      </c>
+      <c r="G35" s="7" t="s">
+        <v>314</v>
+      </c>
+      <c r="H35" s="7" t="s">
+        <v>315</v>
+      </c>
+      <c r="I35" s="7" t="s">
+        <v>316</v>
+      </c>
+      <c r="J35" s="7" t="s">
+        <v>317</v>
+      </c>
+      <c r="K35" s="7" t="s">
+        <v>72</v>
+      </c>
+      <c r="L35" s="7" t="s">
+        <v>73</v>
+      </c>
+      <c r="M35" s="8" t="s">
+        <v>74</v>
+      </c>
+      <c r="N35" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="O35" s="8" t="s">
+        <v>76</v>
+      </c>
+      <c r="P35" s="9" t="s">
+        <v>318</v>
+      </c>
+      <c r="Q35" s="7" t="s">
+        <v>319</v>
+      </c>
+      <c r="R35" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S35" s="7" t="s">
+        <v>320</v>
+      </c>
+      <c r="T35" s="7">
+        <v>1</v>
+      </c>
+      <c r="U35" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V35" s="7" t="s">
+        <v>321</v>
+      </c>
+      <c r="W35" s="7" t="s">
+        <v>322</v>
+      </c>
+      <c r="X35" s="7" t="s">
+        <v>323</v>
+      </c>
+      <c r="Y35" s="7" t="s">
+        <v>324</v>
+      </c>
+      <c r="Z35" s="7">
+        <v>0.5</v>
+      </c>
+      <c r="AA35" s="7"/>
+      <c r="AB35" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC35" s="9" t="s">
+        <v>325</v>
+      </c>
+      <c r="AD35" s="7"/>
+      <c r="AE35" s="7"/>
+      <c r="AF35" s="7"/>
+      <c r="AG35" s="7"/>
+      <c r="AH35" s="7"/>
+      <c r="AI35" s="7"/>
+      <c r="AJ35" s="7"/>
+      <c r="AK35" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="36" spans="1:37">
+      <c r="A36" s="3">
+        <v>34</v>
+      </c>
+      <c r="B36" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="C36" s="3">
+        <v>2026091003</v>
+      </c>
+      <c r="D36" s="3" t="s">
+        <v>326</v>
+      </c>
+      <c r="E36" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="F36" s="3">
+        <v>4856</v>
+      </c>
+      <c r="G36" s="3" t="s">
+        <v>327</v>
+      </c>
+      <c r="H36" s="3" t="s">
+        <v>328</v>
+      </c>
+      <c r="I36" s="3" t="s">
+        <v>329</v>
+      </c>
+      <c r="J36" s="3" t="s">
+        <v>317</v>
+      </c>
+      <c r="K36" s="3" t="s">
+        <v>127</v>
+      </c>
+      <c r="L36" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="M36" s="4" t="s">
+        <v>129</v>
+      </c>
+      <c r="N36" s="3" t="s">
+        <v>130</v>
+      </c>
+      <c r="O36" s="4" t="s">
+        <v>131</v>
+      </c>
+      <c r="P36" s="10" t="s">
+        <v>330</v>
+      </c>
+      <c r="Q36" s="3" t="s">
+        <v>331</v>
+      </c>
+      <c r="R36" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S36" s="3" t="s">
+        <v>320</v>
+      </c>
+      <c r="T36" s="3">
+        <v>1</v>
+      </c>
+      <c r="U36" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V36" s="3" t="s">
+        <v>332</v>
+      </c>
+      <c r="W36" s="3" t="s">
+        <v>333</v>
+      </c>
+      <c r="X36" s="3" t="s">
+        <v>334</v>
+      </c>
+      <c r="Y36" s="3" t="s">
+        <v>324</v>
+      </c>
+      <c r="Z36" s="3">
+        <v>0.5</v>
+      </c>
+      <c r="AA36" s="3"/>
+      <c r="AB36" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC36" s="10" t="s">
+        <v>335</v>
+      </c>
+      <c r="AD36" s="3"/>
+      <c r="AE36" s="3"/>
+      <c r="AF36" s="3"/>
+      <c r="AG36" s="3"/>
+      <c r="AH36" s="3"/>
+      <c r="AI36" s="3"/>
+      <c r="AJ36" s="3"/>
+      <c r="AK36" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="37" spans="1:37">
+      <c r="A37" s="7">
+        <v>35</v>
+      </c>
+      <c r="B37" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="C37" s="7">
+        <v>2026091007</v>
+      </c>
+      <c r="D37" s="7" t="s">
+        <v>336</v>
+      </c>
+      <c r="E37" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="F37" s="7">
+        <v>3890</v>
+      </c>
+      <c r="G37" s="7" t="s">
+        <v>337</v>
+      </c>
+      <c r="H37" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="I37" s="7" t="s">
+        <v>338</v>
+      </c>
+      <c r="J37" s="7" t="s">
+        <v>317</v>
+      </c>
+      <c r="K37" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="L37" s="7" t="s">
+        <v>339</v>
+      </c>
+      <c r="M37" s="8" t="s">
+        <v>340</v>
+      </c>
+      <c r="N37" s="7" t="s">
+        <v>341</v>
+      </c>
+      <c r="O37" s="8" t="s">
+        <v>342</v>
+      </c>
+      <c r="P37" s="9" t="s">
+        <v>343</v>
+      </c>
+      <c r="Q37" s="7" t="s">
+        <v>344</v>
+      </c>
+      <c r="R37" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S37" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="T37" s="7">
+        <v>1</v>
+      </c>
+      <c r="U37" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V37" s="7" t="s">
+        <v>345</v>
+      </c>
+      <c r="W37" s="7" t="s">
+        <v>346</v>
+      </c>
+      <c r="X37" s="7" t="s">
+        <v>347</v>
+      </c>
+      <c r="Y37" s="7" t="s">
+        <v>324</v>
+      </c>
+      <c r="Z37" s="7">
+        <v>0.3</v>
+      </c>
+      <c r="AA37" s="7"/>
+      <c r="AB37" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC37" s="9" t="s">
+        <v>348</v>
+      </c>
+      <c r="AD37" s="7"/>
+      <c r="AE37" s="7"/>
+      <c r="AF37" s="7"/>
+      <c r="AG37" s="7"/>
+      <c r="AH37" s="7"/>
+      <c r="AI37" s="7"/>
+      <c r="AJ37" s="7"/>
+      <c r="AK37" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="38" spans="1:37">
+      <c r="A38" s="3">
+        <v>36</v>
+      </c>
+      <c r="B38" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="C38" s="3">
+        <v>2026091008</v>
+      </c>
+      <c r="D38" s="3" t="s">
+        <v>349</v>
+      </c>
+      <c r="E38" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="F38" s="3" t="s">
+        <v>151</v>
+      </c>
+      <c r="G38" s="3" t="s">
+        <v>152</v>
+      </c>
+      <c r="H38" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="I38" s="3" t="s">
+        <v>350</v>
+      </c>
+      <c r="J38" s="3" t="s">
+        <v>317</v>
+      </c>
+      <c r="K38" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="L38" s="3" t="s">
+        <v>155</v>
+      </c>
+      <c r="M38" s="4" t="s">
+        <v>156</v>
+      </c>
+      <c r="N38" s="3">
+        <v>2307</v>
+      </c>
+      <c r="O38" s="4" t="s">
+        <v>157</v>
+      </c>
+      <c r="P38" s="10" t="s">
+        <v>351</v>
+      </c>
+      <c r="Q38" s="3" t="s">
+        <v>159</v>
+      </c>
+      <c r="R38" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S38" s="3" t="s">
+        <v>160</v>
+      </c>
+      <c r="T38" s="3">
+        <v>1</v>
+      </c>
+      <c r="U38" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V38" s="3" t="s">
+        <v>352</v>
+      </c>
+      <c r="W38" s="3" t="s">
+        <v>353</v>
+      </c>
+      <c r="X38" s="3" t="s">
+        <v>354</v>
+      </c>
+      <c r="Y38" s="3" t="s">
+        <v>324</v>
+      </c>
+      <c r="Z38" s="3">
+        <v>2.4</v>
+      </c>
+      <c r="AA38" s="3"/>
+      <c r="AB38" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC38" s="10" t="s">
+        <v>355</v>
+      </c>
+      <c r="AD38" s="3"/>
+      <c r="AE38" s="3"/>
+      <c r="AF38" s="3"/>
+      <c r="AG38" s="3"/>
+      <c r="AH38" s="3"/>
+      <c r="AI38" s="3"/>
+      <c r="AJ38" s="3"/>
+      <c r="AK38" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="39" spans="1:37">
+      <c r="A39" s="7">
+        <v>37</v>
+      </c>
+      <c r="B39" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="C39" s="7">
+        <v>2026091010</v>
+      </c>
+      <c r="D39" s="7" t="s">
+        <v>356</v>
+      </c>
+      <c r="E39" s="7" t="s">
+        <v>357</v>
+      </c>
+      <c r="F39" s="7" t="s">
+        <v>358</v>
+      </c>
+      <c r="G39" s="7" t="s">
+        <v>359</v>
+      </c>
+      <c r="H39" s="7" t="s">
+        <v>360</v>
+      </c>
+      <c r="I39" s="7" t="s">
+        <v>361</v>
+      </c>
+      <c r="J39" s="7" t="s">
+        <v>317</v>
+      </c>
+      <c r="K39" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="L39" s="7" t="s">
+        <v>265</v>
+      </c>
+      <c r="M39" s="8" t="s">
+        <v>266</v>
+      </c>
+      <c r="N39" s="7">
+        <v>2401</v>
+      </c>
+      <c r="O39" s="8" t="s">
+        <v>362</v>
+      </c>
+      <c r="P39" s="9" t="s">
+        <v>363</v>
+      </c>
+      <c r="Q39" s="7" t="s">
+        <v>364</v>
+      </c>
+      <c r="R39" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S39" s="7" t="s">
+        <v>320</v>
+      </c>
+      <c r="T39" s="7">
+        <v>1</v>
+      </c>
+      <c r="U39" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V39" s="7" t="s">
+        <v>365</v>
+      </c>
+      <c r="W39" s="7" t="s">
+        <v>366</v>
+      </c>
+      <c r="X39" s="7" t="s">
+        <v>367</v>
+      </c>
+      <c r="Y39" s="7" t="s">
+        <v>368</v>
+      </c>
+      <c r="Z39" s="7">
+        <v>1</v>
+      </c>
+      <c r="AA39" s="7"/>
+      <c r="AB39" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC39" s="9" t="s">
+        <v>369</v>
+      </c>
+      <c r="AD39" s="7"/>
+      <c r="AE39" s="7"/>
+      <c r="AF39" s="7"/>
+      <c r="AG39" s="7"/>
+      <c r="AH39" s="7"/>
+      <c r="AI39" s="7"/>
+      <c r="AJ39" s="7"/>
+      <c r="AK39" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="40" spans="1:37">
+      <c r="A40" s="3">
+        <v>38</v>
+      </c>
+      <c r="B40" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="C40" s="3">
+        <v>2026091012</v>
+      </c>
+      <c r="D40" s="3" t="s">
+        <v>370</v>
+      </c>
+      <c r="E40" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="F40" s="3">
+        <v>4397</v>
+      </c>
+      <c r="G40" s="3" t="s">
+        <v>371</v>
+      </c>
+      <c r="H40" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="I40" s="3" t="s">
+        <v>372</v>
+      </c>
+      <c r="J40" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="K40" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="L40" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="M40" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="N40" s="3">
+        <v>6003</v>
+      </c>
+      <c r="O40" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="P40" s="10" t="s">
+        <v>373</v>
+      </c>
+      <c r="Q40" s="3" t="s">
+        <v>374</v>
+      </c>
+      <c r="R40" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S40" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="T40" s="3">
+        <v>1</v>
+      </c>
+      <c r="U40" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V40" s="3" t="s">
+        <v>375</v>
+      </c>
+      <c r="W40" s="3" t="s">
+        <v>376</v>
+      </c>
+      <c r="X40" s="3" t="s">
+        <v>377</v>
+      </c>
+      <c r="Y40" s="3" t="s">
+        <v>324</v>
+      </c>
+      <c r="Z40" s="3">
+        <v>0.3</v>
+      </c>
+      <c r="AA40" s="3"/>
+      <c r="AB40" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC40" s="10" t="s">
+        <v>378</v>
+      </c>
+      <c r="AD40" s="3"/>
+      <c r="AE40" s="3"/>
+      <c r="AF40" s="3"/>
+      <c r="AG40" s="3"/>
+      <c r="AH40" s="3"/>
+      <c r="AI40" s="3"/>
+      <c r="AJ40" s="3"/>
+      <c r="AK40" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="41" spans="1:37">
+      <c r="A41" s="7">
+        <v>39</v>
+      </c>
+      <c r="B41" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="C41" s="7">
+        <v>2026091015</v>
+      </c>
+      <c r="D41" s="7" t="s">
+        <v>379</v>
+      </c>
+      <c r="E41" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="F41" s="7">
+        <v>4260</v>
+      </c>
+      <c r="G41" s="7" t="s">
+        <v>380</v>
+      </c>
+      <c r="H41" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="I41" s="7" t="s">
+        <v>381</v>
+      </c>
+      <c r="J41" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="K41" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="L41" s="7" t="s">
+        <v>155</v>
+      </c>
+      <c r="M41" s="8" t="s">
+        <v>156</v>
+      </c>
+      <c r="N41" s="7">
+        <v>2302</v>
+      </c>
+      <c r="O41" s="8" t="s">
+        <v>382</v>
+      </c>
+      <c r="P41" s="9" t="s">
+        <v>383</v>
+      </c>
+      <c r="Q41" s="7" t="s">
+        <v>384</v>
+      </c>
+      <c r="R41" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S41" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="T41" s="7">
+        <v>1</v>
+      </c>
+      <c r="U41" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V41" s="7" t="s">
+        <v>385</v>
+      </c>
+      <c r="W41" s="7" t="s">
+        <v>386</v>
+      </c>
+      <c r="X41" s="7" t="s">
+        <v>387</v>
+      </c>
+      <c r="Y41" s="7" t="s">
+        <v>324</v>
+      </c>
+      <c r="Z41" s="7">
+        <v>0.5</v>
+      </c>
+      <c r="AA41" s="7"/>
+      <c r="AB41" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC41" s="9" t="s">
+        <v>388</v>
+      </c>
+      <c r="AD41" s="7"/>
+      <c r="AE41" s="7"/>
+      <c r="AF41" s="7"/>
+      <c r="AG41" s="7"/>
+      <c r="AH41" s="7"/>
+      <c r="AI41" s="7"/>
+      <c r="AJ41" s="7"/>
+      <c r="AK41" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="42" spans="1:37">
+      <c r="A42" s="3">
+        <v>40</v>
+      </c>
+      <c r="B42" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="C42" s="3">
+        <v>2026091016</v>
+      </c>
+      <c r="D42" s="3" t="s">
+        <v>389</v>
+      </c>
+      <c r="E42" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="F42" s="3" t="s">
+        <v>390</v>
+      </c>
+      <c r="G42" s="3" t="s">
+        <v>391</v>
+      </c>
+      <c r="H42" s="3" t="s">
+        <v>328</v>
+      </c>
+      <c r="I42" s="3" t="s">
+        <v>392</v>
+      </c>
+      <c r="J42" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="K42" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="L42" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="M42" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="N42" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="O42" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="P42" s="10" t="s">
+        <v>393</v>
+      </c>
+      <c r="Q42" s="3" t="s">
+        <v>394</v>
+      </c>
+      <c r="R42" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S42" s="3" t="s">
+        <v>320</v>
+      </c>
+      <c r="T42" s="3">
+        <v>1</v>
+      </c>
+      <c r="U42" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V42" s="3" t="s">
+        <v>395</v>
+      </c>
+      <c r="W42" s="3" t="s">
+        <v>396</v>
+      </c>
+      <c r="X42" s="3" t="s">
+        <v>397</v>
+      </c>
+      <c r="Y42" s="3" t="s">
+        <v>324</v>
+      </c>
+      <c r="Z42" s="3">
+        <v>1</v>
+      </c>
+      <c r="AA42" s="3"/>
+      <c r="AB42" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC42" s="10" t="s">
+        <v>398</v>
+      </c>
+      <c r="AD42" s="3"/>
+      <c r="AE42" s="3"/>
+      <c r="AF42" s="3"/>
+      <c r="AG42" s="3"/>
+      <c r="AH42" s="3"/>
+      <c r="AI42" s="3"/>
+      <c r="AJ42" s="3"/>
+      <c r="AK42" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="43" spans="1:37">
+      <c r="A43" s="7">
+        <v>41</v>
+      </c>
+      <c r="B43" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="C43" s="7">
+        <v>2026091022</v>
+      </c>
+      <c r="D43" s="7" t="s">
+        <v>399</v>
+      </c>
+      <c r="E43" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="F43" s="7">
+        <v>3941</v>
+      </c>
+      <c r="G43" s="7" t="s">
+        <v>262</v>
+      </c>
+      <c r="H43" s="7" t="s">
+        <v>263</v>
+      </c>
+      <c r="I43" s="7" t="s">
+        <v>400</v>
+      </c>
+      <c r="J43" s="7" t="s">
+        <v>401</v>
+      </c>
+      <c r="K43" s="7" t="s">
+        <v>72</v>
+      </c>
+      <c r="L43" s="7" t="s">
+        <v>265</v>
+      </c>
+      <c r="M43" s="8" t="s">
+        <v>266</v>
+      </c>
+      <c r="N43" s="7">
+        <v>2403</v>
+      </c>
+      <c r="O43" s="8" t="s">
+        <v>402</v>
+      </c>
+      <c r="P43" s="9" t="s">
+        <v>403</v>
+      </c>
+      <c r="Q43" s="7" t="s">
+        <v>269</v>
+      </c>
+      <c r="R43" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S43" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="T43" s="7">
+        <v>1</v>
+      </c>
+      <c r="U43" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V43" s="7" t="s">
+        <v>404</v>
+      </c>
+      <c r="W43" s="7" t="s">
+        <v>322</v>
+      </c>
+      <c r="X43" s="7" t="s">
+        <v>405</v>
+      </c>
+      <c r="Y43" s="7" t="s">
+        <v>406</v>
+      </c>
+      <c r="Z43" s="7">
+        <v>0.4</v>
+      </c>
+      <c r="AA43" s="7"/>
+      <c r="AB43" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC43" s="9" t="s">
+        <v>407</v>
+      </c>
+      <c r="AD43" s="7"/>
+      <c r="AE43" s="7"/>
+      <c r="AF43" s="7"/>
+      <c r="AG43" s="7"/>
+      <c r="AH43" s="7"/>
+      <c r="AI43" s="7"/>
+      <c r="AJ43" s="7"/>
+      <c r="AK43" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="44" spans="1:37">
+      <c r="A44" s="3">
+        <v>42</v>
+      </c>
+      <c r="B44" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="C44" s="3">
+        <v>2026091024</v>
+      </c>
+      <c r="D44" s="3" t="s">
+        <v>408</v>
+      </c>
+      <c r="E44" s="3" t="s">
+        <v>357</v>
+      </c>
+      <c r="F44" s="3">
+        <v>2224</v>
+      </c>
+      <c r="G44" s="3" t="s">
+        <v>409</v>
+      </c>
+      <c r="H44" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="I44" s="3" t="s">
+        <v>410</v>
+      </c>
+      <c r="J44" s="3" t="s">
+        <v>401</v>
+      </c>
+      <c r="K44" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="L44" s="3" t="s">
+        <v>155</v>
+      </c>
+      <c r="M44" s="4" t="s">
+        <v>156</v>
+      </c>
+      <c r="N44" s="3">
+        <v>2306</v>
+      </c>
+      <c r="O44" s="4" t="s">
+        <v>411</v>
+      </c>
+      <c r="P44" s="10" t="s">
+        <v>412</v>
+      </c>
+      <c r="Q44" s="3" t="s">
+        <v>413</v>
+      </c>
+      <c r="R44" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S44" s="3" t="s">
+        <v>160</v>
+      </c>
+      <c r="T44" s="3">
+        <v>1</v>
+      </c>
+      <c r="U44" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V44" s="3" t="s">
+        <v>414</v>
+      </c>
+      <c r="W44" s="3" t="s">
+        <v>415</v>
+      </c>
+      <c r="X44" s="3" t="s">
+        <v>257</v>
+      </c>
+      <c r="Y44" s="3" t="s">
+        <v>416</v>
+      </c>
+      <c r="Z44" s="3">
+        <v>0.5</v>
+      </c>
+      <c r="AA44" s="3"/>
+      <c r="AB44" s="3" t="s">
+        <v>417</v>
+      </c>
+      <c r="AC44" s="10" t="s">
+        <v>418</v>
+      </c>
+      <c r="AD44" s="3"/>
+      <c r="AE44" s="3"/>
+      <c r="AF44" s="3"/>
+      <c r="AG44" s="3"/>
+      <c r="AH44" s="3"/>
+      <c r="AI44" s="3"/>
+      <c r="AJ44" s="3"/>
+      <c r="AK44" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="45" spans="1:37">
+      <c r="A45" s="7">
+        <v>43</v>
+      </c>
+      <c r="B45" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="C45" s="7">
+        <v>2026091027</v>
+      </c>
+      <c r="D45" s="7" t="s">
+        <v>419</v>
+      </c>
+      <c r="E45" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="F45" s="7" t="s">
+        <v>151</v>
+      </c>
+      <c r="G45" s="7" t="s">
+        <v>152</v>
+      </c>
+      <c r="H45" s="7" t="s">
+        <v>153</v>
+      </c>
+      <c r="I45" s="7" t="s">
+        <v>420</v>
+      </c>
+      <c r="J45" s="7" t="s">
+        <v>401</v>
+      </c>
+      <c r="K45" s="7" t="s">
+        <v>72</v>
+      </c>
+      <c r="L45" s="7" t="s">
+        <v>155</v>
+      </c>
+      <c r="M45" s="8" t="s">
+        <v>156</v>
+      </c>
+      <c r="N45" s="7">
+        <v>2307</v>
+      </c>
+      <c r="O45" s="8" t="s">
+        <v>157</v>
+      </c>
+      <c r="P45" s="9" t="s">
+        <v>421</v>
+      </c>
+      <c r="Q45" s="7" t="s">
+        <v>159</v>
+      </c>
+      <c r="R45" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S45" s="7" t="s">
+        <v>160</v>
+      </c>
+      <c r="T45" s="7">
+        <v>1</v>
+      </c>
+      <c r="U45" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V45" s="7" t="s">
+        <v>422</v>
+      </c>
+      <c r="W45" s="7" t="s">
+        <v>353</v>
+      </c>
+      <c r="X45" s="7" t="s">
+        <v>423</v>
+      </c>
+      <c r="Y45" s="7" t="s">
+        <v>424</v>
+      </c>
+      <c r="Z45" s="7">
+        <v>2.6</v>
+      </c>
+      <c r="AA45" s="7"/>
+      <c r="AB45" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC45" s="9" t="s">
+        <v>425</v>
+      </c>
+      <c r="AD45" s="7"/>
+      <c r="AE45" s="7"/>
+      <c r="AF45" s="7"/>
+      <c r="AG45" s="7"/>
+      <c r="AH45" s="7"/>
+      <c r="AI45" s="7"/>
+      <c r="AJ45" s="7"/>
+      <c r="AK45" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="46" spans="1:37">
+      <c r="A46" s="3">
+        <v>44</v>
+      </c>
+      <c r="B46" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="C46" s="3">
+        <v>2026091029</v>
+      </c>
+      <c r="D46" s="3" t="s">
+        <v>426</v>
+      </c>
+      <c r="E46" s="3" t="s">
+        <v>357</v>
+      </c>
+      <c r="F46" s="3">
+        <v>5656</v>
+      </c>
+      <c r="G46" s="3" t="s">
+        <v>427</v>
+      </c>
+      <c r="H46" s="3" t="s">
+        <v>428</v>
+      </c>
+      <c r="I46" s="3" t="s">
+        <v>429</v>
+      </c>
+      <c r="J46" s="3" t="s">
+        <v>401</v>
+      </c>
+      <c r="K46" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="L46" s="3" t="s">
+        <v>265</v>
+      </c>
+      <c r="M46" s="4" t="s">
+        <v>266</v>
+      </c>
+      <c r="N46" s="3">
+        <v>2405</v>
+      </c>
+      <c r="O46" s="4" t="s">
+        <v>430</v>
+      </c>
+      <c r="P46" s="10" t="s">
+        <v>431</v>
+      </c>
+      <c r="Q46" s="3" t="s">
+        <v>432</v>
+      </c>
+      <c r="R46" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S46" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="T46" s="3">
+        <v>1</v>
+      </c>
+      <c r="U46" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V46" s="3" t="s">
+        <v>433</v>
+      </c>
+      <c r="W46" s="3" t="s">
+        <v>434</v>
+      </c>
+      <c r="X46" s="3" t="s">
+        <v>435</v>
+      </c>
+      <c r="Y46" s="3" t="s">
+        <v>436</v>
+      </c>
+      <c r="Z46" s="3">
+        <v>3</v>
+      </c>
+      <c r="AA46" s="3"/>
+      <c r="AB46" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC46" s="10" t="s">
+        <v>437</v>
+      </c>
+      <c r="AD46" s="3"/>
+      <c r="AE46" s="3"/>
+      <c r="AF46" s="3"/>
+      <c r="AG46" s="3"/>
+      <c r="AH46" s="3"/>
+      <c r="AI46" s="3"/>
+      <c r="AJ46" s="3"/>
+      <c r="AK46" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="47" spans="1:37">
+      <c r="A47" s="7">
+        <v>45</v>
+      </c>
+      <c r="B47" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="C47" s="7">
+        <v>2026091063</v>
+      </c>
+      <c r="D47" s="7"/>
+      <c r="E47" s="7"/>
+      <c r="F47" s="7">
+        <v>4397</v>
+      </c>
+      <c r="G47" s="7" t="s">
+        <v>371</v>
+      </c>
+      <c r="H47" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="I47" s="7"/>
+      <c r="J47" s="7"/>
+      <c r="K47" s="7"/>
+      <c r="L47" s="7"/>
+      <c r="M47" s="8"/>
+      <c r="N47" s="7"/>
+      <c r="O47" s="8"/>
+      <c r="P47" s="9"/>
+      <c r="Q47" s="7" t="s">
+        <v>374</v>
+      </c>
+      <c r="R47" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S47" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="T47" s="7">
+        <v>1</v>
+      </c>
+      <c r="U47" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V47" s="7" t="s">
+        <v>438</v>
+      </c>
+      <c r="W47" s="7" t="s">
+        <v>377</v>
+      </c>
+      <c r="X47" s="7" t="s">
+        <v>439</v>
+      </c>
+      <c r="Y47" s="7"/>
+      <c r="Z47" s="7">
+        <v>0.4</v>
+      </c>
+      <c r="AA47" s="7"/>
+      <c r="AB47" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC47" s="9" t="s">
+        <v>67</v>
+      </c>
+      <c r="AD47" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE47" s="7"/>
+      <c r="AF47" s="7"/>
+      <c r="AG47" s="7"/>
+      <c r="AH47" s="7"/>
+      <c r="AI47" s="7"/>
+      <c r="AJ47" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AK47" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="48" spans="1:37">
+      <c r="A48" s="3">
+        <v>46</v>
+      </c>
+      <c r="B48" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="C48" s="3">
+        <v>2026091076</v>
+      </c>
+      <c r="D48" s="3"/>
+      <c r="E48" s="3"/>
+      <c r="F48" s="3" t="s">
+        <v>440</v>
+      </c>
+      <c r="G48" s="3" t="s">
+        <v>441</v>
+      </c>
+      <c r="H48" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="I48" s="3"/>
+      <c r="J48" s="3"/>
+      <c r="K48" s="3"/>
+      <c r="L48" s="3"/>
+      <c r="M48" s="4"/>
+      <c r="N48" s="3"/>
+      <c r="O48" s="4"/>
+      <c r="P48" s="10"/>
+      <c r="Q48" s="3" t="s">
+        <v>442</v>
+      </c>
+      <c r="R48" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S48" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="T48" s="3">
+        <v>1</v>
+      </c>
+      <c r="U48" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V48" s="3" t="s">
+        <v>443</v>
+      </c>
+      <c r="W48" s="3" t="s">
+        <v>444</v>
+      </c>
+      <c r="X48" s="3" t="s">
+        <v>445</v>
+      </c>
+      <c r="Y48" s="3"/>
+      <c r="Z48" s="3">
+        <v>0.2</v>
+      </c>
+      <c r="AA48" s="3"/>
+      <c r="AB48" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC48" s="10" t="s">
+        <v>67</v>
+      </c>
+      <c r="AD48" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE48" s="3"/>
+      <c r="AF48" s="3"/>
+      <c r="AG48" s="3"/>
+      <c r="AH48" s="3"/>
+      <c r="AI48" s="3"/>
+      <c r="AJ48" s="3"/>
+      <c r="AK48" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="49" spans="1:37">
+      <c r="A49" s="7">
+        <v>47</v>
+      </c>
+      <c r="B49" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="C49" s="7">
+        <v>2026091080</v>
+      </c>
+      <c r="D49" s="7"/>
+      <c r="E49" s="7"/>
+      <c r="F49" s="7">
+        <v>3652</v>
+      </c>
+      <c r="G49" s="7" t="s">
+        <v>446</v>
+      </c>
+      <c r="H49" s="7" t="s">
+        <v>328</v>
+      </c>
+      <c r="I49" s="7"/>
+      <c r="J49" s="7"/>
+      <c r="K49" s="7"/>
+      <c r="L49" s="7"/>
+      <c r="M49" s="8"/>
+      <c r="N49" s="7"/>
+      <c r="O49" s="8"/>
+      <c r="P49" s="9"/>
+      <c r="Q49" s="7" t="s">
+        <v>447</v>
+      </c>
+      <c r="R49" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S49" s="7" t="s">
+        <v>320</v>
+      </c>
+      <c r="T49" s="7">
+        <v>1</v>
+      </c>
+      <c r="U49" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V49" s="7" t="s">
+        <v>448</v>
+      </c>
+      <c r="W49" s="7" t="s">
+        <v>434</v>
+      </c>
+      <c r="X49" s="7" t="s">
+        <v>449</v>
+      </c>
+      <c r="Y49" s="7"/>
+      <c r="Z49" s="7">
+        <v>3.8</v>
+      </c>
+      <c r="AA49" s="7"/>
+      <c r="AB49" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC49" s="9" t="s">
+        <v>450</v>
+      </c>
+      <c r="AD49" s="7"/>
+      <c r="AE49" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AF49" s="7"/>
+      <c r="AG49" s="7"/>
+      <c r="AH49" s="7"/>
+      <c r="AI49" s="7"/>
+      <c r="AJ49" s="7"/>
+      <c r="AK49" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="50" spans="1:37">
+      <c r="A50" s="3">
+        <v>48</v>
+      </c>
+      <c r="B50" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="C50" s="3">
+        <v>2026091081</v>
+      </c>
+      <c r="D50" s="3"/>
+      <c r="E50" s="3"/>
+      <c r="F50" s="3" t="s">
+        <v>451</v>
+      </c>
+      <c r="G50" s="3" t="s">
+        <v>452</v>
+      </c>
+      <c r="H50" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="I50" s="3"/>
+      <c r="J50" s="3"/>
+      <c r="K50" s="3"/>
+      <c r="L50" s="3"/>
+      <c r="M50" s="4"/>
+      <c r="N50" s="3"/>
+      <c r="O50" s="4"/>
+      <c r="P50" s="10"/>
+      <c r="Q50" s="3" t="s">
+        <v>453</v>
+      </c>
+      <c r="R50" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S50" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="T50" s="3">
+        <v>1</v>
+      </c>
+      <c r="U50" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V50" s="3" t="s">
+        <v>454</v>
+      </c>
+      <c r="W50" s="3" t="s">
+        <v>455</v>
+      </c>
+      <c r="X50" s="3" t="s">
+        <v>456</v>
+      </c>
+      <c r="Y50" s="3"/>
+      <c r="Z50" s="3">
+        <v>0.2</v>
+      </c>
+      <c r="AA50" s="3"/>
+      <c r="AB50" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC50" s="10" t="s">
+        <v>67</v>
+      </c>
+      <c r="AD50" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE50" s="3"/>
+      <c r="AF50" s="3"/>
+      <c r="AG50" s="3"/>
+      <c r="AH50" s="3"/>
+      <c r="AI50" s="3"/>
+      <c r="AJ50" s="3"/>
+      <c r="AK50" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="51" spans="1:37">
+      <c r="A51" s="7">
+        <v>49</v>
+      </c>
+      <c r="B51" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="C51" s="7">
+        <v>2026091088</v>
+      </c>
+      <c r="D51" s="7"/>
+      <c r="E51" s="7"/>
+      <c r="F51" s="7">
+        <v>2428</v>
+      </c>
+      <c r="G51" s="7" t="s">
+        <v>457</v>
+      </c>
+      <c r="H51" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="I51" s="7"/>
+      <c r="J51" s="7"/>
+      <c r="K51" s="7"/>
+      <c r="L51" s="7"/>
+      <c r="M51" s="8"/>
+      <c r="N51" s="7"/>
+      <c r="O51" s="8"/>
+      <c r="P51" s="9"/>
+      <c r="Q51" s="7" t="s">
+        <v>458</v>
+      </c>
+      <c r="R51" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S51" s="7" t="s">
+        <v>92</v>
+      </c>
+      <c r="T51" s="7">
+        <v>1</v>
+      </c>
+      <c r="U51" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V51" s="7" t="s">
+        <v>459</v>
+      </c>
+      <c r="W51" s="7" t="s">
+        <v>460</v>
+      </c>
+      <c r="X51" s="7" t="s">
+        <v>461</v>
+      </c>
+      <c r="Y51" s="7"/>
+      <c r="Z51" s="7">
+        <v>0.3</v>
+      </c>
+      <c r="AA51" s="7"/>
+      <c r="AB51" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC51" s="9" t="s">
+        <v>67</v>
+      </c>
+      <c r="AD51" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE51" s="7"/>
+      <c r="AF51" s="7"/>
+      <c r="AG51" s="7"/>
+      <c r="AH51" s="7"/>
+      <c r="AI51" s="7"/>
+      <c r="AJ51" s="7"/>
+      <c r="AK51" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="52" spans="1:37">
+      <c r="A52" s="3">
+        <v>50</v>
+      </c>
+      <c r="B52" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="C52" s="3">
+        <v>2026091103</v>
+      </c>
+      <c r="D52" s="3"/>
+      <c r="E52" s="3"/>
+      <c r="F52" s="3">
+        <v>4503</v>
+      </c>
+      <c r="G52" s="3" t="s">
+        <v>462</v>
+      </c>
+      <c r="H52" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="I52" s="3"/>
+      <c r="J52" s="3"/>
+      <c r="K52" s="3"/>
+      <c r="L52" s="3"/>
+      <c r="M52" s="4"/>
+      <c r="N52" s="3"/>
+      <c r="O52" s="4"/>
+      <c r="P52" s="10"/>
+      <c r="Q52" s="3" t="s">
+        <v>463</v>
+      </c>
+      <c r="R52" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S52" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="T52" s="3">
+        <v>1</v>
+      </c>
+      <c r="U52" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V52" s="3" t="s">
+        <v>464</v>
+      </c>
+      <c r="W52" s="3" t="s">
+        <v>465</v>
+      </c>
+      <c r="X52" s="3" t="s">
+        <v>466</v>
+      </c>
+      <c r="Y52" s="3"/>
+      <c r="Z52" s="3">
+        <v>0.3</v>
+      </c>
+      <c r="AA52" s="3"/>
+      <c r="AB52" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC52" s="10" t="s">
+        <v>67</v>
+      </c>
+      <c r="AD52" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE52" s="3"/>
+      <c r="AF52" s="3"/>
+      <c r="AG52" s="3"/>
+      <c r="AH52" s="3"/>
+      <c r="AI52" s="3"/>
+      <c r="AJ52" s="3"/>
+      <c r="AK52" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="53" spans="1:37">
+      <c r="A53" s="7">
+        <v>51</v>
+      </c>
+      <c r="B53" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="C53" s="7">
+        <v>2026091109</v>
+      </c>
+      <c r="D53" s="7"/>
+      <c r="E53" s="7"/>
+      <c r="F53" s="7">
+        <v>4981</v>
+      </c>
+      <c r="G53" s="7" t="s">
+        <v>467</v>
+      </c>
+      <c r="H53" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="I53" s="7"/>
+      <c r="J53" s="7"/>
+      <c r="K53" s="7"/>
+      <c r="L53" s="7"/>
+      <c r="M53" s="8"/>
+      <c r="N53" s="7"/>
+      <c r="O53" s="8"/>
+      <c r="P53" s="9"/>
+      <c r="Q53" s="7" t="s">
+        <v>468</v>
+      </c>
+      <c r="R53" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S53" s="7" t="s">
+        <v>92</v>
+      </c>
+      <c r="T53" s="7">
+        <v>1</v>
+      </c>
+      <c r="U53" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V53" s="7" t="s">
+        <v>469</v>
+      </c>
+      <c r="W53" s="7" t="s">
+        <v>470</v>
+      </c>
+      <c r="X53" s="7" t="s">
+        <v>471</v>
+      </c>
+      <c r="Y53" s="7"/>
+      <c r="Z53" s="7">
+        <v>0.3</v>
+      </c>
+      <c r="AA53" s="7"/>
+      <c r="AB53" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC53" s="9" t="s">
+        <v>67</v>
+      </c>
+      <c r="AD53" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE53" s="7"/>
+      <c r="AF53" s="7"/>
+      <c r="AG53" s="7"/>
+      <c r="AH53" s="7"/>
+      <c r="AI53" s="7"/>
+      <c r="AJ53" s="7"/>
+      <c r="AK53" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="54" spans="1:37">
+      <c r="A54" s="3">
+        <v>52</v>
+      </c>
+      <c r="B54" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="C54" s="3">
+        <v>2026091178</v>
+      </c>
+      <c r="D54" s="3"/>
+      <c r="E54" s="3"/>
+      <c r="F54" s="3">
+        <v>5016</v>
+      </c>
+      <c r="G54" s="3" t="s">
+        <v>472</v>
+      </c>
+      <c r="H54" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="I54" s="3"/>
+      <c r="J54" s="3"/>
+      <c r="K54" s="3"/>
+      <c r="L54" s="3"/>
+      <c r="M54" s="4"/>
+      <c r="N54" s="3"/>
+      <c r="O54" s="4"/>
+      <c r="P54" s="10"/>
+      <c r="Q54" s="3" t="s">
+        <v>473</v>
+      </c>
+      <c r="R54" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S54" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="T54" s="3">
+        <v>1</v>
+      </c>
+      <c r="U54" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V54" s="3" t="s">
+        <v>474</v>
+      </c>
+      <c r="W54" s="3" t="s">
+        <v>323</v>
+      </c>
+      <c r="X54" s="3" t="s">
+        <v>475</v>
+      </c>
+      <c r="Y54" s="3"/>
+      <c r="Z54" s="3">
+        <v>0.3</v>
+      </c>
+      <c r="AA54" s="3"/>
+      <c r="AB54" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC54" s="10" t="s">
+        <v>67</v>
+      </c>
+      <c r="AD54" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE54" s="3"/>
+      <c r="AF54" s="3"/>
+      <c r="AG54" s="3"/>
+      <c r="AH54" s="3"/>
+      <c r="AI54" s="3"/>
+      <c r="AJ54" s="3"/>
+      <c r="AK54" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="55" spans="1:37">
+      <c r="A55" s="7">
+        <v>53</v>
+      </c>
+      <c r="B55" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="C55" s="7">
+        <v>2026091223</v>
+      </c>
+      <c r="D55" s="7"/>
+      <c r="E55" s="7"/>
+      <c r="F55" s="7">
+        <v>3652</v>
+      </c>
+      <c r="G55" s="7" t="s">
+        <v>446</v>
+      </c>
+      <c r="H55" s="7" t="s">
+        <v>328</v>
+      </c>
+      <c r="I55" s="7"/>
+      <c r="J55" s="7"/>
+      <c r="K55" s="7"/>
+      <c r="L55" s="7"/>
+      <c r="M55" s="8"/>
+      <c r="N55" s="7"/>
+      <c r="O55" s="8"/>
+      <c r="P55" s="9"/>
+      <c r="Q55" s="7" t="s">
+        <v>447</v>
+      </c>
+      <c r="R55" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S55" s="7" t="s">
+        <v>320</v>
+      </c>
+      <c r="T55" s="7">
+        <v>1</v>
+      </c>
+      <c r="U55" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V55" s="7" t="s">
+        <v>476</v>
+      </c>
+      <c r="W55" s="7" t="s">
+        <v>449</v>
+      </c>
+      <c r="X55" s="7" t="s">
+        <v>477</v>
+      </c>
+      <c r="Y55" s="7"/>
+      <c r="Z55" s="7">
+        <v>0.3</v>
+      </c>
+      <c r="AA55" s="7"/>
+      <c r="AB55" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC55" s="9" t="s">
+        <v>67</v>
+      </c>
+      <c r="AD55" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE55" s="7"/>
+      <c r="AF55" s="7"/>
+      <c r="AG55" s="7"/>
+      <c r="AH55" s="7"/>
+      <c r="AI55" s="7"/>
+      <c r="AJ55" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AK55" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="56" spans="1:37">
+      <c r="A56" s="3">
+        <v>54</v>
+      </c>
+      <c r="B56" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="C56" s="3">
+        <v>2026091224</v>
+      </c>
+      <c r="D56" s="3" t="s">
+        <v>478</v>
+      </c>
+      <c r="E56" s="3" t="s">
+        <v>357</v>
+      </c>
+      <c r="F56" s="3">
+        <v>3652</v>
+      </c>
+      <c r="G56" s="3" t="s">
+        <v>446</v>
+      </c>
+      <c r="H56" s="3" t="s">
+        <v>328</v>
+      </c>
+      <c r="I56" s="3" t="s">
+        <v>479</v>
+      </c>
+      <c r="J56" s="3" t="s">
+        <v>401</v>
+      </c>
+      <c r="K56" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="L56" s="3" t="s">
+        <v>278</v>
+      </c>
+      <c r="M56" s="4" t="s">
+        <v>279</v>
+      </c>
+      <c r="N56" s="3">
+        <v>3402</v>
+      </c>
+      <c r="O56" s="4" t="s">
+        <v>480</v>
+      </c>
+      <c r="P56" s="10" t="s">
+        <v>481</v>
+      </c>
+      <c r="Q56" s="3" t="s">
+        <v>447</v>
+      </c>
+      <c r="R56" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S56" s="3" t="s">
+        <v>320</v>
+      </c>
+      <c r="T56" s="3">
+        <v>1</v>
+      </c>
+      <c r="U56" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V56" s="3" t="s">
+        <v>482</v>
+      </c>
+      <c r="W56" s="3" t="s">
+        <v>483</v>
+      </c>
+      <c r="X56" s="3" t="s">
+        <v>484</v>
+      </c>
+      <c r="Y56" s="3" t="s">
+        <v>485</v>
+      </c>
+      <c r="Z56" s="3">
+        <v>0.5</v>
+      </c>
+      <c r="AA56" s="3"/>
+      <c r="AB56" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC56" s="10" t="s">
+        <v>486</v>
+      </c>
+      <c r="AD56" s="3"/>
+      <c r="AE56" s="3"/>
+      <c r="AF56" s="3"/>
+      <c r="AG56" s="3"/>
+      <c r="AH56" s="3"/>
+      <c r="AI56" s="3"/>
+      <c r="AJ56" s="3"/>
+      <c r="AK56" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="57" spans="1:37">
+      <c r="A57" s="7">
+        <v>55</v>
+      </c>
+      <c r="B57" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="C57" s="7">
+        <v>2026091264</v>
+      </c>
+      <c r="D57" s="7"/>
+      <c r="E57" s="7"/>
+      <c r="F57" s="7">
+        <v>3606</v>
+      </c>
+      <c r="G57" s="7" t="s">
+        <v>487</v>
+      </c>
+      <c r="H57" s="7" t="s">
+        <v>488</v>
+      </c>
+      <c r="I57" s="7"/>
+      <c r="J57" s="7"/>
+      <c r="K57" s="7"/>
+      <c r="L57" s="7"/>
+      <c r="M57" s="8"/>
+      <c r="N57" s="7"/>
+      <c r="O57" s="8"/>
+      <c r="P57" s="9"/>
+      <c r="Q57" s="7" t="s">
+        <v>489</v>
+      </c>
+      <c r="R57" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S57" s="7" t="s">
+        <v>92</v>
+      </c>
+      <c r="T57" s="7">
+        <v>1</v>
+      </c>
+      <c r="U57" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V57" s="7" t="s">
+        <v>490</v>
+      </c>
+      <c r="W57" s="7" t="s">
+        <v>491</v>
+      </c>
+      <c r="X57" s="7" t="s">
+        <v>492</v>
+      </c>
+      <c r="Y57" s="7"/>
+      <c r="Z57" s="7">
+        <v>0.3</v>
+      </c>
+      <c r="AA57" s="7"/>
+      <c r="AB57" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC57" s="9" t="s">
+        <v>67</v>
+      </c>
+      <c r="AD57" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE57" s="7"/>
+      <c r="AF57" s="7"/>
+      <c r="AG57" s="7"/>
+      <c r="AH57" s="7"/>
+      <c r="AI57" s="7"/>
+      <c r="AJ57" s="7"/>
+      <c r="AK57" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="58" spans="1:37">
+      <c r="A58" s="3">
+        <v>56</v>
+      </c>
+      <c r="B58" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="C58" s="3">
+        <v>2026091278</v>
+      </c>
+      <c r="D58" s="3"/>
+      <c r="E58" s="3"/>
+      <c r="F58" s="3">
+        <v>4933</v>
+      </c>
+      <c r="G58" s="3" t="s">
+        <v>493</v>
+      </c>
+      <c r="H58" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="I58" s="3"/>
+      <c r="J58" s="3"/>
+      <c r="K58" s="3"/>
+      <c r="L58" s="3"/>
+      <c r="M58" s="4"/>
+      <c r="N58" s="3"/>
+      <c r="O58" s="4"/>
+      <c r="P58" s="10"/>
+      <c r="Q58" s="3" t="s">
+        <v>494</v>
+      </c>
+      <c r="R58" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S58" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="T58" s="3">
+        <v>1</v>
+      </c>
+      <c r="U58" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V58" s="3" t="s">
+        <v>495</v>
+      </c>
+      <c r="W58" s="3" t="s">
+        <v>496</v>
+      </c>
+      <c r="X58" s="3" t="s">
+        <v>497</v>
+      </c>
+      <c r="Y58" s="3"/>
+      <c r="Z58" s="3">
+        <v>0.3</v>
+      </c>
+      <c r="AA58" s="3"/>
+      <c r="AB58" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC58" s="10" t="s">
+        <v>67</v>
+      </c>
+      <c r="AD58" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE58" s="3"/>
+      <c r="AF58" s="3"/>
+      <c r="AG58" s="3"/>
+      <c r="AH58" s="3"/>
+      <c r="AI58" s="3"/>
+      <c r="AJ58" s="3"/>
+      <c r="AK58" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="59" spans="1:37">
+      <c r="A59" s="7">
+        <v>57</v>
+      </c>
+      <c r="B59" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="C59" s="7">
+        <v>2026091287</v>
+      </c>
+      <c r="D59" s="7" t="s">
+        <v>498</v>
+      </c>
+      <c r="E59" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="F59" s="7">
+        <v>5604</v>
+      </c>
+      <c r="G59" s="7" t="s">
+        <v>499</v>
+      </c>
+      <c r="H59" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="I59" s="7" t="s">
+        <v>500</v>
+      </c>
+      <c r="J59" s="7" t="s">
+        <v>71</v>
+      </c>
+      <c r="K59" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="L59" s="7" t="s">
+        <v>278</v>
+      </c>
+      <c r="M59" s="8" t="s">
+        <v>279</v>
+      </c>
+      <c r="N59" s="7">
+        <v>3404</v>
+      </c>
+      <c r="O59" s="8" t="s">
+        <v>280</v>
+      </c>
+      <c r="P59" s="9" t="s">
+        <v>501</v>
+      </c>
+      <c r="Q59" s="7" t="s">
+        <v>502</v>
+      </c>
+      <c r="R59" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S59" s="7" t="s">
+        <v>92</v>
+      </c>
+      <c r="T59" s="7">
+        <v>1</v>
+      </c>
+      <c r="U59" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V59" s="7" t="s">
+        <v>503</v>
+      </c>
+      <c r="W59" s="7" t="s">
+        <v>504</v>
+      </c>
+      <c r="X59" s="7" t="s">
+        <v>505</v>
+      </c>
+      <c r="Y59" s="7" t="s">
+        <v>506</v>
+      </c>
+      <c r="Z59" s="7">
+        <v>0.5</v>
+      </c>
+      <c r="AA59" s="7"/>
+      <c r="AB59" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC59" s="9" t="s">
+        <v>507</v>
+      </c>
+      <c r="AD59" s="7"/>
+      <c r="AE59" s="7"/>
+      <c r="AF59" s="7"/>
+      <c r="AG59" s="7"/>
+      <c r="AH59" s="7"/>
+      <c r="AI59" s="7"/>
+      <c r="AJ59" s="7"/>
+      <c r="AK59" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="60" spans="1:37">
+      <c r="A60" s="3">
+        <v>58</v>
+      </c>
+      <c r="B60" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="C60" s="3">
+        <v>2026091293</v>
+      </c>
+      <c r="D60" s="3"/>
+      <c r="E60" s="3"/>
+      <c r="F60" s="3">
+        <v>4690</v>
+      </c>
+      <c r="G60" s="3" t="s">
+        <v>508</v>
+      </c>
+      <c r="H60" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="I60" s="3"/>
+      <c r="J60" s="3"/>
+      <c r="K60" s="3"/>
+      <c r="L60" s="3"/>
+      <c r="M60" s="4"/>
+      <c r="N60" s="3"/>
+      <c r="O60" s="4"/>
+      <c r="P60" s="10"/>
+      <c r="Q60" s="3" t="s">
+        <v>509</v>
+      </c>
+      <c r="R60" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S60" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="T60" s="3">
+        <v>1</v>
+      </c>
+      <c r="U60" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V60" s="3" t="s">
+        <v>510</v>
+      </c>
+      <c r="W60" s="3" t="s">
+        <v>324</v>
+      </c>
+      <c r="X60" s="3" t="s">
+        <v>511</v>
+      </c>
+      <c r="Y60" s="3"/>
+      <c r="Z60" s="3">
+        <v>0.3</v>
+      </c>
+      <c r="AA60" s="3"/>
+      <c r="AB60" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC60" s="10" t="s">
+        <v>67</v>
+      </c>
+      <c r="AD60" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE60" s="3"/>
+      <c r="AF60" s="3"/>
+      <c r="AG60" s="3"/>
+      <c r="AH60" s="3"/>
+      <c r="AI60" s="3"/>
+      <c r="AJ60" s="3"/>
+      <c r="AK60" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="61" spans="1:37">
+      <c r="A61" s="7">
+        <v>59</v>
+      </c>
+      <c r="B61" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="C61" s="7">
+        <v>2026091391</v>
+      </c>
+      <c r="D61" s="7"/>
+      <c r="E61" s="7"/>
+      <c r="F61" s="7">
+        <v>3551</v>
+      </c>
+      <c r="G61" s="7" t="s">
+        <v>512</v>
+      </c>
+      <c r="H61" s="7" t="s">
+        <v>153</v>
+      </c>
+      <c r="I61" s="7"/>
+      <c r="J61" s="7"/>
+      <c r="K61" s="7"/>
+      <c r="L61" s="7"/>
+      <c r="M61" s="8"/>
+      <c r="N61" s="7"/>
+      <c r="O61" s="8"/>
+      <c r="P61" s="9"/>
+      <c r="Q61" s="7" t="s">
+        <v>513</v>
+      </c>
+      <c r="R61" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S61" s="7" t="s">
+        <v>160</v>
+      </c>
+      <c r="T61" s="7">
+        <v>1</v>
+      </c>
+      <c r="U61" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V61" s="7" t="s">
+        <v>514</v>
+      </c>
+      <c r="W61" s="7" t="s">
+        <v>515</v>
+      </c>
+      <c r="X61" s="7" t="s">
+        <v>516</v>
+      </c>
+      <c r="Y61" s="7"/>
+      <c r="Z61" s="7">
+        <v>3.3</v>
+      </c>
+      <c r="AA61" s="7"/>
+      <c r="AB61" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC61" s="9" t="s">
+        <v>517</v>
+      </c>
+      <c r="AD61" s="7"/>
+      <c r="AE61" s="7"/>
+      <c r="AF61" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AG61" s="7"/>
+      <c r="AH61" s="7"/>
+      <c r="AI61" s="7"/>
+      <c r="AJ61" s="7"/>
+      <c r="AK61" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="62" spans="1:37">
+      <c r="A62" s="3">
+        <v>60</v>
+      </c>
+      <c r="B62" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="C62" s="3">
+        <v>2026091392</v>
+      </c>
+      <c r="D62" s="3"/>
+      <c r="E62" s="3"/>
+      <c r="F62" s="3">
+        <v>3551</v>
+      </c>
+      <c r="G62" s="3" t="s">
+        <v>512</v>
+      </c>
+      <c r="H62" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="I62" s="3"/>
+      <c r="J62" s="3"/>
+      <c r="K62" s="3"/>
+      <c r="L62" s="3"/>
+      <c r="M62" s="4"/>
+      <c r="N62" s="3"/>
+      <c r="O62" s="4"/>
+      <c r="P62" s="10"/>
+      <c r="Q62" s="3" t="s">
+        <v>513</v>
+      </c>
+      <c r="R62" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S62" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="T62" s="3">
+        <v>1</v>
+      </c>
+      <c r="U62" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V62" s="3" t="s">
+        <v>518</v>
+      </c>
+      <c r="W62" s="3" t="s">
+        <v>515</v>
+      </c>
+      <c r="X62" s="3" t="s">
+        <v>519</v>
+      </c>
+      <c r="Y62" s="3"/>
+      <c r="Z62" s="3">
+        <v>3</v>
+      </c>
+      <c r="AA62" s="3"/>
+      <c r="AB62" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC62" s="10" t="s">
+        <v>520</v>
+      </c>
+      <c r="AD62" s="3"/>
+      <c r="AE62" s="3"/>
+      <c r="AF62" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AG62" s="3"/>
+      <c r="AH62" s="3"/>
+      <c r="AI62" s="3"/>
+      <c r="AJ62" s="3"/>
+      <c r="AK62" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="63" spans="1:37">
+      <c r="A63" s="7">
+        <v>61</v>
+      </c>
+      <c r="B63" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="C63" s="7">
+        <v>2026091397</v>
+      </c>
+      <c r="D63" s="7"/>
+      <c r="E63" s="7"/>
+      <c r="F63" s="7">
+        <v>3017</v>
+      </c>
+      <c r="G63" s="7" t="s">
+        <v>521</v>
+      </c>
+      <c r="H63" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="I63" s="7"/>
+      <c r="J63" s="7"/>
+      <c r="K63" s="7"/>
+      <c r="L63" s="7"/>
+      <c r="M63" s="8"/>
+      <c r="N63" s="7"/>
+      <c r="O63" s="8"/>
+      <c r="P63" s="9"/>
+      <c r="Q63" s="7" t="s">
+        <v>522</v>
+      </c>
+      <c r="R63" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S63" s="7" t="s">
+        <v>92</v>
+      </c>
+      <c r="T63" s="7">
+        <v>1</v>
+      </c>
+      <c r="U63" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V63" s="7" t="s">
+        <v>523</v>
+      </c>
+      <c r="W63" s="7" t="s">
+        <v>524</v>
+      </c>
+      <c r="X63" s="7" t="s">
+        <v>525</v>
+      </c>
+      <c r="Y63" s="7"/>
+      <c r="Z63" s="7">
+        <v>0.3</v>
+      </c>
+      <c r="AA63" s="7"/>
+      <c r="AB63" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC63" s="9" t="s">
+        <v>67</v>
+      </c>
+      <c r="AD63" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE63" s="7"/>
+      <c r="AF63" s="7"/>
+      <c r="AG63" s="7"/>
+      <c r="AH63" s="7"/>
+      <c r="AI63" s="7"/>
+      <c r="AJ63" s="7"/>
+      <c r="AK63" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="64" spans="1:37">
+      <c r="A64" s="3">
+        <v>62</v>
+      </c>
+      <c r="B64" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="C64" s="3">
+        <v>2026091480</v>
+      </c>
+      <c r="D64" s="3"/>
+      <c r="E64" s="3"/>
+      <c r="F64" s="3">
+        <v>2180</v>
+      </c>
+      <c r="G64" s="3" t="s">
+        <v>526</v>
+      </c>
+      <c r="H64" s="3" t="s">
+        <v>140</v>
+      </c>
+      <c r="I64" s="3"/>
+      <c r="J64" s="3"/>
+      <c r="K64" s="3"/>
+      <c r="L64" s="3"/>
+      <c r="M64" s="4"/>
+      <c r="N64" s="3"/>
+      <c r="O64" s="4"/>
+      <c r="P64" s="4"/>
+      <c r="Q64" s="3" t="s">
+        <v>527</v>
+      </c>
+      <c r="R64" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S64" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="T64" s="3">
+        <v>1</v>
+      </c>
+      <c r="U64" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V64" s="3" t="s">
+        <v>528</v>
+      </c>
+      <c r="W64" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="X64" s="3" t="s">
+        <v>530</v>
+      </c>
+      <c r="Y64" s="3"/>
+      <c r="Z64" s="3">
+        <v>0.4</v>
+      </c>
+      <c r="AA64" s="3"/>
+      <c r="AB64" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC64" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="AD64" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE64" s="3"/>
+      <c r="AF64" s="3"/>
+      <c r="AG64" s="3"/>
+      <c r="AH64" s="3"/>
+      <c r="AI64" s="3"/>
+      <c r="AJ64" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AK64" s="3" t="s">
         <v>60</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto commit - 09101245
</commit_message>
<xml_diff>
--- a/IM/202609_HL_Maintain_Report.xlsx
+++ b/IM/202609_HL_Maintain_Report.xlsx
@@ -11,16 +11,16 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Report'!$1:$2</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Report'!$A$1:$AK$64</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Report'!$A$1:$AK$74</definedName>
   </definedNames>
   <calcPr calcId="999999" calcMode="auto" calcCompleted="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="531">
-  <si>
-    <t>萊爾富 工作統計表  篩選月份：202609   (  製表日期:2026-09-08  )</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="612">
+  <si>
+    <t>萊爾富 工作統計表  篩選月份：202609   (  製表日期:2026-09-10  )</t>
   </si>
   <si>
     <t>項次</t>
@@ -1638,6 +1638,250 @@
   </si>
   <si>
     <t>2026-09-08 16:57:00</t>
+  </si>
+  <si>
+    <t>14316115090801</t>
+  </si>
+  <si>
+    <t>五股工商店</t>
+  </si>
+  <si>
+    <t>2026-09-08 18:19:20</t>
+  </si>
+  <si>
+    <t>09/0818:19緊急叫修:門市反應SC(SHUTTLE7S)無網路、顯示伺服器異常，門市告知已有自行重啟SC，PING1不通無法VNC其他網路正常，引導門市查看HUB孔位燈號發現1PORT未亮燈，重新插拔1PORT後仍無反應，解MAC後開2PORT引導門市更換仍未亮燈，請門市查看SC後方網路孔發現疑似水晶頭有斷裂狀況無法重新插拔...需請台芝到店協助協助 P.S.如後續處理有更換硬碟，請跟店長宣達：1.請門市先回報代收會計 2.請確認SC的代收資料是否正確 (須與代收單據逐一核對)與門市確認帳務做到09/08，報表已列印</t>
+  </si>
+  <si>
+    <t>THILF04316</t>
+  </si>
+  <si>
+    <t>2026-09-08 18:24:42</t>
+  </si>
+  <si>
+    <t>2026-09-09 09:00:00</t>
+  </si>
+  <si>
+    <t>2026-09-09 09:30:00</t>
+  </si>
+  <si>
+    <t>2026-09-09 11:24:00</t>
+  </si>
+  <si>
+    <t>更換網路線</t>
+  </si>
+  <si>
+    <t>E4856115090901</t>
+  </si>
+  <si>
+    <t>2026-09-09 07:24:37</t>
+  </si>
+  <si>
+    <t>F603</t>
+  </si>
+  <si>
+    <t>門市反應TM2多卡機(QP3000E)無法使用也無法靠卡交易，協助門市TM版更後點選一卡通開機顯示0801錯誤訊息，悠遊卡重開顯示悠遊卡通訊逾時...請台芝到店協助(TM機2,悠遊卡機故障無法連線.沒有反應)</t>
+  </si>
+  <si>
+    <t>2026-09-09 09:10:38</t>
+  </si>
+  <si>
+    <t>2026-09-09 09:45:00</t>
+  </si>
+  <si>
+    <t>2026-09-09 10:15:00</t>
+  </si>
+  <si>
+    <t>2026-09-10 13:10:00</t>
+  </si>
+  <si>
+    <t>重插io版排線</t>
+  </si>
+  <si>
+    <t>三重金陵店</t>
+  </si>
+  <si>
+    <t>THILF03359</t>
+  </si>
+  <si>
+    <t>2026-09-09 11:32:02</t>
+  </si>
+  <si>
+    <t>2026-09-09 11:05:00</t>
+  </si>
+  <si>
+    <t>2026-09-09 11:27:00</t>
+  </si>
+  <si>
+    <t>12442115090901</t>
+  </si>
+  <si>
+    <t>八里商港店</t>
+  </si>
+  <si>
+    <t>新北市八里區</t>
+  </si>
+  <si>
+    <t>2026-09-09 11:50:44</t>
+  </si>
+  <si>
+    <t>2026年07月份 HUB週期維護:PING91不通無法連線HUB，其他線路正常</t>
+  </si>
+  <si>
+    <t>THILF02442</t>
+  </si>
+  <si>
+    <t>2026-09-09 11:51:15</t>
+  </si>
+  <si>
+    <t>2026-09-09 11:20:00</t>
+  </si>
+  <si>
+    <t>2026-09-09 11:52:00</t>
+  </si>
+  <si>
+    <t>2026-09-10 15:51:00</t>
+  </si>
+  <si>
+    <t>重新設定HUB，測試皆為正常
++HUB</t>
+  </si>
+  <si>
+    <t>三重頂崁店</t>
+  </si>
+  <si>
+    <t>THILF04698</t>
+  </si>
+  <si>
+    <t>2026-09-09 12:08:36</t>
+  </si>
+  <si>
+    <t>2026-09-09 11:40:00</t>
+  </si>
+  <si>
+    <t>2026-09-09 12:03:00</t>
+  </si>
+  <si>
+    <t>E4316115090901</t>
+  </si>
+  <si>
+    <t>2026-09-09 13:00:55</t>
+  </si>
+  <si>
+    <t>HL29</t>
+  </si>
+  <si>
+    <t>HL-CCD掃描器(SC)</t>
+  </si>
+  <si>
+    <t>無電源反應、無紅光</t>
+  </si>
+  <si>
+    <t>門市反應SC CCD掃描器(AT20B)無電源反應無亮燈，已有將線路重新拔插仍無法排除...還請台芝到店協助(無作用)</t>
+  </si>
+  <si>
+    <t>2026-09-09 13:34:27</t>
+  </si>
+  <si>
+    <t>2026-09-10 10:21:00</t>
+  </si>
+  <si>
+    <t>2026-09-10 10:51:00</t>
+  </si>
+  <si>
+    <t>2026-09-10 17:34:00</t>
+  </si>
+  <si>
+    <t>掃槍的USB脫落，插回後測試正常</t>
+  </si>
+  <si>
+    <t>E4282115090901</t>
+  </si>
+  <si>
+    <t>林口建林店</t>
+  </si>
+  <si>
+    <t>2026-09-09 21:33:14</t>
+  </si>
+  <si>
+    <t>HLM3</t>
+  </si>
+  <si>
+    <t>HL-LIFE-ET 標籤印表機</t>
+  </si>
+  <si>
+    <t>M301</t>
+  </si>
+  <si>
+    <t>切刀卡紙，切紙不正常</t>
+  </si>
+  <si>
+    <t>門市反應LIFE ET(標籤印表機)正常綠燈，但列印時裁切的位置不正確，已有重開標籤機重裝紙捲仍異常...須請台芝到店協助(更換標籤紙後發現切紙不正常)9/9 21:41 門市電話未接聽，手機號碼轉語音</t>
+  </si>
+  <si>
+    <t>THILF04282</t>
+  </si>
+  <si>
+    <t>2026-09-09 21:54:03</t>
+  </si>
+  <si>
+    <t>2026-09-10 11:03:00</t>
+  </si>
+  <si>
+    <t>2026-09-10 11:33:00</t>
+  </si>
+  <si>
+    <t>2026-09-11 01:54:00</t>
+  </si>
+  <si>
+    <t>矯正標籤紙捲後測試正常</t>
+  </si>
+  <si>
+    <t>14019115091001</t>
+  </si>
+  <si>
+    <t>永和永霖店</t>
+  </si>
+  <si>
+    <t>2026-09-10 10:08:42</t>
+  </si>
+  <si>
+    <t>THILF04019</t>
+  </si>
+  <si>
+    <t>2026-09-10 10:09:16</t>
+  </si>
+  <si>
+    <t>2026-09-10 09:50:00</t>
+  </si>
+  <si>
+    <t>2026-09-10 10:13:00</t>
+  </si>
+  <si>
+    <t>2026-09-11 14:09:00</t>
+  </si>
+  <si>
+    <t>重置hub設定 +hub</t>
+  </si>
+  <si>
+    <t>2026-09-10 10:17:58</t>
+  </si>
+  <si>
+    <t>2026-09-10 09:30:00</t>
+  </si>
+  <si>
+    <t>永和福和花園</t>
+  </si>
+  <si>
+    <t>THILF03082</t>
+  </si>
+  <si>
+    <t>2026-09-10 10:49:10</t>
+  </si>
+  <si>
+    <t>2026-09-10 10:23:00</t>
+  </si>
+  <si>
+    <t>2026-09-10 10:45:00</t>
   </si>
 </sst>
 </file>
@@ -2051,7 +2295,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AK64"/>
+  <dimension ref="A1:AK74"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="true" style="0"/>
@@ -7516,7 +7760,7 @@
       <c r="M64" s="4"/>
       <c r="N64" s="3"/>
       <c r="O64" s="4"/>
-      <c r="P64" s="4"/>
+      <c r="P64" s="10"/>
       <c r="Q64" s="3" t="s">
         <v>527</v>
       </c>
@@ -7549,7 +7793,7 @@
       <c r="AB64" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="AC64" s="4" t="s">
+      <c r="AC64" s="10" t="s">
         <v>67</v>
       </c>
       <c r="AD64" s="3" t="s">
@@ -7564,6 +7808,904 @@
         <v>60</v>
       </c>
       <c r="AK64" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="65" spans="1:37">
+      <c r="A65" s="7">
+        <v>63</v>
+      </c>
+      <c r="B65" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="C65" s="7">
+        <v>2026091487</v>
+      </c>
+      <c r="D65" s="7" t="s">
+        <v>531</v>
+      </c>
+      <c r="E65" s="7" t="s">
+        <v>357</v>
+      </c>
+      <c r="F65" s="7">
+        <v>4316</v>
+      </c>
+      <c r="G65" s="7" t="s">
+        <v>532</v>
+      </c>
+      <c r="H65" s="7" t="s">
+        <v>315</v>
+      </c>
+      <c r="I65" s="7" t="s">
+        <v>533</v>
+      </c>
+      <c r="J65" s="7" t="s">
+        <v>71</v>
+      </c>
+      <c r="K65" s="7" t="s">
+        <v>186</v>
+      </c>
+      <c r="L65" s="7" t="s">
+        <v>265</v>
+      </c>
+      <c r="M65" s="8" t="s">
+        <v>266</v>
+      </c>
+      <c r="N65" s="7">
+        <v>2401</v>
+      </c>
+      <c r="O65" s="8" t="s">
+        <v>362</v>
+      </c>
+      <c r="P65" s="9" t="s">
+        <v>534</v>
+      </c>
+      <c r="Q65" s="7" t="s">
+        <v>535</v>
+      </c>
+      <c r="R65" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S65" s="7" t="s">
+        <v>320</v>
+      </c>
+      <c r="T65" s="7">
+        <v>1</v>
+      </c>
+      <c r="U65" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V65" s="7" t="s">
+        <v>536</v>
+      </c>
+      <c r="W65" s="7" t="s">
+        <v>537</v>
+      </c>
+      <c r="X65" s="7" t="s">
+        <v>538</v>
+      </c>
+      <c r="Y65" s="7" t="s">
+        <v>539</v>
+      </c>
+      <c r="Z65" s="7">
+        <v>0.5</v>
+      </c>
+      <c r="AA65" s="7"/>
+      <c r="AB65" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC65" s="9" t="s">
+        <v>540</v>
+      </c>
+      <c r="AD65" s="7"/>
+      <c r="AE65" s="7"/>
+      <c r="AF65" s="7"/>
+      <c r="AG65" s="7"/>
+      <c r="AH65" s="7"/>
+      <c r="AI65" s="7"/>
+      <c r="AJ65" s="7"/>
+      <c r="AK65" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="66" spans="1:37">
+      <c r="A66" s="3">
+        <v>64</v>
+      </c>
+      <c r="B66" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="C66" s="3">
+        <v>2026091489</v>
+      </c>
+      <c r="D66" s="3" t="s">
+        <v>541</v>
+      </c>
+      <c r="E66" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="F66" s="3">
+        <v>4856</v>
+      </c>
+      <c r="G66" s="3" t="s">
+        <v>327</v>
+      </c>
+      <c r="H66" s="3" t="s">
+        <v>328</v>
+      </c>
+      <c r="I66" s="3" t="s">
+        <v>542</v>
+      </c>
+      <c r="J66" s="3" t="s">
+        <v>126</v>
+      </c>
+      <c r="K66" s="3" t="s">
+        <v>127</v>
+      </c>
+      <c r="L66" s="3" t="s">
+        <v>339</v>
+      </c>
+      <c r="M66" s="4" t="s">
+        <v>340</v>
+      </c>
+      <c r="N66" s="3" t="s">
+        <v>543</v>
+      </c>
+      <c r="O66" s="4" t="s">
+        <v>108</v>
+      </c>
+      <c r="P66" s="10" t="s">
+        <v>544</v>
+      </c>
+      <c r="Q66" s="3" t="s">
+        <v>331</v>
+      </c>
+      <c r="R66" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S66" s="3" t="s">
+        <v>320</v>
+      </c>
+      <c r="T66" s="3">
+        <v>1</v>
+      </c>
+      <c r="U66" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V66" s="3" t="s">
+        <v>545</v>
+      </c>
+      <c r="W66" s="3" t="s">
+        <v>546</v>
+      </c>
+      <c r="X66" s="3" t="s">
+        <v>547</v>
+      </c>
+      <c r="Y66" s="3" t="s">
+        <v>548</v>
+      </c>
+      <c r="Z66" s="3">
+        <v>0.5</v>
+      </c>
+      <c r="AA66" s="3"/>
+      <c r="AB66" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC66" s="10" t="s">
+        <v>549</v>
+      </c>
+      <c r="AD66" s="3"/>
+      <c r="AE66" s="3"/>
+      <c r="AF66" s="3"/>
+      <c r="AG66" s="3"/>
+      <c r="AH66" s="3"/>
+      <c r="AI66" s="3"/>
+      <c r="AJ66" s="3"/>
+      <c r="AK66" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="67" spans="1:37">
+      <c r="A67" s="7">
+        <v>65</v>
+      </c>
+      <c r="B67" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="C67" s="7">
+        <v>2026091531</v>
+      </c>
+      <c r="D67" s="7"/>
+      <c r="E67" s="7"/>
+      <c r="F67" s="7">
+        <v>3359</v>
+      </c>
+      <c r="G67" s="7" t="s">
+        <v>550</v>
+      </c>
+      <c r="H67" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="I67" s="7"/>
+      <c r="J67" s="7"/>
+      <c r="K67" s="7"/>
+      <c r="L67" s="7"/>
+      <c r="M67" s="8"/>
+      <c r="N67" s="7"/>
+      <c r="O67" s="8"/>
+      <c r="P67" s="9"/>
+      <c r="Q67" s="7" t="s">
+        <v>551</v>
+      </c>
+      <c r="R67" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S67" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="T67" s="7">
+        <v>1</v>
+      </c>
+      <c r="U67" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V67" s="7" t="s">
+        <v>552</v>
+      </c>
+      <c r="W67" s="7" t="s">
+        <v>553</v>
+      </c>
+      <c r="X67" s="7" t="s">
+        <v>554</v>
+      </c>
+      <c r="Y67" s="7"/>
+      <c r="Z67" s="7">
+        <v>0.4</v>
+      </c>
+      <c r="AA67" s="7"/>
+      <c r="AB67" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC67" s="9" t="s">
+        <v>67</v>
+      </c>
+      <c r="AD67" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE67" s="7"/>
+      <c r="AF67" s="7"/>
+      <c r="AG67" s="7"/>
+      <c r="AH67" s="7"/>
+      <c r="AI67" s="7"/>
+      <c r="AJ67" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AK67" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="68" spans="1:37">
+      <c r="A68" s="3">
+        <v>66</v>
+      </c>
+      <c r="B68" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="C68" s="3">
+        <v>2026091535</v>
+      </c>
+      <c r="D68" s="3" t="s">
+        <v>555</v>
+      </c>
+      <c r="E68" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="F68" s="3">
+        <v>2442</v>
+      </c>
+      <c r="G68" s="3" t="s">
+        <v>556</v>
+      </c>
+      <c r="H68" s="3" t="s">
+        <v>557</v>
+      </c>
+      <c r="I68" s="3" t="s">
+        <v>558</v>
+      </c>
+      <c r="J68" s="3" t="s">
+        <v>126</v>
+      </c>
+      <c r="K68" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="L68" s="3" t="s">
+        <v>278</v>
+      </c>
+      <c r="M68" s="4" t="s">
+        <v>279</v>
+      </c>
+      <c r="N68" s="3">
+        <v>3404</v>
+      </c>
+      <c r="O68" s="4" t="s">
+        <v>280</v>
+      </c>
+      <c r="P68" s="10" t="s">
+        <v>559</v>
+      </c>
+      <c r="Q68" s="3" t="s">
+        <v>560</v>
+      </c>
+      <c r="R68" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S68" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="T68" s="3">
+        <v>1</v>
+      </c>
+      <c r="U68" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V68" s="3" t="s">
+        <v>561</v>
+      </c>
+      <c r="W68" s="3" t="s">
+        <v>562</v>
+      </c>
+      <c r="X68" s="3" t="s">
+        <v>563</v>
+      </c>
+      <c r="Y68" s="3" t="s">
+        <v>564</v>
+      </c>
+      <c r="Z68" s="3">
+        <v>0.5</v>
+      </c>
+      <c r="AA68" s="3"/>
+      <c r="AB68" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC68" s="10" t="s">
+        <v>565</v>
+      </c>
+      <c r="AD68" s="3"/>
+      <c r="AE68" s="3"/>
+      <c r="AF68" s="3"/>
+      <c r="AG68" s="3"/>
+      <c r="AH68" s="3"/>
+      <c r="AI68" s="3"/>
+      <c r="AJ68" s="3"/>
+      <c r="AK68" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="69" spans="1:37">
+      <c r="A69" s="7">
+        <v>67</v>
+      </c>
+      <c r="B69" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="C69" s="7">
+        <v>2026091539</v>
+      </c>
+      <c r="D69" s="7"/>
+      <c r="E69" s="7"/>
+      <c r="F69" s="7">
+        <v>4698</v>
+      </c>
+      <c r="G69" s="7" t="s">
+        <v>566</v>
+      </c>
+      <c r="H69" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="I69" s="7"/>
+      <c r="J69" s="7"/>
+      <c r="K69" s="7"/>
+      <c r="L69" s="7"/>
+      <c r="M69" s="8"/>
+      <c r="N69" s="7"/>
+      <c r="O69" s="8"/>
+      <c r="P69" s="9"/>
+      <c r="Q69" s="7" t="s">
+        <v>567</v>
+      </c>
+      <c r="R69" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S69" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="T69" s="7">
+        <v>1</v>
+      </c>
+      <c r="U69" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V69" s="7" t="s">
+        <v>568</v>
+      </c>
+      <c r="W69" s="7" t="s">
+        <v>569</v>
+      </c>
+      <c r="X69" s="7" t="s">
+        <v>570</v>
+      </c>
+      <c r="Y69" s="7"/>
+      <c r="Z69" s="7">
+        <v>0.4</v>
+      </c>
+      <c r="AA69" s="7"/>
+      <c r="AB69" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC69" s="9" t="s">
+        <v>67</v>
+      </c>
+      <c r="AD69" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE69" s="7"/>
+      <c r="AF69" s="7"/>
+      <c r="AG69" s="7"/>
+      <c r="AH69" s="7"/>
+      <c r="AI69" s="7"/>
+      <c r="AJ69" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AK69" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="70" spans="1:37">
+      <c r="A70" s="3">
+        <v>68</v>
+      </c>
+      <c r="B70" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="C70" s="3">
+        <v>2026091552</v>
+      </c>
+      <c r="D70" s="3" t="s">
+        <v>571</v>
+      </c>
+      <c r="E70" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="F70" s="3">
+        <v>4316</v>
+      </c>
+      <c r="G70" s="3" t="s">
+        <v>532</v>
+      </c>
+      <c r="H70" s="3" t="s">
+        <v>315</v>
+      </c>
+      <c r="I70" s="3" t="s">
+        <v>572</v>
+      </c>
+      <c r="J70" s="3" t="s">
+        <v>126</v>
+      </c>
+      <c r="K70" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="L70" s="3" t="s">
+        <v>573</v>
+      </c>
+      <c r="M70" s="4" t="s">
+        <v>574</v>
+      </c>
+      <c r="N70" s="3">
+        <v>2902</v>
+      </c>
+      <c r="O70" s="4" t="s">
+        <v>575</v>
+      </c>
+      <c r="P70" s="10" t="s">
+        <v>576</v>
+      </c>
+      <c r="Q70" s="3" t="s">
+        <v>535</v>
+      </c>
+      <c r="R70" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S70" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="T70" s="3">
+        <v>1</v>
+      </c>
+      <c r="U70" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V70" s="3" t="s">
+        <v>577</v>
+      </c>
+      <c r="W70" s="3" t="s">
+        <v>578</v>
+      </c>
+      <c r="X70" s="3" t="s">
+        <v>579</v>
+      </c>
+      <c r="Y70" s="3" t="s">
+        <v>580</v>
+      </c>
+      <c r="Z70" s="3">
+        <v>0.5</v>
+      </c>
+      <c r="AA70" s="3"/>
+      <c r="AB70" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC70" s="10" t="s">
+        <v>581</v>
+      </c>
+      <c r="AD70" s="3"/>
+      <c r="AE70" s="3"/>
+      <c r="AF70" s="3"/>
+      <c r="AG70" s="3"/>
+      <c r="AH70" s="3"/>
+      <c r="AI70" s="3"/>
+      <c r="AJ70" s="3"/>
+      <c r="AK70" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="71" spans="1:37">
+      <c r="A71" s="7">
+        <v>69</v>
+      </c>
+      <c r="B71" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="C71" s="7">
+        <v>2026091632</v>
+      </c>
+      <c r="D71" s="7" t="s">
+        <v>582</v>
+      </c>
+      <c r="E71" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="F71" s="7">
+        <v>4282</v>
+      </c>
+      <c r="G71" s="7" t="s">
+        <v>583</v>
+      </c>
+      <c r="H71" s="7" t="s">
+        <v>428</v>
+      </c>
+      <c r="I71" s="7" t="s">
+        <v>584</v>
+      </c>
+      <c r="J71" s="7" t="s">
+        <v>126</v>
+      </c>
+      <c r="K71" s="7" t="s">
+        <v>186</v>
+      </c>
+      <c r="L71" s="7" t="s">
+        <v>585</v>
+      </c>
+      <c r="M71" s="8" t="s">
+        <v>586</v>
+      </c>
+      <c r="N71" s="7" t="s">
+        <v>587</v>
+      </c>
+      <c r="O71" s="8" t="s">
+        <v>588</v>
+      </c>
+      <c r="P71" s="9" t="s">
+        <v>589</v>
+      </c>
+      <c r="Q71" s="7" t="s">
+        <v>590</v>
+      </c>
+      <c r="R71" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S71" s="7" t="s">
+        <v>92</v>
+      </c>
+      <c r="T71" s="7">
+        <v>1</v>
+      </c>
+      <c r="U71" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V71" s="7" t="s">
+        <v>591</v>
+      </c>
+      <c r="W71" s="7" t="s">
+        <v>592</v>
+      </c>
+      <c r="X71" s="7" t="s">
+        <v>593</v>
+      </c>
+      <c r="Y71" s="7" t="s">
+        <v>594</v>
+      </c>
+      <c r="Z71" s="7">
+        <v>0.5</v>
+      </c>
+      <c r="AA71" s="7"/>
+      <c r="AB71" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC71" s="9" t="s">
+        <v>595</v>
+      </c>
+      <c r="AD71" s="7"/>
+      <c r="AE71" s="7"/>
+      <c r="AF71" s="7"/>
+      <c r="AG71" s="7"/>
+      <c r="AH71" s="7"/>
+      <c r="AI71" s="7"/>
+      <c r="AJ71" s="7"/>
+      <c r="AK71" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="72" spans="1:37">
+      <c r="A72" s="3">
+        <v>70</v>
+      </c>
+      <c r="B72" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="C72" s="3">
+        <v>2026091662</v>
+      </c>
+      <c r="D72" s="3" t="s">
+        <v>596</v>
+      </c>
+      <c r="E72" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="F72" s="3">
+        <v>4019</v>
+      </c>
+      <c r="G72" s="3" t="s">
+        <v>597</v>
+      </c>
+      <c r="H72" s="3" t="s">
+        <v>263</v>
+      </c>
+      <c r="I72" s="3" t="s">
+        <v>598</v>
+      </c>
+      <c r="J72" s="3" t="s">
+        <v>236</v>
+      </c>
+      <c r="K72" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="L72" s="3" t="s">
+        <v>278</v>
+      </c>
+      <c r="M72" s="4" t="s">
+        <v>279</v>
+      </c>
+      <c r="N72" s="3">
+        <v>3404</v>
+      </c>
+      <c r="O72" s="4" t="s">
+        <v>280</v>
+      </c>
+      <c r="P72" s="10" t="s">
+        <v>559</v>
+      </c>
+      <c r="Q72" s="3" t="s">
+        <v>599</v>
+      </c>
+      <c r="R72" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S72" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="T72" s="3">
+        <v>1</v>
+      </c>
+      <c r="U72" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V72" s="3" t="s">
+        <v>600</v>
+      </c>
+      <c r="W72" s="3" t="s">
+        <v>601</v>
+      </c>
+      <c r="X72" s="3" t="s">
+        <v>602</v>
+      </c>
+      <c r="Y72" s="3" t="s">
+        <v>603</v>
+      </c>
+      <c r="Z72" s="3">
+        <v>0.4</v>
+      </c>
+      <c r="AA72" s="3"/>
+      <c r="AB72" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC72" s="10" t="s">
+        <v>604</v>
+      </c>
+      <c r="AD72" s="3"/>
+      <c r="AE72" s="3"/>
+      <c r="AF72" s="3"/>
+      <c r="AG72" s="3"/>
+      <c r="AH72" s="3"/>
+      <c r="AI72" s="3"/>
+      <c r="AJ72" s="3"/>
+      <c r="AK72" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="73" spans="1:37">
+      <c r="A73" s="7">
+        <v>71</v>
+      </c>
+      <c r="B73" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="C73" s="7">
+        <v>2026091665</v>
+      </c>
+      <c r="D73" s="7"/>
+      <c r="E73" s="7"/>
+      <c r="F73" s="7">
+        <v>4019</v>
+      </c>
+      <c r="G73" s="7" t="s">
+        <v>597</v>
+      </c>
+      <c r="H73" s="7" t="s">
+        <v>263</v>
+      </c>
+      <c r="I73" s="7"/>
+      <c r="J73" s="7"/>
+      <c r="K73" s="7"/>
+      <c r="L73" s="7"/>
+      <c r="M73" s="8"/>
+      <c r="N73" s="7"/>
+      <c r="O73" s="8"/>
+      <c r="P73" s="9"/>
+      <c r="Q73" s="7" t="s">
+        <v>599</v>
+      </c>
+      <c r="R73" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S73" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="T73" s="7">
+        <v>1</v>
+      </c>
+      <c r="U73" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V73" s="7" t="s">
+        <v>605</v>
+      </c>
+      <c r="W73" s="7" t="s">
+        <v>606</v>
+      </c>
+      <c r="X73" s="7" t="s">
+        <v>601</v>
+      </c>
+      <c r="Y73" s="7"/>
+      <c r="Z73" s="7">
+        <v>0.3</v>
+      </c>
+      <c r="AA73" s="7"/>
+      <c r="AB73" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC73" s="9" t="s">
+        <v>67</v>
+      </c>
+      <c r="AD73" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE73" s="7"/>
+      <c r="AF73" s="7"/>
+      <c r="AG73" s="7"/>
+      <c r="AH73" s="7"/>
+      <c r="AI73" s="7"/>
+      <c r="AJ73" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AK73" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="74" spans="1:37">
+      <c r="A74" s="3">
+        <v>72</v>
+      </c>
+      <c r="B74" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="C74" s="3">
+        <v>2026091675</v>
+      </c>
+      <c r="D74" s="3"/>
+      <c r="E74" s="3"/>
+      <c r="F74" s="3">
+        <v>3082</v>
+      </c>
+      <c r="G74" s="3" t="s">
+        <v>607</v>
+      </c>
+      <c r="H74" s="3" t="s">
+        <v>263</v>
+      </c>
+      <c r="I74" s="3"/>
+      <c r="J74" s="3"/>
+      <c r="K74" s="3"/>
+      <c r="L74" s="3"/>
+      <c r="M74" s="4"/>
+      <c r="N74" s="3"/>
+      <c r="O74" s="4"/>
+      <c r="P74" s="4"/>
+      <c r="Q74" s="3" t="s">
+        <v>608</v>
+      </c>
+      <c r="R74" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S74" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="T74" s="3">
+        <v>1</v>
+      </c>
+      <c r="U74" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V74" s="3" t="s">
+        <v>609</v>
+      </c>
+      <c r="W74" s="3" t="s">
+        <v>610</v>
+      </c>
+      <c r="X74" s="3" t="s">
+        <v>611</v>
+      </c>
+      <c r="Y74" s="3"/>
+      <c r="Z74" s="3">
+        <v>0.4</v>
+      </c>
+      <c r="AA74" s="3"/>
+      <c r="AB74" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC74" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="AD74" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE74" s="3"/>
+      <c r="AF74" s="3"/>
+      <c r="AG74" s="3"/>
+      <c r="AH74" s="3"/>
+      <c r="AI74" s="3"/>
+      <c r="AJ74" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AK74" s="3" t="s">
         <v>60</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto commit - 09111736
</commit_message>
<xml_diff>
--- a/IM/202609_HL_Maintain_Report.xlsx
+++ b/IM/202609_HL_Maintain_Report.xlsx
@@ -11,16 +11,16 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Report'!$1:$2</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Report'!$A$1:$AK$74</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Report'!$A$1:$AK$91</definedName>
   </definedNames>
   <calcPr calcId="999999" calcMode="auto" calcCompleted="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="612">
-  <si>
-    <t>萊爾富 工作統計表  篩選月份：202609   (  製表日期:2026-09-10  )</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="728">
+  <si>
+    <t>萊爾富 工作統計表  篩選月份：202609   (  製表日期:2026-09-11  )</t>
   </si>
   <si>
     <t>項次</t>
@@ -1882,6 +1882,357 @@
   </si>
   <si>
     <t>2026-09-10 10:45:00</t>
+  </si>
+  <si>
+    <t>13551115091001</t>
+  </si>
+  <si>
+    <t>2026-09-10 12:50:35</t>
+  </si>
+  <si>
+    <t>F601</t>
+  </si>
+  <si>
+    <t>無法加值</t>
+  </si>
+  <si>
+    <t>門市反應TM2多卡機(QP3000E)悠遊卡顯示通訊逾時，協助門市TM版更後點選一卡通開機顯示0801錯誤訊息，悠遊卡重開顯示悠遊卡通訊逾時...請台芝到店協助</t>
+  </si>
+  <si>
+    <t>2026-09-10 12:51:43</t>
+  </si>
+  <si>
+    <t>2026-09-10 15:01:00</t>
+  </si>
+  <si>
+    <t>2026-09-10 15:22:00</t>
+  </si>
+  <si>
+    <t>2026-09-11 16:51:00</t>
+  </si>
+  <si>
+    <t>換下8183001945 換上8183003234</t>
+  </si>
+  <si>
+    <t>龜山頂湖店</t>
+  </si>
+  <si>
+    <t>THILF03692</t>
+  </si>
+  <si>
+    <t>2026-09-10 13:03:52</t>
+  </si>
+  <si>
+    <t>2026-09-10 12:40:00</t>
+  </si>
+  <si>
+    <t>2026-09-10 13:00:00</t>
+  </si>
+  <si>
+    <t>E4983115091001</t>
+  </si>
+  <si>
+    <t>板橋藝文店</t>
+  </si>
+  <si>
+    <t>2026-09-10 13:38:08</t>
+  </si>
+  <si>
+    <t>抽屜無法正常開關</t>
+  </si>
+  <si>
+    <t>門市反應tm1收銀機(TCX800)(抽屜顏色:黑色、鑰匙孔位子(中)、鎖頭編號:無編號)抽屜內陷卡在軌道...請台芝到店協助(抽屜卡住)</t>
+  </si>
+  <si>
+    <t>THILF04983</t>
+  </si>
+  <si>
+    <t>2026-09-10 13:50:16</t>
+  </si>
+  <si>
+    <t>2026-09-11 12:30:00</t>
+  </si>
+  <si>
+    <t>2026-09-11 12:53:00</t>
+  </si>
+  <si>
+    <t>2026-09-11 17:50:00</t>
+  </si>
+  <si>
+    <t>更換錢箱
+換上：81Z1003570
+換下：81Z1001039</t>
+  </si>
+  <si>
+    <t>龜山桃燿店</t>
+  </si>
+  <si>
+    <t>THILF02763</t>
+  </si>
+  <si>
+    <t>2026-09-10 14:27:17</t>
+  </si>
+  <si>
+    <t>2026-09-10 14:00:00</t>
+  </si>
+  <si>
+    <t>2026-09-10 14:20:00</t>
+  </si>
+  <si>
+    <t>龜山警大店</t>
+  </si>
+  <si>
+    <t>THILF04629</t>
+  </si>
+  <si>
+    <t>2026-09-10 14:53:34</t>
+  </si>
+  <si>
+    <t>2026-09-10 14:30:00</t>
+  </si>
+  <si>
+    <t>2026-09-10 14:50:00</t>
+  </si>
+  <si>
+    <t>中和霸氣店</t>
+  </si>
+  <si>
+    <t>THILF04748</t>
+  </si>
+  <si>
+    <t>2026-09-10 16:00:56</t>
+  </si>
+  <si>
+    <t>2026-09-10 15:38:00</t>
+  </si>
+  <si>
+    <t>2026-09-10 16:00:00</t>
+  </si>
+  <si>
+    <t>ED087115091101</t>
+  </si>
+  <si>
+    <t>D087</t>
+  </si>
+  <si>
+    <t>三重中興北</t>
+  </si>
+  <si>
+    <t>2026-09-11 03:49:48</t>
+  </si>
+  <si>
+    <t>門市反應SC CCD掃描器(CLab1070)無電源反應、無亮紅光，門市告知拔不到線路...請台芝到店協助(掃描器故障)</t>
+  </si>
+  <si>
+    <t>THILF0D087</t>
+  </si>
+  <si>
+    <t>2026-09-11 09:04:08</t>
+  </si>
+  <si>
+    <t>2026-09-11 13:10:00</t>
+  </si>
+  <si>
+    <t>2026-09-11 13:31:00</t>
+  </si>
+  <si>
+    <t>2026-09-14 13:04:00</t>
+  </si>
+  <si>
+    <t>重新插拔掃槍</t>
+  </si>
+  <si>
+    <t>14084115091101</t>
+  </si>
+  <si>
+    <t>三重昌隆店</t>
+  </si>
+  <si>
+    <t>2026-09-11 08:37:23</t>
+  </si>
+  <si>
+    <t>SC(SHUTTLE6S)2026/9/11 (週五) 上午 08:35 總公司宸宇來信: 有關4084三重昌隆店 SC第二顆硬碟異常，請協助通知派工到店更換不備份還原。請協助緊急派工，到店更換sc第二顆硬碟，資料不備份， 謝謝。..須請台芝到店協助 PS.若因更換HD.請跟店長宣達:1.請門市先回報代收會計 2.請確認SC的代收資料是否正確 (須與代收單據逐一核對) 與門市確認帳關到09/10，與通訊嘉芳確認都有收到</t>
+  </si>
+  <si>
+    <t>THILF04084</t>
+  </si>
+  <si>
+    <t>2026-09-11 09:05:14</t>
+  </si>
+  <si>
+    <t>2026-09-11 09:45:00</t>
+  </si>
+  <si>
+    <t>2026-09-11 10:58:00</t>
+  </si>
+  <si>
+    <t>2026-09-11 15:05:00</t>
+  </si>
+  <si>
+    <t>更換第二顆硬碟不備份還原。 已跟店家告知回報代收會計。</t>
+  </si>
+  <si>
+    <t>桃縣桃旺店</t>
+  </si>
+  <si>
+    <t>THILF02566</t>
+  </si>
+  <si>
+    <t>2026-09-11 11:58:41</t>
+  </si>
+  <si>
+    <t>2026-09-11 11:20:00</t>
+  </si>
+  <si>
+    <t>2026-09-11 11:40:00</t>
+  </si>
+  <si>
+    <t>桃縣內溪店</t>
+  </si>
+  <si>
+    <t>THILF02201</t>
+  </si>
+  <si>
+    <t>2026-09-11 12:17:26</t>
+  </si>
+  <si>
+    <t>2026-09-11 11:50:00</t>
+  </si>
+  <si>
+    <t>2026-09-11 12:10:00</t>
+  </si>
+  <si>
+    <t>蘆竹南山店</t>
+  </si>
+  <si>
+    <t>THILF02501</t>
+  </si>
+  <si>
+    <t>2026-09-11 12:39:20</t>
+  </si>
+  <si>
+    <t>2026-09-11 12:20:00</t>
+  </si>
+  <si>
+    <t>2026-09-11 12:40:00</t>
+  </si>
+  <si>
+    <t>蘆竹興安店</t>
+  </si>
+  <si>
+    <t>THILF03881</t>
+  </si>
+  <si>
+    <t>2026-09-11 14:11:22</t>
+  </si>
+  <si>
+    <t>2026-09-11 13:30:00</t>
+  </si>
+  <si>
+    <t>2026-09-11 13:50:00</t>
+  </si>
+  <si>
+    <t>14698115091102</t>
+  </si>
+  <si>
+    <t>2026-09-11 14:10:19</t>
+  </si>
+  <si>
+    <t>HL25</t>
+  </si>
+  <si>
+    <t>HL-SC螢幕</t>
+  </si>
+  <si>
+    <t>螢幕畫面閃爍頻繁或無畫面</t>
+  </si>
+  <si>
+    <t>門市反應SC螢幕(LCD22)黑畫面有亮電源燈，請門市重新拔插螢幕後方線路+切換器仍異常，PING1通可VNC，客服查看畫面正常，與門市確認監視器與SC畫面共用，切到監視器也無畫面...請台芝到店協助</t>
+  </si>
+  <si>
+    <t>2026-09-11 14:16:00</t>
+  </si>
+  <si>
+    <t>2026-09-11 14:40:00</t>
+  </si>
+  <si>
+    <t>2026-09-11 14:57:00</t>
+  </si>
+  <si>
+    <t>2026-09-14 18:16:00</t>
+  </si>
+  <si>
+    <t>螢幕切換器無電源反應。 sc直接對接螢幕可正常使用</t>
+  </si>
+  <si>
+    <t>12255115091101</t>
+  </si>
+  <si>
+    <t>蘆竹六福店</t>
+  </si>
+  <si>
+    <t>2026-09-11 15:02:07</t>
+  </si>
+  <si>
+    <t>2026年7月份 hub調查異常：PING91不通無法連線HUB，其他線路正常</t>
+  </si>
+  <si>
+    <t>THILF02255</t>
+  </si>
+  <si>
+    <t>2026-09-11 15:03:36</t>
+  </si>
+  <si>
+    <t>2026-09-11 14:30:00</t>
+  </si>
+  <si>
+    <t>2026-09-11 14:50:00</t>
+  </si>
+  <si>
+    <t>2026-09-14 19:03:00</t>
+  </si>
+  <si>
+    <t>設定HUB完成
++HUB</t>
+  </si>
+  <si>
+    <t>2026-09-11 15:21:20</t>
+  </si>
+  <si>
+    <t>2026-09-11 15:10:00</t>
+  </si>
+  <si>
+    <t>PMQ3+TVV</t>
+  </si>
+  <si>
+    <t>龜山南上店</t>
+  </si>
+  <si>
+    <t>THILF04035</t>
+  </si>
+  <si>
+    <t>2026-09-11 16:06:00</t>
+  </si>
+  <si>
+    <t>2026-09-11 15:40:00</t>
+  </si>
+  <si>
+    <t>2026-09-11 16:00:00</t>
+  </si>
+  <si>
+    <t>龜山崇優店</t>
+  </si>
+  <si>
+    <t>THILF04197</t>
+  </si>
+  <si>
+    <t>2026-09-11 16:35:56</t>
+  </si>
+  <si>
+    <t>2026-09-11 16:10:00</t>
+  </si>
+  <si>
+    <t>2026-09-11 16:30:00</t>
   </si>
 </sst>
 </file>
@@ -2295,7 +2646,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AK74"/>
+  <dimension ref="A1:AK91"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="true" style="0"/>
@@ -8658,7 +9009,7 @@
       <c r="M74" s="4"/>
       <c r="N74" s="3"/>
       <c r="O74" s="4"/>
-      <c r="P74" s="4"/>
+      <c r="P74" s="10"/>
       <c r="Q74" s="3" t="s">
         <v>608</v>
       </c>
@@ -8691,7 +9042,7 @@
       <c r="AB74" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="AC74" s="4" t="s">
+      <c r="AC74" s="10" t="s">
         <v>67</v>
       </c>
       <c r="AD74" s="3" t="s">
@@ -8706,6 +9057,1437 @@
         <v>60</v>
       </c>
       <c r="AK74" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="75" spans="1:37">
+      <c r="A75" s="7">
+        <v>73</v>
+      </c>
+      <c r="B75" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="C75" s="7">
+        <v>2026091700</v>
+      </c>
+      <c r="D75" s="7" t="s">
+        <v>612</v>
+      </c>
+      <c r="E75" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="F75" s="7">
+        <v>3551</v>
+      </c>
+      <c r="G75" s="7" t="s">
+        <v>512</v>
+      </c>
+      <c r="H75" s="7" t="s">
+        <v>153</v>
+      </c>
+      <c r="I75" s="7" t="s">
+        <v>613</v>
+      </c>
+      <c r="J75" s="7" t="s">
+        <v>236</v>
+      </c>
+      <c r="K75" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="L75" s="7" t="s">
+        <v>339</v>
+      </c>
+      <c r="M75" s="8" t="s">
+        <v>340</v>
+      </c>
+      <c r="N75" s="7" t="s">
+        <v>614</v>
+      </c>
+      <c r="O75" s="8" t="s">
+        <v>615</v>
+      </c>
+      <c r="P75" s="9" t="s">
+        <v>616</v>
+      </c>
+      <c r="Q75" s="7" t="s">
+        <v>513</v>
+      </c>
+      <c r="R75" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S75" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="T75" s="7">
+        <v>1</v>
+      </c>
+      <c r="U75" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V75" s="7" t="s">
+        <v>617</v>
+      </c>
+      <c r="W75" s="7" t="s">
+        <v>618</v>
+      </c>
+      <c r="X75" s="7" t="s">
+        <v>619</v>
+      </c>
+      <c r="Y75" s="7" t="s">
+        <v>620</v>
+      </c>
+      <c r="Z75" s="7">
+        <v>0.4</v>
+      </c>
+      <c r="AA75" s="7"/>
+      <c r="AB75" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC75" s="9" t="s">
+        <v>621</v>
+      </c>
+      <c r="AD75" s="7"/>
+      <c r="AE75" s="7"/>
+      <c r="AF75" s="7"/>
+      <c r="AG75" s="7"/>
+      <c r="AH75" s="7"/>
+      <c r="AI75" s="7"/>
+      <c r="AJ75" s="7"/>
+      <c r="AK75" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="76" spans="1:37">
+      <c r="A76" s="3">
+        <v>74</v>
+      </c>
+      <c r="B76" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="C76" s="3">
+        <v>2026091704</v>
+      </c>
+      <c r="D76" s="3"/>
+      <c r="E76" s="3"/>
+      <c r="F76" s="3">
+        <v>3692</v>
+      </c>
+      <c r="G76" s="3" t="s">
+        <v>622</v>
+      </c>
+      <c r="H76" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="I76" s="3"/>
+      <c r="J76" s="3"/>
+      <c r="K76" s="3"/>
+      <c r="L76" s="3"/>
+      <c r="M76" s="4"/>
+      <c r="N76" s="3"/>
+      <c r="O76" s="4"/>
+      <c r="P76" s="10"/>
+      <c r="Q76" s="3" t="s">
+        <v>623</v>
+      </c>
+      <c r="R76" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S76" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="T76" s="3">
+        <v>1</v>
+      </c>
+      <c r="U76" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V76" s="3" t="s">
+        <v>624</v>
+      </c>
+      <c r="W76" s="3" t="s">
+        <v>625</v>
+      </c>
+      <c r="X76" s="3" t="s">
+        <v>626</v>
+      </c>
+      <c r="Y76" s="3"/>
+      <c r="Z76" s="3">
+        <v>0.3</v>
+      </c>
+      <c r="AA76" s="3"/>
+      <c r="AB76" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC76" s="10" t="s">
+        <v>67</v>
+      </c>
+      <c r="AD76" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE76" s="3"/>
+      <c r="AF76" s="3"/>
+      <c r="AG76" s="3"/>
+      <c r="AH76" s="3"/>
+      <c r="AI76" s="3"/>
+      <c r="AJ76" s="3"/>
+      <c r="AK76" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="77" spans="1:37">
+      <c r="A77" s="7">
+        <v>75</v>
+      </c>
+      <c r="B77" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="C77" s="7">
+        <v>2026091718</v>
+      </c>
+      <c r="D77" s="7" t="s">
+        <v>627</v>
+      </c>
+      <c r="E77" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="F77" s="7">
+        <v>4983</v>
+      </c>
+      <c r="G77" s="7" t="s">
+        <v>628</v>
+      </c>
+      <c r="H77" s="7" t="s">
+        <v>153</v>
+      </c>
+      <c r="I77" s="7" t="s">
+        <v>629</v>
+      </c>
+      <c r="J77" s="7" t="s">
+        <v>236</v>
+      </c>
+      <c r="K77" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="L77" s="7" t="s">
+        <v>155</v>
+      </c>
+      <c r="M77" s="8" t="s">
+        <v>156</v>
+      </c>
+      <c r="N77" s="7">
+        <v>2305</v>
+      </c>
+      <c r="O77" s="8" t="s">
+        <v>630</v>
+      </c>
+      <c r="P77" s="9" t="s">
+        <v>631</v>
+      </c>
+      <c r="Q77" s="7" t="s">
+        <v>632</v>
+      </c>
+      <c r="R77" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S77" s="7" t="s">
+        <v>160</v>
+      </c>
+      <c r="T77" s="7">
+        <v>1</v>
+      </c>
+      <c r="U77" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V77" s="7" t="s">
+        <v>633</v>
+      </c>
+      <c r="W77" s="7" t="s">
+        <v>634</v>
+      </c>
+      <c r="X77" s="7" t="s">
+        <v>635</v>
+      </c>
+      <c r="Y77" s="7" t="s">
+        <v>636</v>
+      </c>
+      <c r="Z77" s="7">
+        <v>0.4</v>
+      </c>
+      <c r="AA77" s="7"/>
+      <c r="AB77" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC77" s="9" t="s">
+        <v>637</v>
+      </c>
+      <c r="AD77" s="7"/>
+      <c r="AE77" s="7"/>
+      <c r="AF77" s="7"/>
+      <c r="AG77" s="7"/>
+      <c r="AH77" s="7"/>
+      <c r="AI77" s="7"/>
+      <c r="AJ77" s="7"/>
+      <c r="AK77" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="78" spans="1:37">
+      <c r="A78" s="3">
+        <v>76</v>
+      </c>
+      <c r="B78" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="C78" s="3">
+        <v>2026091724</v>
+      </c>
+      <c r="D78" s="3"/>
+      <c r="E78" s="3"/>
+      <c r="F78" s="3">
+        <v>2763</v>
+      </c>
+      <c r="G78" s="3" t="s">
+        <v>638</v>
+      </c>
+      <c r="H78" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="I78" s="3"/>
+      <c r="J78" s="3"/>
+      <c r="K78" s="3"/>
+      <c r="L78" s="3"/>
+      <c r="M78" s="4"/>
+      <c r="N78" s="3"/>
+      <c r="O78" s="4"/>
+      <c r="P78" s="10"/>
+      <c r="Q78" s="3" t="s">
+        <v>639</v>
+      </c>
+      <c r="R78" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S78" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="T78" s="3">
+        <v>1</v>
+      </c>
+      <c r="U78" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V78" s="3" t="s">
+        <v>640</v>
+      </c>
+      <c r="W78" s="3" t="s">
+        <v>641</v>
+      </c>
+      <c r="X78" s="3" t="s">
+        <v>642</v>
+      </c>
+      <c r="Y78" s="3"/>
+      <c r="Z78" s="3">
+        <v>0.3</v>
+      </c>
+      <c r="AA78" s="3"/>
+      <c r="AB78" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC78" s="10" t="s">
+        <v>67</v>
+      </c>
+      <c r="AD78" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE78" s="3"/>
+      <c r="AF78" s="3"/>
+      <c r="AG78" s="3"/>
+      <c r="AH78" s="3"/>
+      <c r="AI78" s="3"/>
+      <c r="AJ78" s="3"/>
+      <c r="AK78" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="79" spans="1:37">
+      <c r="A79" s="7">
+        <v>77</v>
+      </c>
+      <c r="B79" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="C79" s="7">
+        <v>2026091732</v>
+      </c>
+      <c r="D79" s="7"/>
+      <c r="E79" s="7"/>
+      <c r="F79" s="7">
+        <v>4629</v>
+      </c>
+      <c r="G79" s="7" t="s">
+        <v>643</v>
+      </c>
+      <c r="H79" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="I79" s="7"/>
+      <c r="J79" s="7"/>
+      <c r="K79" s="7"/>
+      <c r="L79" s="7"/>
+      <c r="M79" s="8"/>
+      <c r="N79" s="7"/>
+      <c r="O79" s="8"/>
+      <c r="P79" s="9"/>
+      <c r="Q79" s="7" t="s">
+        <v>644</v>
+      </c>
+      <c r="R79" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S79" s="7" t="s">
+        <v>92</v>
+      </c>
+      <c r="T79" s="7">
+        <v>1</v>
+      </c>
+      <c r="U79" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V79" s="7" t="s">
+        <v>645</v>
+      </c>
+      <c r="W79" s="7" t="s">
+        <v>646</v>
+      </c>
+      <c r="X79" s="7" t="s">
+        <v>647</v>
+      </c>
+      <c r="Y79" s="7"/>
+      <c r="Z79" s="7">
+        <v>0.3</v>
+      </c>
+      <c r="AA79" s="7"/>
+      <c r="AB79" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC79" s="9" t="s">
+        <v>67</v>
+      </c>
+      <c r="AD79" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE79" s="7"/>
+      <c r="AF79" s="7"/>
+      <c r="AG79" s="7"/>
+      <c r="AH79" s="7"/>
+      <c r="AI79" s="7"/>
+      <c r="AJ79" s="7"/>
+      <c r="AK79" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="80" spans="1:37">
+      <c r="A80" s="3">
+        <v>78</v>
+      </c>
+      <c r="B80" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="C80" s="3">
+        <v>2026091773</v>
+      </c>
+      <c r="D80" s="3"/>
+      <c r="E80" s="3"/>
+      <c r="F80" s="3">
+        <v>4748</v>
+      </c>
+      <c r="G80" s="3" t="s">
+        <v>648</v>
+      </c>
+      <c r="H80" s="3" t="s">
+        <v>140</v>
+      </c>
+      <c r="I80" s="3"/>
+      <c r="J80" s="3"/>
+      <c r="K80" s="3"/>
+      <c r="L80" s="3"/>
+      <c r="M80" s="4"/>
+      <c r="N80" s="3"/>
+      <c r="O80" s="4"/>
+      <c r="P80" s="10"/>
+      <c r="Q80" s="3" t="s">
+        <v>649</v>
+      </c>
+      <c r="R80" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S80" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="T80" s="3">
+        <v>1</v>
+      </c>
+      <c r="U80" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V80" s="3" t="s">
+        <v>650</v>
+      </c>
+      <c r="W80" s="3" t="s">
+        <v>651</v>
+      </c>
+      <c r="X80" s="3" t="s">
+        <v>652</v>
+      </c>
+      <c r="Y80" s="3"/>
+      <c r="Z80" s="3">
+        <v>0.4</v>
+      </c>
+      <c r="AA80" s="3"/>
+      <c r="AB80" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC80" s="10" t="s">
+        <v>67</v>
+      </c>
+      <c r="AD80" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE80" s="3"/>
+      <c r="AF80" s="3"/>
+      <c r="AG80" s="3"/>
+      <c r="AH80" s="3"/>
+      <c r="AI80" s="3"/>
+      <c r="AJ80" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AK80" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="81" spans="1:37">
+      <c r="A81" s="7">
+        <v>79</v>
+      </c>
+      <c r="B81" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="C81" s="7">
+        <v>2026091786</v>
+      </c>
+      <c r="D81" s="7" t="s">
+        <v>653</v>
+      </c>
+      <c r="E81" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="F81" s="7" t="s">
+        <v>654</v>
+      </c>
+      <c r="G81" s="7" t="s">
+        <v>655</v>
+      </c>
+      <c r="H81" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="I81" s="7" t="s">
+        <v>656</v>
+      </c>
+      <c r="J81" s="7" t="s">
+        <v>250</v>
+      </c>
+      <c r="K81" s="7" t="s">
+        <v>127</v>
+      </c>
+      <c r="L81" s="7" t="s">
+        <v>573</v>
+      </c>
+      <c r="M81" s="8" t="s">
+        <v>574</v>
+      </c>
+      <c r="N81" s="7">
+        <v>2902</v>
+      </c>
+      <c r="O81" s="8" t="s">
+        <v>575</v>
+      </c>
+      <c r="P81" s="9" t="s">
+        <v>657</v>
+      </c>
+      <c r="Q81" s="7" t="s">
+        <v>658</v>
+      </c>
+      <c r="R81" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S81" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="T81" s="7">
+        <v>1</v>
+      </c>
+      <c r="U81" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V81" s="7" t="s">
+        <v>659</v>
+      </c>
+      <c r="W81" s="7" t="s">
+        <v>660</v>
+      </c>
+      <c r="X81" s="7" t="s">
+        <v>661</v>
+      </c>
+      <c r="Y81" s="7" t="s">
+        <v>662</v>
+      </c>
+      <c r="Z81" s="7">
+        <v>0.4</v>
+      </c>
+      <c r="AA81" s="7"/>
+      <c r="AB81" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC81" s="9" t="s">
+        <v>663</v>
+      </c>
+      <c r="AD81" s="7"/>
+      <c r="AE81" s="7"/>
+      <c r="AF81" s="7"/>
+      <c r="AG81" s="7"/>
+      <c r="AH81" s="7"/>
+      <c r="AI81" s="7"/>
+      <c r="AJ81" s="7"/>
+      <c r="AK81" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="82" spans="1:37">
+      <c r="A82" s="3">
+        <v>80</v>
+      </c>
+      <c r="B82" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="C82" s="3">
+        <v>2026091787</v>
+      </c>
+      <c r="D82" s="3" t="s">
+        <v>664</v>
+      </c>
+      <c r="E82" s="3" t="s">
+        <v>357</v>
+      </c>
+      <c r="F82" s="3">
+        <v>4084</v>
+      </c>
+      <c r="G82" s="3" t="s">
+        <v>665</v>
+      </c>
+      <c r="H82" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="I82" s="3" t="s">
+        <v>666</v>
+      </c>
+      <c r="J82" s="3" t="s">
+        <v>250</v>
+      </c>
+      <c r="K82" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="L82" s="3" t="s">
+        <v>265</v>
+      </c>
+      <c r="M82" s="4" t="s">
+        <v>266</v>
+      </c>
+      <c r="N82" s="3">
+        <v>2405</v>
+      </c>
+      <c r="O82" s="4" t="s">
+        <v>430</v>
+      </c>
+      <c r="P82" s="10" t="s">
+        <v>667</v>
+      </c>
+      <c r="Q82" s="3" t="s">
+        <v>668</v>
+      </c>
+      <c r="R82" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S82" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="T82" s="3">
+        <v>1</v>
+      </c>
+      <c r="U82" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V82" s="3" t="s">
+        <v>669</v>
+      </c>
+      <c r="W82" s="3" t="s">
+        <v>670</v>
+      </c>
+      <c r="X82" s="3" t="s">
+        <v>671</v>
+      </c>
+      <c r="Y82" s="3" t="s">
+        <v>672</v>
+      </c>
+      <c r="Z82" s="3">
+        <v>1.2</v>
+      </c>
+      <c r="AA82" s="3"/>
+      <c r="AB82" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC82" s="10" t="s">
+        <v>673</v>
+      </c>
+      <c r="AD82" s="3"/>
+      <c r="AE82" s="3"/>
+      <c r="AF82" s="3"/>
+      <c r="AG82" s="3"/>
+      <c r="AH82" s="3"/>
+      <c r="AI82" s="3"/>
+      <c r="AJ82" s="3"/>
+      <c r="AK82" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="83" spans="1:37">
+      <c r="A83" s="7">
+        <v>81</v>
+      </c>
+      <c r="B83" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="C83" s="7">
+        <v>2026091849</v>
+      </c>
+      <c r="D83" s="7"/>
+      <c r="E83" s="7"/>
+      <c r="F83" s="7">
+        <v>2566</v>
+      </c>
+      <c r="G83" s="7" t="s">
+        <v>674</v>
+      </c>
+      <c r="H83" s="7" t="s">
+        <v>205</v>
+      </c>
+      <c r="I83" s="7"/>
+      <c r="J83" s="7"/>
+      <c r="K83" s="7"/>
+      <c r="L83" s="7"/>
+      <c r="M83" s="8"/>
+      <c r="N83" s="7"/>
+      <c r="O83" s="8"/>
+      <c r="P83" s="9"/>
+      <c r="Q83" s="7" t="s">
+        <v>675</v>
+      </c>
+      <c r="R83" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S83" s="7" t="s">
+        <v>92</v>
+      </c>
+      <c r="T83" s="7">
+        <v>1</v>
+      </c>
+      <c r="U83" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V83" s="7" t="s">
+        <v>676</v>
+      </c>
+      <c r="W83" s="7" t="s">
+        <v>677</v>
+      </c>
+      <c r="X83" s="7" t="s">
+        <v>678</v>
+      </c>
+      <c r="Y83" s="7"/>
+      <c r="Z83" s="7">
+        <v>0.3</v>
+      </c>
+      <c r="AA83" s="7"/>
+      <c r="AB83" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC83" s="9" t="s">
+        <v>67</v>
+      </c>
+      <c r="AD83" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE83" s="7"/>
+      <c r="AF83" s="7"/>
+      <c r="AG83" s="7"/>
+      <c r="AH83" s="7"/>
+      <c r="AI83" s="7"/>
+      <c r="AJ83" s="7"/>
+      <c r="AK83" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="84" spans="1:37">
+      <c r="A84" s="3">
+        <v>82</v>
+      </c>
+      <c r="B84" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="C84" s="3">
+        <v>2026091860</v>
+      </c>
+      <c r="D84" s="3"/>
+      <c r="E84" s="3"/>
+      <c r="F84" s="3">
+        <v>2201</v>
+      </c>
+      <c r="G84" s="3" t="s">
+        <v>679</v>
+      </c>
+      <c r="H84" s="3" t="s">
+        <v>205</v>
+      </c>
+      <c r="I84" s="3"/>
+      <c r="J84" s="3"/>
+      <c r="K84" s="3"/>
+      <c r="L84" s="3"/>
+      <c r="M84" s="4"/>
+      <c r="N84" s="3"/>
+      <c r="O84" s="4"/>
+      <c r="P84" s="10"/>
+      <c r="Q84" s="3" t="s">
+        <v>680</v>
+      </c>
+      <c r="R84" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S84" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="T84" s="3">
+        <v>1</v>
+      </c>
+      <c r="U84" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V84" s="3" t="s">
+        <v>681</v>
+      </c>
+      <c r="W84" s="3" t="s">
+        <v>682</v>
+      </c>
+      <c r="X84" s="3" t="s">
+        <v>683</v>
+      </c>
+      <c r="Y84" s="3"/>
+      <c r="Z84" s="3">
+        <v>0.3</v>
+      </c>
+      <c r="AA84" s="3"/>
+      <c r="AB84" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC84" s="10" t="s">
+        <v>67</v>
+      </c>
+      <c r="AD84" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE84" s="3"/>
+      <c r="AF84" s="3"/>
+      <c r="AG84" s="3"/>
+      <c r="AH84" s="3"/>
+      <c r="AI84" s="3"/>
+      <c r="AJ84" s="3"/>
+      <c r="AK84" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="85" spans="1:37">
+      <c r="A85" s="7">
+        <v>83</v>
+      </c>
+      <c r="B85" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="C85" s="7">
+        <v>2026091862</v>
+      </c>
+      <c r="D85" s="7"/>
+      <c r="E85" s="7"/>
+      <c r="F85" s="7">
+        <v>2501</v>
+      </c>
+      <c r="G85" s="7" t="s">
+        <v>684</v>
+      </c>
+      <c r="H85" s="7" t="s">
+        <v>205</v>
+      </c>
+      <c r="I85" s="7"/>
+      <c r="J85" s="7"/>
+      <c r="K85" s="7"/>
+      <c r="L85" s="7"/>
+      <c r="M85" s="8"/>
+      <c r="N85" s="7"/>
+      <c r="O85" s="8"/>
+      <c r="P85" s="9"/>
+      <c r="Q85" s="7" t="s">
+        <v>685</v>
+      </c>
+      <c r="R85" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S85" s="7" t="s">
+        <v>92</v>
+      </c>
+      <c r="T85" s="7">
+        <v>1</v>
+      </c>
+      <c r="U85" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V85" s="7" t="s">
+        <v>686</v>
+      </c>
+      <c r="W85" s="7" t="s">
+        <v>687</v>
+      </c>
+      <c r="X85" s="7" t="s">
+        <v>688</v>
+      </c>
+      <c r="Y85" s="7"/>
+      <c r="Z85" s="7">
+        <v>0.3</v>
+      </c>
+      <c r="AA85" s="7"/>
+      <c r="AB85" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC85" s="9" t="s">
+        <v>67</v>
+      </c>
+      <c r="AD85" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE85" s="7"/>
+      <c r="AF85" s="7"/>
+      <c r="AG85" s="7"/>
+      <c r="AH85" s="7"/>
+      <c r="AI85" s="7"/>
+      <c r="AJ85" s="7"/>
+      <c r="AK85" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="86" spans="1:37">
+      <c r="A86" s="3">
+        <v>84</v>
+      </c>
+      <c r="B86" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="C86" s="3">
+        <v>2026091884</v>
+      </c>
+      <c r="D86" s="3"/>
+      <c r="E86" s="3"/>
+      <c r="F86" s="3">
+        <v>3881</v>
+      </c>
+      <c r="G86" s="3" t="s">
+        <v>689</v>
+      </c>
+      <c r="H86" s="3" t="s">
+        <v>205</v>
+      </c>
+      <c r="I86" s="3"/>
+      <c r="J86" s="3"/>
+      <c r="K86" s="3"/>
+      <c r="L86" s="3"/>
+      <c r="M86" s="4"/>
+      <c r="N86" s="3"/>
+      <c r="O86" s="4"/>
+      <c r="P86" s="10"/>
+      <c r="Q86" s="3" t="s">
+        <v>690</v>
+      </c>
+      <c r="R86" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S86" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="T86" s="3">
+        <v>1</v>
+      </c>
+      <c r="U86" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V86" s="3" t="s">
+        <v>691</v>
+      </c>
+      <c r="W86" s="3" t="s">
+        <v>692</v>
+      </c>
+      <c r="X86" s="3" t="s">
+        <v>693</v>
+      </c>
+      <c r="Y86" s="3"/>
+      <c r="Z86" s="3">
+        <v>0.3</v>
+      </c>
+      <c r="AA86" s="3"/>
+      <c r="AB86" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC86" s="10" t="s">
+        <v>67</v>
+      </c>
+      <c r="AD86" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE86" s="3"/>
+      <c r="AF86" s="3"/>
+      <c r="AG86" s="3"/>
+      <c r="AH86" s="3"/>
+      <c r="AI86" s="3"/>
+      <c r="AJ86" s="3"/>
+      <c r="AK86" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="87" spans="1:37">
+      <c r="A87" s="7">
+        <v>85</v>
+      </c>
+      <c r="B87" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="C87" s="7">
+        <v>2026091886</v>
+      </c>
+      <c r="D87" s="7" t="s">
+        <v>694</v>
+      </c>
+      <c r="E87" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="F87" s="7">
+        <v>4698</v>
+      </c>
+      <c r="G87" s="7" t="s">
+        <v>566</v>
+      </c>
+      <c r="H87" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="I87" s="7" t="s">
+        <v>695</v>
+      </c>
+      <c r="J87" s="7" t="s">
+        <v>250</v>
+      </c>
+      <c r="K87" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="L87" s="7" t="s">
+        <v>696</v>
+      </c>
+      <c r="M87" s="8" t="s">
+        <v>697</v>
+      </c>
+      <c r="N87" s="7">
+        <v>2501</v>
+      </c>
+      <c r="O87" s="8" t="s">
+        <v>698</v>
+      </c>
+      <c r="P87" s="9" t="s">
+        <v>699</v>
+      </c>
+      <c r="Q87" s="7" t="s">
+        <v>567</v>
+      </c>
+      <c r="R87" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S87" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="T87" s="7">
+        <v>1</v>
+      </c>
+      <c r="U87" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V87" s="7" t="s">
+        <v>700</v>
+      </c>
+      <c r="W87" s="7" t="s">
+        <v>701</v>
+      </c>
+      <c r="X87" s="7" t="s">
+        <v>702</v>
+      </c>
+      <c r="Y87" s="7" t="s">
+        <v>703</v>
+      </c>
+      <c r="Z87" s="7">
+        <v>0.3</v>
+      </c>
+      <c r="AA87" s="7"/>
+      <c r="AB87" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC87" s="9" t="s">
+        <v>704</v>
+      </c>
+      <c r="AD87" s="7"/>
+      <c r="AE87" s="7"/>
+      <c r="AF87" s="7"/>
+      <c r="AG87" s="7"/>
+      <c r="AH87" s="7"/>
+      <c r="AI87" s="7"/>
+      <c r="AJ87" s="7"/>
+      <c r="AK87" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="88" spans="1:37">
+      <c r="A88" s="3">
+        <v>86</v>
+      </c>
+      <c r="B88" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="C88" s="3">
+        <v>2026091898</v>
+      </c>
+      <c r="D88" s="3" t="s">
+        <v>705</v>
+      </c>
+      <c r="E88" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="F88" s="3">
+        <v>2255</v>
+      </c>
+      <c r="G88" s="3" t="s">
+        <v>706</v>
+      </c>
+      <c r="H88" s="3" t="s">
+        <v>205</v>
+      </c>
+      <c r="I88" s="3" t="s">
+        <v>707</v>
+      </c>
+      <c r="J88" s="3" t="s">
+        <v>250</v>
+      </c>
+      <c r="K88" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="L88" s="3" t="s">
+        <v>278</v>
+      </c>
+      <c r="M88" s="4" t="s">
+        <v>279</v>
+      </c>
+      <c r="N88" s="3">
+        <v>3404</v>
+      </c>
+      <c r="O88" s="4" t="s">
+        <v>280</v>
+      </c>
+      <c r="P88" s="10" t="s">
+        <v>708</v>
+      </c>
+      <c r="Q88" s="3" t="s">
+        <v>709</v>
+      </c>
+      <c r="R88" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S88" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="T88" s="3">
+        <v>1</v>
+      </c>
+      <c r="U88" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V88" s="3" t="s">
+        <v>710</v>
+      </c>
+      <c r="W88" s="3" t="s">
+        <v>711</v>
+      </c>
+      <c r="X88" s="3" t="s">
+        <v>712</v>
+      </c>
+      <c r="Y88" s="3" t="s">
+        <v>713</v>
+      </c>
+      <c r="Z88" s="3">
+        <v>0.3</v>
+      </c>
+      <c r="AA88" s="3"/>
+      <c r="AB88" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC88" s="10" t="s">
+        <v>714</v>
+      </c>
+      <c r="AD88" s="3"/>
+      <c r="AE88" s="3"/>
+      <c r="AF88" s="3"/>
+      <c r="AG88" s="3"/>
+      <c r="AH88" s="3"/>
+      <c r="AI88" s="3"/>
+      <c r="AJ88" s="3"/>
+      <c r="AK88" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="89" spans="1:37">
+      <c r="A89" s="7">
+        <v>87</v>
+      </c>
+      <c r="B89" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="C89" s="7">
+        <v>2026091903</v>
+      </c>
+      <c r="D89" s="7"/>
+      <c r="E89" s="7"/>
+      <c r="F89" s="7">
+        <v>2255</v>
+      </c>
+      <c r="G89" s="7" t="s">
+        <v>706</v>
+      </c>
+      <c r="H89" s="7" t="s">
+        <v>205</v>
+      </c>
+      <c r="I89" s="7"/>
+      <c r="J89" s="7"/>
+      <c r="K89" s="7"/>
+      <c r="L89" s="7"/>
+      <c r="M89" s="8"/>
+      <c r="N89" s="7"/>
+      <c r="O89" s="8"/>
+      <c r="P89" s="9"/>
+      <c r="Q89" s="7" t="s">
+        <v>709</v>
+      </c>
+      <c r="R89" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S89" s="7" t="s">
+        <v>92</v>
+      </c>
+      <c r="T89" s="7">
+        <v>1</v>
+      </c>
+      <c r="U89" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V89" s="7" t="s">
+        <v>715</v>
+      </c>
+      <c r="W89" s="7" t="s">
+        <v>712</v>
+      </c>
+      <c r="X89" s="7" t="s">
+        <v>716</v>
+      </c>
+      <c r="Y89" s="7"/>
+      <c r="Z89" s="7">
+        <v>0.3</v>
+      </c>
+      <c r="AA89" s="7"/>
+      <c r="AB89" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC89" s="9" t="s">
+        <v>717</v>
+      </c>
+      <c r="AD89" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE89" s="7"/>
+      <c r="AF89" s="7"/>
+      <c r="AG89" s="7"/>
+      <c r="AH89" s="7"/>
+      <c r="AI89" s="7"/>
+      <c r="AJ89" s="7"/>
+      <c r="AK89" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="90" spans="1:37">
+      <c r="A90" s="3">
+        <v>88</v>
+      </c>
+      <c r="B90" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="C90" s="3">
+        <v>2026091919</v>
+      </c>
+      <c r="D90" s="3"/>
+      <c r="E90" s="3"/>
+      <c r="F90" s="3">
+        <v>4035</v>
+      </c>
+      <c r="G90" s="3" t="s">
+        <v>718</v>
+      </c>
+      <c r="H90" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="I90" s="3"/>
+      <c r="J90" s="3"/>
+      <c r="K90" s="3"/>
+      <c r="L90" s="3"/>
+      <c r="M90" s="4"/>
+      <c r="N90" s="3"/>
+      <c r="O90" s="4"/>
+      <c r="P90" s="10"/>
+      <c r="Q90" s="3" t="s">
+        <v>719</v>
+      </c>
+      <c r="R90" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S90" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="T90" s="3">
+        <v>1</v>
+      </c>
+      <c r="U90" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V90" s="3" t="s">
+        <v>720</v>
+      </c>
+      <c r="W90" s="3" t="s">
+        <v>721</v>
+      </c>
+      <c r="X90" s="3" t="s">
+        <v>722</v>
+      </c>
+      <c r="Y90" s="3"/>
+      <c r="Z90" s="3">
+        <v>0.3</v>
+      </c>
+      <c r="AA90" s="3"/>
+      <c r="AB90" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC90" s="10" t="s">
+        <v>67</v>
+      </c>
+      <c r="AD90" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE90" s="3"/>
+      <c r="AF90" s="3"/>
+      <c r="AG90" s="3"/>
+      <c r="AH90" s="3"/>
+      <c r="AI90" s="3"/>
+      <c r="AJ90" s="3"/>
+      <c r="AK90" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="91" spans="1:37">
+      <c r="A91" s="7">
+        <v>89</v>
+      </c>
+      <c r="B91" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="C91" s="7">
+        <v>2026091933</v>
+      </c>
+      <c r="D91" s="7"/>
+      <c r="E91" s="7"/>
+      <c r="F91" s="7">
+        <v>4197</v>
+      </c>
+      <c r="G91" s="7" t="s">
+        <v>723</v>
+      </c>
+      <c r="H91" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="I91" s="7"/>
+      <c r="J91" s="7"/>
+      <c r="K91" s="7"/>
+      <c r="L91" s="7"/>
+      <c r="M91" s="8"/>
+      <c r="N91" s="7"/>
+      <c r="O91" s="8"/>
+      <c r="P91" s="8"/>
+      <c r="Q91" s="7" t="s">
+        <v>724</v>
+      </c>
+      <c r="R91" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S91" s="7" t="s">
+        <v>92</v>
+      </c>
+      <c r="T91" s="7">
+        <v>1</v>
+      </c>
+      <c r="U91" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="V91" s="7" t="s">
+        <v>725</v>
+      </c>
+      <c r="W91" s="7" t="s">
+        <v>726</v>
+      </c>
+      <c r="X91" s="7" t="s">
+        <v>727</v>
+      </c>
+      <c r="Y91" s="7"/>
+      <c r="Z91" s="7">
+        <v>0.3</v>
+      </c>
+      <c r="AA91" s="7"/>
+      <c r="AB91" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC91" s="8" t="s">
+        <v>67</v>
+      </c>
+      <c r="AD91" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE91" s="7"/>
+      <c r="AF91" s="7"/>
+      <c r="AG91" s="7"/>
+      <c r="AH91" s="7"/>
+      <c r="AI91" s="7"/>
+      <c r="AJ91" s="7"/>
+      <c r="AK91" s="7" t="s">
         <v>60</v>
       </c>
     </row>

</xml_diff>